<commit_message>
Điền giả định cơ sở dự án Vân Canh 2
</commit_message>
<xml_diff>
--- a/PTKTTC_Ver1.xlsx
+++ b/PTKTTC_Ver1.xlsx
@@ -2,9 +2,73 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" r:id="R3878c96f78bc4091"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" r:id="R1de55419e3224262"/>
   </x:sheets>
 </x:workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:authors>
+    <x:author>tc={11F66432-3307-873B-12A7-4C732E0186EA}</x:author>
+    <x:author>tc={F3757FEC-73D4-ABA4-0914-CE3007BB35CA}</x:author>
+    <x:author>tc={F2BADE1D-790A-3D7B-F48A-7A5B2281F0C8}</x:author>
+    <x:author>tc={D528358C-641E-4296-3905-F551C67979C5}</x:author>
+    <x:author>tc={C36BD088-EB2C-AE04-C47F-4F689DECD2D5}</x:author>
+  </x:authors>
+  <x:commentList>
+    <x:comment ref="D22" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Nguồn: thông tin do người dùng cung cấp — suất vốn đầu tư 31 tỷ VND/MW.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="D41" authorId="1">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Giả định typical 30% dùng cho mô hình sơ bộ. Đây không phải kết quả nghiên cứu năng lượng; cần thay bằng AEP P50/P90 từ WindPRO hoặc báo cáo đánh giá năng lượng.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="D44" authorId="2">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Nguồn: Quyết định 1508/QĐ-BCT ngày 30/05/2025 của Bộ Công Thương. Giá tối đa điện gió trên đất liền khu vực miền Trung: 1.807,4 VND/kWh, chưa VAT. https://moit.gov.vn/van-ban-phap-luat/quyet-dinh-phe-duyet-khung-gia-phat-dien-loai-hinh-nha-may-dien-gio-nam-2025.html</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="D50" authorId="3">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Giả định typical: O&amp;M năm đầu bằng 2% CAPEX chưa VAT = 111,6 tỷ VND/năm. Cần thay bằng báo giá O&amp;M và ngân sách vận hành thực tế.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="D68" authorId="4">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Giả định dự án đầu tư mới trong lĩnh vực sản xuất năng lượng tái tạo đủ điều kiện ưu đãi: thuế suất 10% trong 15 năm, miễn 4 năm và giảm 50% trong 9 năm tiếp theo. Phải xác minh điều kiện áp dụng theo Luật Thuế TNDN 2025 và Nghị định 320/2025/NĐ-CP. https://vanban.chinhphu.vn/?classid=0&amp;docid=217301&amp;pageid=27160</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+  </x:commentList>
+</x:comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -13,15 +77,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="8">
-    <x:numFmt numFmtId="200" formatCode="0"/>
-    <x:numFmt numFmtId="201" formatCode="#,##0.00;[Red](#,##0.00);-"/>
-    <x:numFmt numFmtId="202" formatCode="0.0%"/>
-    <x:numFmt numFmtId="203" formatCode="0.0"/>
-    <x:numFmt numFmtId="204" formatCode="#,##0;[Red](#,##0);-"/>
-    <x:numFmt numFmtId="205" formatCode="0.00%"/>
-    <x:numFmt numFmtId="206" formatCode="0.00x"/>
-    <x:numFmt numFmtId="207" formatCode="@"/>
+  <x:numFmts count="12">
+    <x:numFmt numFmtId="200" formatCode="#,##0.0;[Red](#,##0.0);-"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
+    <x:numFmt numFmtId="202" formatCode="#,##0.00;[Red](#,##0.00);-"/>
+    <x:numFmt numFmtId="203" formatCode="0.0%"/>
+    <x:numFmt numFmtId="204" formatCode="0.0"/>
+    <x:numFmt numFmtId="205" formatCode="#,##0;[Red](#,##0);-"/>
+    <x:numFmt numFmtId="206" formatCode="0.00%"/>
+    <x:numFmt numFmtId="207" formatCode="0.00x"/>
+    <x:numFmt numFmtId="208" formatCode="#,##0.0"/>
+    <x:numFmt numFmtId="209" formatCode="#,##0"/>
+    <x:numFmt numFmtId="210" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="211" formatCode="@"/>
   </x:numFmts>
   <x:fonts count="10">
     <x:font>
@@ -159,7 +227,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="107">
+  <x:cellXfs count="114">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -264,22 +332,22 @@
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -291,25 +359,25 @@
     <x:xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="202" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="202" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="203" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="204" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="202" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -334,19 +402,22 @@
     <x:xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="203" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="204" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="205" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="206" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="205" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="206" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="206" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -369,10 +440,10 @@
     <x:xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="208" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="208" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -387,13 +458,31 @@
     <x:xf numFmtId="202" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="209" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="209" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="210" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -480,6 +569,12 @@
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:person displayName="Hoang" id="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}"/>
+</xltc:personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -673,6 +768,26 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:threadedComment ref="D22" dT="2026-07-27T08:40:11.144" personId="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}" id="{11F66432-3307-873B-12A7-4C732E0186EA}">
+    <xltc:text>Nguồn: thông tin do người dùng cung cấp — suất vốn đầu tư 31 tỷ VND/MW.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="D41" dT="2026-07-27T08:40:11.145" personId="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}" id="{F3757FEC-73D4-ABA4-0914-CE3007BB35CA}">
+    <xltc:text>Giả định typical 30% dùng cho mô hình sơ bộ. Đây không phải kết quả nghiên cứu năng lượng; cần thay bằng AEP P50/P90 từ WindPRO hoặc báo cáo đánh giá năng lượng.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="D44" dT="2026-07-27T08:40:11.145" personId="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}" id="{F2BADE1D-790A-3D7B-F48A-7A5B2281F0C8}">
+    <xltc:text>Nguồn: Quyết định 1508/QĐ-BCT ngày 30/05/2025 của Bộ Công Thương. Giá tối đa điện gió trên đất liền khu vực miền Trung: 1.807,4 VND/kWh, chưa VAT. https://moit.gov.vn/van-ban-phap-luat/quyet-dinh-phe-duyet-khung-gia-phat-dien-loai-hinh-nha-may-dien-gio-nam-2025.html</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="D50" dT="2026-07-27T08:40:11.145" personId="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}" id="{D528358C-641E-4296-3905-F551C67979C5}">
+    <xltc:text>Giả định typical: O&amp;M năm đầu bằng 2% CAPEX chưa VAT = 111,6 tỷ VND/năm. Cần thay bằng báo giá O&amp;M và ngân sách vận hành thực tế.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="D68" dT="2026-07-27T08:40:11.145" personId="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}" id="{C36BD088-EB2C-AE04-C47F-4F689DECD2D5}">
+    <xltc:text>Giả định dự án đầu tư mới trong lĩnh vực sản xuất năng lượng tái tạo đủ điều kiện ưu đãi: thuế suất 10% trong 15 năm, miễn 4 năm và giảm 50% trong 9 năm tiếp theo. Phải xác minh điều kiện áp dụng theo Luật Thuế TNDN 2025 và Nghị định 320/2025/NĐ-CP. https://vanban.chinhphu.vn/?classid=0&amp;docid=217301&amp;pageid=27160</xltc:text>
+  </xltc:threadedComment>
+</xltc:ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -700,10 +815,10 @@
       <x:c r="E1" s="5"/>
       <x:c r="F1" s="5"/>
       <x:c r="G1" s="5"/>
-      <x:c r="H1" s="96"/>
-      <x:c r="I1" s="96"/>
-      <x:c r="J1" s="96"/>
-      <x:c r="K1" s="96"/>
+      <x:c r="H1" s="103"/>
+      <x:c r="I1" s="103"/>
+      <x:c r="J1" s="103"/>
+      <x:c r="K1" s="103"/>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="10" t="str">
@@ -715,71 +830,71 @@
       <x:c r="E2" s="10"/>
       <x:c r="F2" s="10"/>
       <x:c r="G2" s="10"/>
-      <x:c r="H2" s="96"/>
-      <x:c r="I2" s="96"/>
-      <x:c r="J2" s="96"/>
-      <x:c r="K2" s="96"/>
+      <x:c r="H2" s="103"/>
+      <x:c r="I2" s="103"/>
+      <x:c r="J2" s="103"/>
+      <x:c r="K2" s="103"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="97" t="str">
-        <x:v>Phiên bản: Ver1  |  Ngày lập: 27/07/2026  |  Đơn vị tiền tệ mặc định: tỷ VND</x:v>
-      </x:c>
-      <x:c r="B3" s="97"/>
-      <x:c r="C3" s="97"/>
-      <x:c r="D3" s="97"/>
-      <x:c r="E3" s="97"/>
-      <x:c r="F3" s="97"/>
-      <x:c r="G3" s="97"/>
-      <x:c r="H3" s="96"/>
-      <x:c r="I3" s="96"/>
-      <x:c r="J3" s="96"/>
-      <x:c r="K3" s="96"/>
+      <x:c r="A3" s="104" t="str">
+        <x:v>Phiên bản: Ver1.1  |  Cập nhật: 27/07/2026  |  Đơn vị tiền tệ mặc định: tỷ VND</x:v>
+      </x:c>
+      <x:c r="B3" s="104"/>
+      <x:c r="C3" s="104"/>
+      <x:c r="D3" s="104"/>
+      <x:c r="E3" s="104"/>
+      <x:c r="F3" s="104"/>
+      <x:c r="G3" s="104"/>
+      <x:c r="H3" s="103"/>
+      <x:c r="I3" s="103"/>
+      <x:c r="J3" s="103"/>
+      <x:c r="K3" s="103"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="96"/>
-      <x:c r="B4" s="96"/>
-      <x:c r="C4" s="96"/>
-      <x:c r="D4" s="96"/>
-      <x:c r="E4" s="96"/>
-      <x:c r="F4" s="96"/>
-      <x:c r="G4" s="96"/>
-      <x:c r="H4" s="96"/>
-      <x:c r="I4" s="96"/>
-      <x:c r="J4" s="96"/>
-      <x:c r="K4" s="96"/>
+      <x:c r="A4" s="103"/>
+      <x:c r="B4" s="103"/>
+      <x:c r="C4" s="103"/>
+      <x:c r="D4" s="103"/>
+      <x:c r="E4" s="103"/>
+      <x:c r="F4" s="103"/>
+      <x:c r="G4" s="103"/>
+      <x:c r="H4" s="103"/>
+      <x:c r="I4" s="103"/>
+      <x:c r="J4" s="103"/>
+      <x:c r="K4" s="103"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="98" t="str">
+      <x:c r="A5" s="105" t="str">
         <x:v>QUY ƯỚC MÀU</x:v>
       </x:c>
-      <x:c r="B5" s="98"/>
-      <x:c r="C5" s="96"/>
-      <x:c r="D5" s="96"/>
-      <x:c r="E5" s="96"/>
-      <x:c r="F5" s="96"/>
-      <x:c r="G5" s="96"/>
-      <x:c r="H5" s="96"/>
-      <x:c r="I5" s="99" t="str">
+      <x:c r="B5" s="105"/>
+      <x:c r="C5" s="103"/>
+      <x:c r="D5" s="103"/>
+      <x:c r="E5" s="103"/>
+      <x:c r="F5" s="103"/>
+      <x:c r="G5" s="103"/>
+      <x:c r="H5" s="103"/>
+      <x:c r="I5" s="106" t="str">
         <x:v>KẾT QUẢ TÍNH NHANH</x:v>
       </x:c>
-      <x:c r="J5" s="99"/>
-      <x:c r="K5" s="99"/>
+      <x:c r="J5" s="106"/>
+      <x:c r="K5" s="106"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="96" t="str">
+      <x:c r="A6" s="103" t="str">
         <x:v>Số liệu phải nhập</x:v>
       </x:c>
-      <x:c r="B6" s="100" t="str">
+      <x:c r="B6" s="107" t="str">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="C6" s="96"/>
+      <x:c r="C6" s="103"/>
       <x:c r="D6" s="23" t="str">
         <x:v>Chữ đậm: thông số hoặc kết quả quan trọng</x:v>
       </x:c>
       <x:c r="E6" s="23"/>
       <x:c r="F6" s="23"/>
       <x:c r="G6" s="23"/>
-      <x:c r="H6" s="96"/>
+      <x:c r="H6" s="103"/>
       <x:c r="I6" s="71" t="str">
         <x:v>Chỉ tiêu</x:v>
       </x:c>
@@ -791,47 +906,49 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="96" t="str">
+      <x:c r="A7" s="103" t="str">
         <x:v>Kết quả tính toán</x:v>
       </x:c>
-      <x:c r="B7" s="101" t="n">
+      <x:c r="B7" s="108" t="n">
         <x:f>1+1</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C7" s="96"/>
+      <x:c r="C7" s="103"/>
       <x:c r="D7" s="25" t="str">
         <x:v>Ô để trống hoặc ghi 0 nếu nội dung tùy chọn không áp dụng.</x:v>
       </x:c>
       <x:c r="E7" s="25"/>
       <x:c r="F7" s="25"/>
       <x:c r="G7" s="25"/>
-      <x:c r="H7" s="96"/>
-      <x:c r="I7" s="84" t="str">
+      <x:c r="H7" s="103"/>
+      <x:c r="I7" s="85" t="str">
+        <x:v>Công suất lắp đặt</x:v>
+      </x:c>
+      <x:c r="J7" s="89" t="n">
+        <x:f>IF(D12="","",D12)</x:f>
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="K7" s="85" t="str">
+        <x:v>MW</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="103"/>
+      <x:c r="B8" s="103"/>
+      <x:c r="C8" s="103"/>
+      <x:c r="D8" s="103"/>
+      <x:c r="E8" s="103"/>
+      <x:c r="F8" s="103"/>
+      <x:c r="G8" s="103"/>
+      <x:c r="H8" s="103"/>
+      <x:c r="I8" s="85" t="str">
         <x:v>Năm COD</x:v>
       </x:c>
-      <x:c r="J7" s="88" t="str">
+      <x:c r="J8" s="91" t="n">
         <x:f>IF(D16="","",D16)</x:f>
-      </x:c>
-      <x:c r="K7" s="84" t="str">
-        <x:v>Năm</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="96"/>
-      <x:c r="B8" s="96"/>
-      <x:c r="C8" s="96"/>
-      <x:c r="D8" s="96"/>
-      <x:c r="E8" s="96"/>
-      <x:c r="F8" s="96"/>
-      <x:c r="G8" s="96"/>
-      <x:c r="H8" s="96"/>
-      <x:c r="I8" s="84" t="str">
-        <x:v>Năm kết thúc vận hành</x:v>
-      </x:c>
-      <x:c r="J8" s="88" t="str">
-        <x:f>IF(D18="","",D18)</x:f>
-      </x:c>
-      <x:c r="K8" s="84" t="str">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="K8" s="85" t="str">
         <x:v>Năm</x:v>
       </x:c>
     </x:row>
@@ -857,549 +974,602 @@
       <x:c r="G9" s="38" t="str">
         <x:v>Ghi chú</x:v>
       </x:c>
-      <x:c r="H9" s="96"/>
-      <x:c r="I9" s="84" t="str">
-        <x:v>Tổng thời gian dự án</x:v>
-      </x:c>
-      <x:c r="J9" s="88" t="str">
-        <x:f>IF(OR(D15="",D17=""),"",D15+D17)</x:f>
-      </x:c>
-      <x:c r="K9" s="84" t="str">
+      <x:c r="H9" s="103"/>
+      <x:c r="I9" s="85" t="str">
+        <x:v>Năm kết thúc vận hành</x:v>
+      </x:c>
+      <x:c r="J9" s="91" t="n">
+        <x:f>IF(D18="","",D18)</x:f>
+        <x:v>2046</x:v>
+      </x:c>
+      <x:c r="K9" s="85" t="str">
         <x:v>Năm</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" hidden="0" customHeight="1">
-      <x:c r="A10" s="98" t="str">
+      <x:c r="A10" s="105" t="str">
         <x:v>1. THÔNG TIN CHUNG VÀ TIẾN ĐỘ DỰ ÁN</x:v>
       </x:c>
       <x:c r="B10" s="40"/>
-      <x:c r="C10" s="98"/>
+      <x:c r="C10" s="105"/>
       <x:c r="D10" s="40"/>
-      <x:c r="E10" s="98"/>
-      <x:c r="F10" s="98"/>
-      <x:c r="G10" s="104"/>
-      <x:c r="H10" s="96"/>
-      <x:c r="I10" s="96"/>
-      <x:c r="J10" s="96"/>
-      <x:c r="K10" s="96"/>
-    </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="102" t="str">
+      <x:c r="E10" s="105"/>
+      <x:c r="F10" s="105"/>
+      <x:c r="G10" s="111"/>
+      <x:c r="H10" s="103"/>
+      <x:c r="I10" s="103"/>
+      <x:c r="J10" s="103"/>
+      <x:c r="K10" s="103"/>
+    </x:row>
+    <x:row r="11" ht="24" hidden="0" customHeight="1">
+      <x:c r="A11" s="109" t="str">
         <x:v>GEN-01</x:v>
       </x:c>
       <x:c r="B11" s="47" t="str">
         <x:v>Tên dự án</x:v>
       </x:c>
-      <x:c r="C11" s="102" t="str">
+      <x:c r="C11" s="109" t="str">
         <x:v>Project</x:v>
       </x:c>
-      <x:c r="D11" s="46"/>
-      <x:c r="E11" s="102" t="str">
+      <x:c r="D11" s="46" t="str">
+        <x:v>Dự án Nhà máy điện gió Vân Canh 2</x:v>
+      </x:c>
+      <x:c r="E11" s="109" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="F11" s="102" t="str">
+      <x:c r="F11" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G11" s="43" t="str">
-        <x:v>Nhập tên đầy đủ của dự án.</x:v>
-      </x:c>
-      <x:c r="H11" s="96"/>
-      <x:c r="I11" s="84" t="str">
+        <x:v>Theo thông tin do người dùng cung cấp.</x:v>
+      </x:c>
+      <x:c r="H11" s="103"/>
+      <x:c r="I11" s="85" t="str">
         <x:v>Vốn đầu tư bao gồm VAT</x:v>
       </x:c>
-      <x:c r="J11" s="90" t="str">
+      <x:c r="J11" s="93" t="n">
         <x:f>IF(D25="","",D25)</x:f>
-      </x:c>
-      <x:c r="K11" s="84" t="str">
+        <x:v>6138.000000000001</x:v>
+      </x:c>
+      <x:c r="K11" s="85" t="str">
         <x:v>Tỷ VND</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="102" t="str">
+      <x:c r="A12" s="109" t="str">
         <x:v>GEN-02</x:v>
       </x:c>
-      <x:c r="B12" s="43" t="str">
-        <x:v>Đồng tiền tính toán</x:v>
-      </x:c>
-      <x:c r="C12" s="102" t="str">
-        <x:v>Currency</x:v>
-      </x:c>
-      <x:c r="D12" s="49" t="str">
-        <x:v>VND</x:v>
-      </x:c>
-      <x:c r="E12" s="102" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="F12" s="102" t="str">
+      <x:c r="B12" s="47" t="str">
+        <x:v>Công suất lắp đặt</x:v>
+      </x:c>
+      <x:c r="C12" s="109" t="str">
+        <x:v>Capacity</x:v>
+      </x:c>
+      <x:c r="D12" s="49" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="E12" s="109" t="str">
+        <x:v>MW</x:v>
+      </x:c>
+      <x:c r="F12" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G12" s="43" t="str">
-        <x:v>Ver1 sử dụng VND; giá trị tiền tệ trình bày theo tỷ VND.</x:v>
-      </x:c>
-      <x:c r="H12" s="96"/>
-      <x:c r="I12" s="84" t="str">
-        <x:v>Cơ sở vốn đầu tư kinh tế</x:v>
-      </x:c>
-      <x:c r="J12" s="90" t="str">
-        <x:f>IF(D26="","",D26)</x:f>
-      </x:c>
-      <x:c r="K12" s="84" t="str">
-        <x:v>Tỷ VND</x:v>
+        <x:v>Dùng tính vốn đầu tư và sản lượng điện.</x:v>
+      </x:c>
+      <x:c r="H12" s="103"/>
+      <x:c r="I12" s="85" t="str">
+        <x:v>Suất vốn đầu tư</x:v>
+      </x:c>
+      <x:c r="J12" s="93" t="n">
+        <x:f>IF(D22="","",D22)</x:f>
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="K12" s="85" t="str">
+        <x:v>Tỷ VND/MW</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="102" t="str">
+      <x:c r="A13" s="109" t="str">
         <x:v>GEN-03</x:v>
       </x:c>
       <x:c r="B13" s="43" t="str">
         <x:v>Năm cơ sở của giá</x:v>
       </x:c>
-      <x:c r="C13" s="102" t="str">
+      <x:c r="C13" s="109" t="str">
         <x:v>Base year</x:v>
       </x:c>
-      <x:c r="D13" s="51" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="E13" s="102" t="str">
+      <x:c r="D13" s="52" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="E13" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F13" s="102" t="str">
+      <x:c r="F13" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G13" s="43" t="str">
-        <x:v>Năm quy đổi các khoản vốn đầu tư, giá điện và O&amp;M.</x:v>
-      </x:c>
-      <x:c r="H13" s="96"/>
-      <x:c r="I13" s="84" t="str">
+        <x:v>Giá điện và các giả định đầu vào được quy về mặt bằng năm 2025.</x:v>
+      </x:c>
+      <x:c r="H13" s="103"/>
+      <x:c r="I13" s="85" t="str">
         <x:v>Giá trị khoản vay</x:v>
       </x:c>
-      <x:c r="J13" s="90" t="str">
+      <x:c r="J13" s="93" t="n">
         <x:f>IF(D63="","",D63)</x:f>
-      </x:c>
-      <x:c r="K13" s="84" t="str">
+        <x:v>3905.9999999999995</x:v>
+      </x:c>
+      <x:c r="K13" s="85" t="str">
         <x:v>Tỷ VND</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="102" t="str">
+      <x:c r="A14" s="109" t="str">
         <x:v>GEN-04</x:v>
       </x:c>
       <x:c r="B14" s="47" t="str">
         <x:v>Năm bắt đầu đầu tư</x:v>
       </x:c>
-      <x:c r="C14" s="102" t="str">
+      <x:c r="C14" s="109" t="str">
         <x:v>Start year</x:v>
       </x:c>
       <x:c r="D14" s="53" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="E14" s="102" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="E14" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F14" s="102" t="str">
+      <x:c r="F14" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G14" s="43" t="str">
-        <x:v>Năm bắt đầu phát sinh dòng tiền đầu tư.</x:v>
-      </x:c>
-      <x:c r="H14" s="96"/>
-      <x:c r="I14" s="84" t="str">
+        <x:v>Giả định cơ sở để thiết lập tiến độ dự án.</x:v>
+      </x:c>
+      <x:c r="H14" s="103"/>
+      <x:c r="I14" s="85" t="str">
         <x:v>Vốn chủ sở hữu ban đầu</x:v>
       </x:c>
-      <x:c r="J14" s="90" t="str">
+      <x:c r="J14" s="93" t="n">
         <x:f>IF(D64="","",D64)</x:f>
-      </x:c>
-      <x:c r="K14" s="84" t="str">
+        <x:v>1674.0000000000005</x:v>
+      </x:c>
+      <x:c r="K14" s="85" t="str">
         <x:v>Tỷ VND</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="102" t="str">
+      <x:c r="A15" s="109" t="str">
         <x:v>GEN-05</x:v>
       </x:c>
       <x:c r="B15" s="47" t="str">
         <x:v>Thời gian xây dựng</x:v>
       </x:c>
-      <x:c r="C15" s="102" t="str">
+      <x:c r="C15" s="109" t="str">
         <x:v>Construction</x:v>
       </x:c>
-      <x:c r="D15" s="53"/>
-      <x:c r="E15" s="102" t="str">
+      <x:c r="D15" s="53" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E15" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F15" s="102" t="str">
+      <x:c r="F15" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G15" s="43" t="str">
-        <x:v>Nhập số năm xây dựng; tối đa 5 năm trong Ver1.</x:v>
-      </x:c>
-      <x:c r="H15" s="96"/>
-      <x:c r="I15" s="96"/>
-      <x:c r="J15" s="96"/>
-      <x:c r="K15" s="96"/>
+        <x:v>Giả định typical; tối đa 5 năm trong Ver1.</x:v>
+      </x:c>
+      <x:c r="H15" s="103"/>
+      <x:c r="I15" s="103"/>
+      <x:c r="J15" s="103"/>
+      <x:c r="K15" s="103"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="102" t="str">
+      <x:c r="A16" s="109" t="str">
         <x:v>GEN-06</x:v>
       </x:c>
       <x:c r="B16" s="47" t="str">
         <x:v>Năm vận hành thương mại</x:v>
       </x:c>
-      <x:c r="C16" s="102" t="str">
+      <x:c r="C16" s="109" t="str">
         <x:v>COD year</x:v>
       </x:c>
-      <x:c r="D16" s="57" t="str">
+      <x:c r="D16" s="57" t="n">
         <x:f>IF(OR(D14="",D15=""),"",D14+D15)</x:f>
-      </x:c>
-      <x:c r="E16" s="102" t="str">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="E16" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F16" s="102" t="str">
+      <x:c r="F16" s="109" t="str">
         <x:v>Tự tính</x:v>
       </x:c>
       <x:c r="G16" s="43" t="str">
         <x:v>Năm bắt đầu ghi nhận sản lượng và doanh thu.</x:v>
       </x:c>
-      <x:c r="H16" s="96"/>
-      <x:c r="I16" s="84" t="str">
-        <x:v>Doanh thu năm đầu</x:v>
-      </x:c>
-      <x:c r="J16" s="90" t="str">
-        <x:f>IF(D47="","",D47)</x:f>
-      </x:c>
-      <x:c r="K16" s="84" t="str">
-        <x:v>Tỷ VND</x:v>
+      <x:c r="H16" s="103"/>
+      <x:c r="I16" s="85" t="str">
+        <x:v>Sản lượng điện năm đầu</x:v>
+      </x:c>
+      <x:c r="J16" s="95" t="n">
+        <x:f>IF(D42="","",D42)</x:f>
+        <x:v>473040</x:v>
+      </x:c>
+      <x:c r="K16" s="85" t="str">
+        <x:v>MWh</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
-      <x:c r="A17" s="102" t="str">
+      <x:c r="A17" s="109" t="str">
         <x:v>GEN-07</x:v>
       </x:c>
       <x:c r="B17" s="47" t="str">
         <x:v>Thời gian vận hành</x:v>
       </x:c>
-      <x:c r="C17" s="102" t="str">
+      <x:c r="C17" s="109" t="str">
         <x:v>Operating life</x:v>
       </x:c>
-      <x:c r="D17" s="53"/>
-      <x:c r="E17" s="102" t="str">
+      <x:c r="D17" s="53" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E17" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F17" s="102" t="str">
+      <x:c r="F17" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G17" s="43" t="str">
-        <x:v>Thời gian phân tích vận hành dự án.</x:v>
-      </x:c>
-      <x:c r="H17" s="96"/>
-      <x:c r="I17" s="84" t="str">
-        <x:v>EBITDA năm đầu</x:v>
-      </x:c>
-      <x:c r="J17" s="90" t="str">
-        <x:f>IF(D52="","",D52)</x:f>
-      </x:c>
-      <x:c r="K17" s="84" t="str">
-        <x:v>Tỷ VND</x:v>
+        <x:v>Giả định typical cho mô hình cơ sở.</x:v>
+      </x:c>
+      <x:c r="H17" s="103"/>
+      <x:c r="I17" s="85" t="str">
+        <x:v>Giá bán điện</x:v>
+      </x:c>
+      <x:c r="J17" s="97" t="n">
+        <x:f>IF(D44="","",D44)</x:f>
+        <x:v>1807.4</x:v>
+      </x:c>
+      <x:c r="K17" s="85" t="str">
+        <x:v>VND/kWh</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="102" t="str">
+      <x:c r="A18" s="109" t="str">
         <x:v>GEN-08</x:v>
       </x:c>
       <x:c r="B18" s="47" t="str">
         <x:v>Năm kết thúc vận hành</x:v>
       </x:c>
-      <x:c r="C18" s="102" t="str">
+      <x:c r="C18" s="109" t="str">
         <x:v>End year</x:v>
       </x:c>
-      <x:c r="D18" s="57" t="str">
+      <x:c r="D18" s="57" t="n">
         <x:f>IF(OR(D16="",D17=""),"",D16+D17-1)</x:f>
-      </x:c>
-      <x:c r="E18" s="102" t="str">
+        <x:v>2046</x:v>
+      </x:c>
+      <x:c r="E18" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F18" s="102" t="str">
+      <x:c r="F18" s="109" t="str">
         <x:v>Tự tính</x:v>
       </x:c>
       <x:c r="G18" s="43" t="str">
         <x:v>Năm cuối cùng của thời gian phân tích.</x:v>
       </x:c>
-      <x:c r="H18" s="96"/>
-      <x:c r="I18" s="84" t="str">
-        <x:v>Biên EBITDA năm đầu</x:v>
-      </x:c>
-      <x:c r="J18" s="92" t="str">
-        <x:f>IF(OR(D47="",D47=0,D52=""),"",D52/D47)</x:f>
-      </x:c>
-      <x:c r="K18" s="84" t="str">
-        <x:v>%</x:v>
+      <x:c r="H18" s="103"/>
+      <x:c r="I18" s="85" t="str">
+        <x:v>Doanh thu năm đầu</x:v>
+      </x:c>
+      <x:c r="J18" s="93" t="n">
+        <x:f>IF(D47="","",D47)</x:f>
+        <x:v>854.972496</x:v>
+      </x:c>
+      <x:c r="K18" s="85" t="str">
+        <x:v>Tỷ VND</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="103"/>
-      <x:c r="B19" s="96"/>
-      <x:c r="C19" s="103"/>
-      <x:c r="D19" s="96"/>
-      <x:c r="E19" s="103"/>
-      <x:c r="F19" s="103"/>
-      <x:c r="G19" s="105"/>
-      <x:c r="H19" s="96"/>
-      <x:c r="I19" s="96"/>
-      <x:c r="J19" s="96"/>
-      <x:c r="K19" s="96"/>
+      <x:c r="A19" s="110"/>
+      <x:c r="B19" s="103"/>
+      <x:c r="C19" s="110"/>
+      <x:c r="D19" s="103"/>
+      <x:c r="E19" s="110"/>
+      <x:c r="F19" s="110"/>
+      <x:c r="G19" s="112"/>
+      <x:c r="H19" s="103"/>
+      <x:c r="I19" s="85" t="str">
+        <x:v>Chi phí O&amp;M năm đầu</x:v>
+      </x:c>
+      <x:c r="J19" s="93" t="n">
+        <x:f>IF(D50="","",D50)</x:f>
+        <x:v>111.6</x:v>
+      </x:c>
+      <x:c r="K19" s="85" t="str">
+        <x:v>Tỷ VND</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="22" hidden="0" customHeight="1">
-      <x:c r="A20" s="98" t="str">
+      <x:c r="A20" s="105" t="str">
         <x:v>2. VỐN ĐẦU TƯ</x:v>
       </x:c>
       <x:c r="B20" s="40"/>
-      <x:c r="C20" s="98"/>
+      <x:c r="C20" s="105"/>
       <x:c r="D20" s="40"/>
-      <x:c r="E20" s="98"/>
-      <x:c r="F20" s="98"/>
-      <x:c r="G20" s="104"/>
-      <x:c r="H20" s="96"/>
-      <x:c r="I20" s="84" t="str">
-        <x:v>Kiểm tra giải ngân</x:v>
-      </x:c>
-      <x:c r="J20" s="95" t="str">
-        <x:f>IF(D37="","",IF(ABS(D37-1)&lt;0.000001,"OK","CHƯA ĐỦ 100%"))</x:f>
-      </x:c>
-      <x:c r="K20" s="84" t="str">
-        <x:v>-</x:v>
+      <x:c r="E20" s="105"/>
+      <x:c r="F20" s="105"/>
+      <x:c r="G20" s="111"/>
+      <x:c r="H20" s="103"/>
+      <x:c r="I20" s="85" t="str">
+        <x:v>EBITDA năm đầu</x:v>
+      </x:c>
+      <x:c r="J20" s="93" t="n">
+        <x:f>IF(D52="","",D52)</x:f>
+        <x:v>743.372496</x:v>
+      </x:c>
+      <x:c r="K20" s="85" t="str">
+        <x:v>Tỷ VND</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" hidden="0" customHeight="1">
-      <x:c r="A21" s="102" t="str">
+      <x:c r="A21" s="109" t="str">
         <x:v>CAP-01</x:v>
       </x:c>
       <x:c r="B21" s="47" t="str">
         <x:v>Tổng vốn đầu tư chưa VAT</x:v>
       </x:c>
-      <x:c r="C21" s="102" t="str">
+      <x:c r="C21" s="109" t="str">
         <x:v>CAPEX</x:v>
       </x:c>
-      <x:c r="D21" s="58"/>
-      <x:c r="E21" s="102" t="str">
+      <x:c r="D21" s="58" t="n">
+        <x:f>IF(OR(D12="",D22=""),"",D12*D22)</x:f>
+        <x:v>5580</x:v>
+      </x:c>
+      <x:c r="E21" s="109" t="str">
         <x:v>Tỷ VND</x:v>
       </x:c>
-      <x:c r="F21" s="102" t="str">
+      <x:c r="F21" s="109" t="str">
+        <x:v>Tự tính</x:v>
+      </x:c>
+      <x:c r="G21" s="43" t="str">
+        <x:v>Công suất nhân suất vốn đầu tư; chưa bao gồm VAT và lãi vay xây dựng.</x:v>
+      </x:c>
+      <x:c r="H21" s="103"/>
+      <x:c r="I21" s="85" t="str">
+        <x:v>Biên EBITDA năm đầu</x:v>
+      </x:c>
+      <x:c r="J21" s="99" t="n">
+        <x:f>IF(OR(D47="",D47=0,D52=""),"",D52/D47)</x:f>
+        <x:v>0.8694694852499676</x:v>
+      </x:c>
+      <x:c r="K21" s="85" t="str">
+        <x:v>%</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="109" t="str">
+        <x:v>CAP-02</x:v>
+      </x:c>
+      <x:c r="B22" s="47" t="str">
+        <x:v>Suất vốn đầu tư</x:v>
+      </x:c>
+      <x:c r="C22" s="109" t="str">
+        <x:v>Unit CAPEX</x:v>
+      </x:c>
+      <x:c r="D22" s="59" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E22" s="109" t="str">
+        <x:v>Tỷ VND/MW</x:v>
+      </x:c>
+      <x:c r="F22" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
-      <x:c r="G21" s="43" t="str">
-        <x:v>Không bao gồm VAT được khấu trừ/hoàn; chưa bao gồm lãi vay xây dựng.</x:v>
-      </x:c>
-      <x:c r="H21" s="96"/>
-      <x:c r="I21" s="96"/>
-      <x:c r="J21" s="96"/>
-      <x:c r="K21" s="96"/>
-    </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
-      <x:c r="A22" s="102" t="str">
-        <x:v>CAP-02</x:v>
-      </x:c>
-      <x:c r="B22" s="47" t="str">
+      <x:c r="G22" s="43" t="str">
+        <x:v>Theo thông tin do người dùng cung cấp.</x:v>
+      </x:c>
+      <x:c r="H22" s="103"/>
+      <x:c r="I22" s="103"/>
+      <x:c r="J22" s="103"/>
+      <x:c r="K22" s="103"/>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="109" t="str">
+        <x:v>CAP-03</x:v>
+      </x:c>
+      <x:c r="B23" s="47" t="str">
         <x:v>Thuế suất VAT đầu tư</x:v>
       </x:c>
-      <x:c r="C22" s="102" t="str">
+      <x:c r="C23" s="109" t="str">
         <x:v>VAT capex</x:v>
       </x:c>
-      <x:c r="D22" s="59"/>
-      <x:c r="E22" s="102" t="str">
+      <x:c r="D23" s="60" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="E23" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F22" s="102" t="str">
+      <x:c r="F23" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
-      <x:c r="G22" s="43" t="str">
-        <x:v>Nhập theo tỷ lệ thập phân, ví dụ 10% nhập 10%.</x:v>
-      </x:c>
-      <x:c r="H22" s="96"/>
-      <x:c r="I22" s="96"/>
-      <x:c r="J22" s="96"/>
-      <x:c r="K22" s="96"/>
-    </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
-      <x:c r="A23" s="102" t="str">
-        <x:v>CAP-03</x:v>
-      </x:c>
-      <x:c r="B23" s="43" t="str">
+      <x:c r="G23" s="43" t="str">
+        <x:v>Giả định cơ sở; cần cập nhật theo hợp đồng và quy định áp dụng.</x:v>
+      </x:c>
+      <x:c r="H23" s="103"/>
+      <x:c r="I23" s="85" t="str">
+        <x:v>Kiểm tra giải ngân</x:v>
+      </x:c>
+      <x:c r="J23" s="102" t="str">
+        <x:f>IF(D37="","",IF(ABS(D37-1)&lt;0.000001,"OK","CHƯA ĐỦ 100%"))</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="K23" s="85" t="str">
+        <x:v>-</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="109" t="str">
+        <x:v>CAP-04</x:v>
+      </x:c>
+      <x:c r="B24" s="43" t="str">
         <x:v>Tỷ lệ VAT được khấu trừ/hoàn</x:v>
       </x:c>
-      <x:c r="C23" s="102" t="str">
+      <x:c r="C24" s="109" t="str">
         <x:v>VAT recoverable</x:v>
       </x:c>
-      <x:c r="D23" s="60"/>
-      <x:c r="E23" s="102" t="str">
+      <x:c r="D24" s="61" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E24" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F23" s="102" t="str">
+      <x:c r="F24" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
-      <x:c r="G23" s="43" t="str">
-        <x:v>Phần VAT có thể được khấu trừ hoặc hoàn lại.</x:v>
-      </x:c>
-      <x:c r="H23" s="96"/>
-      <x:c r="I23" s="96"/>
-      <x:c r="J23" s="96"/>
-      <x:c r="K23" s="96"/>
-    </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
-      <x:c r="A24" s="102" t="str">
-        <x:v>CAP-04</x:v>
-      </x:c>
-      <x:c r="B24" s="43" t="str">
-        <x:v>Thời gian hoàn VAT</x:v>
-      </x:c>
-      <x:c r="C24" s="102" t="str">
-        <x:v>VAT lag</x:v>
-      </x:c>
-      <x:c r="D24" s="61"/>
-      <x:c r="E24" s="102" t="str">
-        <x:v>Năm</x:v>
-      </x:c>
-      <x:c r="F24" s="102" t="str">
-        <x:v>Tùy chọn</x:v>
-      </x:c>
       <x:c r="G24" s="43" t="str">
-        <x:v>Nhập 0 nếu VAT được khấu trừ ngay.</x:v>
-      </x:c>
-      <x:c r="H24" s="96"/>
-      <x:c r="I24" s="96"/>
-      <x:c r="J24" s="96"/>
-      <x:c r="K24" s="96"/>
+        <x:v>Giả định toàn bộ VAT đầu vào đủ điều kiện được khấu trừ/hoàn.</x:v>
+      </x:c>
+      <x:c r="H24" s="103"/>
+      <x:c r="I24" s="103"/>
+      <x:c r="J24" s="103"/>
+      <x:c r="K24" s="103"/>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
-      <x:c r="A25" s="102" t="str">
+      <x:c r="A25" s="109" t="str">
         <x:v>CAP-05</x:v>
       </x:c>
       <x:c r="B25" s="47" t="str">
         <x:v>Tổng vốn đầu tư bao gồm VAT</x:v>
       </x:c>
-      <x:c r="C25" s="102" t="str">
+      <x:c r="C25" s="109" t="str">
         <x:v>CAPEX incl. VAT</x:v>
       </x:c>
-      <x:c r="D25" s="62" t="str">
-        <x:f>IF(OR(D21="",D22=""),"",D21*(1+D22))</x:f>
-      </x:c>
-      <x:c r="E25" s="102" t="str">
+      <x:c r="D25" s="58" t="n">
+        <x:f>IF(OR(D21="",D23=""),"",D21*(1+D23))</x:f>
+        <x:v>6138.000000000001</x:v>
+      </x:c>
+      <x:c r="E25" s="109" t="str">
         <x:v>Tỷ VND</x:v>
       </x:c>
-      <x:c r="F25" s="102" t="str">
+      <x:c r="F25" s="109" t="str">
         <x:v>Tự tính</x:v>
       </x:c>
       <x:c r="G25" s="43" t="str">
         <x:v>Tổng nhu cầu tiền đầu tư trước khi nhận hoàn VAT.</x:v>
       </x:c>
-      <x:c r="H25" s="96"/>
-      <x:c r="I25" s="96"/>
-      <x:c r="J25" s="96"/>
-      <x:c r="K25" s="96"/>
+      <x:c r="H25" s="103"/>
+      <x:c r="I25" s="103"/>
+      <x:c r="J25" s="103"/>
+      <x:c r="K25" s="103"/>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
-      <x:c r="A26" s="102" t="str">
+      <x:c r="A26" s="109" t="str">
         <x:v>CAP-06</x:v>
       </x:c>
       <x:c r="B26" s="47" t="str">
         <x:v>Cơ sở vốn đầu tư kinh tế</x:v>
       </x:c>
-      <x:c r="C26" s="102" t="str">
+      <x:c r="C26" s="109" t="str">
         <x:v>Economic CAPEX</x:v>
       </x:c>
-      <x:c r="D26" s="62" t="str">
-        <x:f>IF(OR(D21="",D22="",D23=""),"",D21+D21*D22*(1-D23))</x:f>
-      </x:c>
-      <x:c r="E26" s="102" t="str">
+      <x:c r="D26" s="58" t="n">
+        <x:f>IF(OR(D21="",D23="",D24=""),"",D21+D21*D23*(1-D24))</x:f>
+        <x:v>5580</x:v>
+      </x:c>
+      <x:c r="E26" s="109" t="str">
         <x:v>Tỷ VND</x:v>
       </x:c>
-      <x:c r="F26" s="102" t="str">
+      <x:c r="F26" s="109" t="str">
         <x:v>Tự tính</x:v>
       </x:c>
       <x:c r="G26" s="43" t="str">
         <x:v>CAPEX chưa VAT cộng phần VAT không được khấu trừ/hoàn.</x:v>
       </x:c>
-      <x:c r="H26" s="96"/>
-      <x:c r="I26" s="96"/>
-      <x:c r="J26" s="96"/>
-      <x:c r="K26" s="96"/>
+      <x:c r="H26" s="103"/>
+      <x:c r="I26" s="103"/>
+      <x:c r="J26" s="103"/>
+      <x:c r="K26" s="103"/>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
-      <x:c r="A27" s="102" t="str">
+      <x:c r="A27" s="109" t="str">
         <x:v>CAP-07</x:v>
       </x:c>
       <x:c r="B27" s="43" t="str">
-        <x:v>Giá trị thu hồi cuối dự án</x:v>
-      </x:c>
-      <x:c r="C27" s="102" t="str">
-        <x:v>Residual value</x:v>
-      </x:c>
-      <x:c r="D27" s="63"/>
-      <x:c r="E27" s="102" t="str">
+        <x:v>Thời gian hoàn VAT</x:v>
+      </x:c>
+      <x:c r="C27" s="109" t="str">
+        <x:v>VAT lag</x:v>
+      </x:c>
+      <x:c r="D27" s="62" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E27" s="109" t="str">
+        <x:v>Năm</x:v>
+      </x:c>
+      <x:c r="F27" s="109" t="str">
+        <x:v>Tùy chọn</x:v>
+      </x:c>
+      <x:c r="G27" s="43" t="str">
+        <x:v>Giả định hoàn/khấu trừ VAT sau 1 năm.</x:v>
+      </x:c>
+      <x:c r="H27" s="103"/>
+      <x:c r="I27" s="103"/>
+      <x:c r="J27" s="103"/>
+      <x:c r="K27" s="103"/>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="109" t="str">
+        <x:v>CAP-08</x:v>
+      </x:c>
+      <x:c r="B28" s="43" t="str">
+        <x:v>Giá trị thu hồi ròng cuối dự án</x:v>
+      </x:c>
+      <x:c r="C28" s="109" t="str">
+        <x:v>Net terminal value</x:v>
+      </x:c>
+      <x:c r="D28" s="63" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E28" s="109" t="str">
         <x:v>Tỷ VND</x:v>
       </x:c>
-      <x:c r="F27" s="102" t="str">
+      <x:c r="F28" s="109" t="str">
         <x:v>Tùy chọn</x:v>
       </x:c>
-      <x:c r="G27" s="43" t="str">
-        <x:v>Nhập 0 nếu không xét.</x:v>
-      </x:c>
-      <x:c r="H27" s="96"/>
-      <x:c r="I27" s="96"/>
-      <x:c r="J27" s="96"/>
-      <x:c r="K27" s="96"/>
-    </x:row>
-    <x:row r="28" ht="15" hidden="0" customHeight="1">
-      <x:c r="A28" s="102" t="str">
-        <x:v>CAP-08</x:v>
-      </x:c>
-      <x:c r="B28" s="43" t="str">
-        <x:v>Chi phí tháo dỡ cuối dự án</x:v>
-      </x:c>
-      <x:c r="C28" s="102" t="str">
-        <x:v>Decommissioning</x:v>
-      </x:c>
-      <x:c r="D28" s="63"/>
-      <x:c r="E28" s="102" t="str">
-        <x:v>Tỷ VND</x:v>
-      </x:c>
-      <x:c r="F28" s="102" t="str">
-        <x:v>Tùy chọn</x:v>
-      </x:c>
       <x:c r="G28" s="43" t="str">
-        <x:v>Nhập 0 nếu đã được bù trừ vào giá trị thu hồi.</x:v>
-      </x:c>
-      <x:c r="H28" s="96"/>
-      <x:c r="I28" s="96"/>
-      <x:c r="J28" s="96"/>
-      <x:c r="K28" s="96"/>
+        <x:v>Giá trị thu hồi trừ chi phí tháo dỡ; giả định cơ sở bằng 0.</x:v>
+      </x:c>
+      <x:c r="H28" s="103"/>
+      <x:c r="I28" s="103"/>
+      <x:c r="J28" s="103"/>
+      <x:c r="K28" s="103"/>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
-      <x:c r="A29" s="103"/>
-      <x:c r="B29" s="96"/>
-      <x:c r="C29" s="103"/>
-      <x:c r="D29" s="96"/>
-      <x:c r="E29" s="103"/>
-      <x:c r="F29" s="103"/>
-      <x:c r="G29" s="105"/>
-      <x:c r="H29" s="96"/>
-      <x:c r="I29" s="96"/>
-      <x:c r="J29" s="96"/>
-      <x:c r="K29" s="96"/>
+      <x:c r="A29" s="110"/>
+      <x:c r="B29" s="103"/>
+      <x:c r="C29" s="110"/>
+      <x:c r="D29" s="103"/>
+      <x:c r="E29" s="110"/>
+      <x:c r="F29" s="110"/>
+      <x:c r="G29" s="112"/>
+      <x:c r="H29" s="103"/>
+      <x:c r="I29" s="103"/>
+      <x:c r="J29" s="103"/>
+      <x:c r="K29" s="103"/>
     </x:row>
     <x:row r="30" ht="22" hidden="0" customHeight="1">
-      <x:c r="A30" s="98" t="str">
+      <x:c r="A30" s="105" t="str">
         <x:v>3. TIẾN ĐỘ GIẢI NGÂN VỐN ĐẦU TƯ</x:v>
       </x:c>
       <x:c r="B30" s="40"/>
-      <x:c r="C30" s="98"/>
+      <x:c r="C30" s="105"/>
       <x:c r="D30" s="40"/>
-      <x:c r="E30" s="98"/>
-      <x:c r="F30" s="98"/>
-      <x:c r="G30" s="104"/>
-      <x:c r="H30" s="96"/>
-      <x:c r="I30" s="96"/>
-      <x:c r="J30" s="96"/>
-      <x:c r="K30" s="96"/>
+      <x:c r="E30" s="105"/>
+      <x:c r="F30" s="105"/>
+      <x:c r="G30" s="111"/>
+      <x:c r="H30" s="103"/>
+      <x:c r="I30" s="103"/>
+      <x:c r="J30" s="103"/>
+      <x:c r="K30" s="103"/>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="71" t="str">
@@ -1420,1082 +1590,1145 @@
       <x:c r="F31" s="72" t="str">
         <x:v>Trạng thái</x:v>
       </x:c>
-      <x:c r="G31" s="106" t="str">
+      <x:c r="G31" s="113" t="str">
         <x:v>Ghi chú</x:v>
       </x:c>
-      <x:c r="H31" s="96"/>
-      <x:c r="I31" s="96"/>
-      <x:c r="J31" s="96"/>
-      <x:c r="K31" s="96"/>
+      <x:c r="H31" s="103"/>
+      <x:c r="I31" s="103"/>
+      <x:c r="J31" s="103"/>
+      <x:c r="K31" s="103"/>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
-      <x:c r="A32" s="102" t="str">
+      <x:c r="A32" s="109" t="str">
         <x:v>DIS-01</x:v>
       </x:c>
       <x:c r="B32" s="43" t="str">
         <x:v>Năm xây dựng 1</x:v>
       </x:c>
-      <x:c r="C32" s="102" t="str">
+      <x:c r="C32" s="109" t="str">
         <x:v>Year 1</x:v>
       </x:c>
-      <x:c r="D32" s="60"/>
-      <x:c r="E32" s="102" t="str">
+      <x:c r="D32" s="61" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="E32" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F32" s="102" t="str">
+      <x:c r="F32" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G32" s="43" t="str">
-        <x:v>Nhập 0 nếu năm này không phát sinh giải ngân.</x:v>
-      </x:c>
-      <x:c r="H32" s="96"/>
-      <x:c r="I32" s="96"/>
-      <x:c r="J32" s="96"/>
-      <x:c r="K32" s="96"/>
+        <x:v>Giả định typical: giải ngân 40% năm 1 và 60% năm 2.</x:v>
+      </x:c>
+      <x:c r="H32" s="103"/>
+      <x:c r="I32" s="103"/>
+      <x:c r="J32" s="103"/>
+      <x:c r="K32" s="103"/>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
-      <x:c r="A33" s="102" t="str">
+      <x:c r="A33" s="109" t="str">
         <x:v>DIS-02</x:v>
       </x:c>
       <x:c r="B33" s="43" t="str">
         <x:v>Năm xây dựng 2</x:v>
       </x:c>
-      <x:c r="C33" s="102" t="str">
+      <x:c r="C33" s="109" t="str">
         <x:v>Year 2</x:v>
       </x:c>
-      <x:c r="D33" s="60"/>
-      <x:c r="E33" s="102" t="str">
+      <x:c r="D33" s="61" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="E33" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F33" s="102" t="str">
+      <x:c r="F33" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G33" s="43" t="str">
-        <x:v>Nhập 0 nếu năm này không phát sinh giải ngân.</x:v>
-      </x:c>
-      <x:c r="H33" s="96"/>
-      <x:c r="I33" s="96"/>
-      <x:c r="J33" s="96"/>
-      <x:c r="K33" s="96"/>
+        <x:v>Giả định typical: giải ngân 40% năm 1 và 60% năm 2.</x:v>
+      </x:c>
+      <x:c r="H33" s="103"/>
+      <x:c r="I33" s="103"/>
+      <x:c r="J33" s="103"/>
+      <x:c r="K33" s="103"/>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
-      <x:c r="A34" s="102" t="str">
+      <x:c r="A34" s="109" t="str">
         <x:v>DIS-03</x:v>
       </x:c>
       <x:c r="B34" s="43" t="str">
         <x:v>Năm xây dựng 3</x:v>
       </x:c>
-      <x:c r="C34" s="102" t="str">
+      <x:c r="C34" s="109" t="str">
         <x:v>Year 3</x:v>
       </x:c>
-      <x:c r="D34" s="60"/>
-      <x:c r="E34" s="102" t="str">
+      <x:c r="D34" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E34" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F34" s="102" t="str">
+      <x:c r="F34" s="109" t="str">
         <x:v>Tùy chọn</x:v>
       </x:c>
       <x:c r="G34" s="43" t="str">
-        <x:v>Nhập 0 nếu năm này không phát sinh giải ngân.</x:v>
-      </x:c>
-      <x:c r="H34" s="96"/>
-      <x:c r="I34" s="96"/>
-      <x:c r="J34" s="96"/>
-      <x:c r="K34" s="96"/>
+        <x:v>Không phát sinh trong kịch bản cơ sở.</x:v>
+      </x:c>
+      <x:c r="H34" s="103"/>
+      <x:c r="I34" s="103"/>
+      <x:c r="J34" s="103"/>
+      <x:c r="K34" s="103"/>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
-      <x:c r="A35" s="102" t="str">
+      <x:c r="A35" s="109" t="str">
         <x:v>DIS-04</x:v>
       </x:c>
       <x:c r="B35" s="43" t="str">
         <x:v>Năm xây dựng 4</x:v>
       </x:c>
-      <x:c r="C35" s="102" t="str">
+      <x:c r="C35" s="109" t="str">
         <x:v>Year 4</x:v>
       </x:c>
-      <x:c r="D35" s="60"/>
-      <x:c r="E35" s="102" t="str">
+      <x:c r="D35" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E35" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F35" s="102" t="str">
+      <x:c r="F35" s="109" t="str">
         <x:v>Tùy chọn</x:v>
       </x:c>
       <x:c r="G35" s="43" t="str">
-        <x:v>Nhập 0 nếu năm này không phát sinh giải ngân.</x:v>
-      </x:c>
-      <x:c r="H35" s="96"/>
-      <x:c r="I35" s="96"/>
-      <x:c r="J35" s="96"/>
-      <x:c r="K35" s="96"/>
+        <x:v>Không phát sinh trong kịch bản cơ sở.</x:v>
+      </x:c>
+      <x:c r="H35" s="103"/>
+      <x:c r="I35" s="103"/>
+      <x:c r="J35" s="103"/>
+      <x:c r="K35" s="103"/>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
-      <x:c r="A36" s="102" t="str">
+      <x:c r="A36" s="109" t="str">
         <x:v>DIS-05</x:v>
       </x:c>
       <x:c r="B36" s="43" t="str">
         <x:v>Năm xây dựng 5</x:v>
       </x:c>
-      <x:c r="C36" s="102" t="str">
+      <x:c r="C36" s="109" t="str">
         <x:v>Year 5</x:v>
       </x:c>
-      <x:c r="D36" s="60"/>
-      <x:c r="E36" s="102" t="str">
+      <x:c r="D36" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E36" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F36" s="102" t="str">
+      <x:c r="F36" s="109" t="str">
         <x:v>Tùy chọn</x:v>
       </x:c>
       <x:c r="G36" s="43" t="str">
-        <x:v>Nhập 0 nếu năm này không phát sinh giải ngân.</x:v>
-      </x:c>
-      <x:c r="H36" s="96"/>
-      <x:c r="I36" s="96"/>
-      <x:c r="J36" s="96"/>
-      <x:c r="K36" s="96"/>
+        <x:v>Không phát sinh trong kịch bản cơ sở.</x:v>
+      </x:c>
+      <x:c r="H36" s="103"/>
+      <x:c r="I36" s="103"/>
+      <x:c r="J36" s="103"/>
+      <x:c r="K36" s="103"/>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
-      <x:c r="A37" s="102" t="str">
+      <x:c r="A37" s="109" t="str">
         <x:v>DIS-06</x:v>
       </x:c>
       <x:c r="B37" s="47" t="str">
         <x:v>Tổng tỷ lệ giải ngân</x:v>
       </x:c>
-      <x:c r="C37" s="102" t="str">
+      <x:c r="C37" s="109" t="str">
         <x:v>Total</x:v>
       </x:c>
-      <x:c r="D37" s="74" t="str">
+      <x:c r="D37" s="74" t="n">
         <x:f>IF(COUNT(D32:D36)=0,"",SUM(D32:D36))</x:f>
-      </x:c>
-      <x:c r="E37" s="102" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E37" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F37" s="102" t="str">
+      <x:c r="F37" s="109" t="str">
         <x:v>Kiểm tra</x:v>
       </x:c>
       <x:c r="G37" s="43" t="str">
         <x:v>Phải bằng 100%.</x:v>
       </x:c>
-      <x:c r="H37" s="96"/>
-      <x:c r="I37" s="96"/>
-      <x:c r="J37" s="96"/>
-      <x:c r="K37" s="96"/>
+      <x:c r="H37" s="103"/>
+      <x:c r="I37" s="103"/>
+      <x:c r="J37" s="103"/>
+      <x:c r="K37" s="103"/>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
-      <x:c r="A38" s="103"/>
-      <x:c r="B38" s="96"/>
-      <x:c r="C38" s="103"/>
-      <x:c r="D38" s="96"/>
-      <x:c r="E38" s="103"/>
-      <x:c r="F38" s="103"/>
-      <x:c r="G38" s="105"/>
-      <x:c r="H38" s="96"/>
-      <x:c r="I38" s="96"/>
-      <x:c r="J38" s="96"/>
-      <x:c r="K38" s="96"/>
+      <x:c r="A38" s="110"/>
+      <x:c r="B38" s="103"/>
+      <x:c r="C38" s="110"/>
+      <x:c r="D38" s="103"/>
+      <x:c r="E38" s="110"/>
+      <x:c r="F38" s="110"/>
+      <x:c r="G38" s="112"/>
+      <x:c r="H38" s="103"/>
+      <x:c r="I38" s="103"/>
+      <x:c r="J38" s="103"/>
+      <x:c r="K38" s="103"/>
     </x:row>
     <x:row r="39" ht="22" hidden="0" customHeight="1">
-      <x:c r="A39" s="98" t="str">
+      <x:c r="A39" s="105" t="str">
         <x:v>4. SẢN LƯỢNG VÀ DOANH THU</x:v>
       </x:c>
       <x:c r="B39" s="40"/>
-      <x:c r="C39" s="98"/>
+      <x:c r="C39" s="105"/>
       <x:c r="D39" s="40"/>
-      <x:c r="E39" s="98"/>
-      <x:c r="F39" s="98"/>
-      <x:c r="G39" s="104"/>
-      <x:c r="H39" s="96"/>
-      <x:c r="I39" s="96"/>
-      <x:c r="J39" s="96"/>
-      <x:c r="K39" s="96"/>
+      <x:c r="E39" s="105"/>
+      <x:c r="F39" s="105"/>
+      <x:c r="G39" s="111"/>
+      <x:c r="H39" s="103"/>
+      <x:c r="I39" s="103"/>
+      <x:c r="J39" s="103"/>
+      <x:c r="K39" s="103"/>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
-      <x:c r="A40" s="102" t="str">
+      <x:c r="A40" s="109" t="str">
         <x:v>REV-01</x:v>
       </x:c>
       <x:c r="B40" s="43" t="str">
         <x:v>Kịch bản sản lượng</x:v>
       </x:c>
-      <x:c r="C40" s="102" t="str">
+      <x:c r="C40" s="109" t="str">
         <x:v>Energy case</x:v>
       </x:c>
-      <x:c r="D40" s="49" t="str">
+      <x:c r="D40" s="75" t="str">
         <x:v>P50</x:v>
       </x:c>
-      <x:c r="E40" s="102" t="str">
+      <x:c r="E40" s="109" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="F40" s="102" t="str">
+      <x:c r="F40" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G40" s="43" t="str">
         <x:v>Chọn P50, P75, P90 hoặc Khác.</x:v>
       </x:c>
-      <x:c r="H40" s="96"/>
-      <x:c r="I40" s="96"/>
-      <x:c r="J40" s="96"/>
-      <x:c r="K40" s="96"/>
-    </x:row>
-    <x:row r="41" ht="15" hidden="0" customHeight="1">
-      <x:c r="A41" s="102" t="str">
+      <x:c r="H40" s="103"/>
+      <x:c r="I40" s="103"/>
+      <x:c r="J40" s="103"/>
+      <x:c r="K40" s="103"/>
+    </x:row>
+    <x:row r="41" ht="24" hidden="0" customHeight="1">
+      <x:c r="A41" s="109" t="str">
         <x:v>REV-02</x:v>
       </x:c>
       <x:c r="B41" s="47" t="str">
+        <x:v>Hệ số công suất ròng</x:v>
+      </x:c>
+      <x:c r="C41" s="109" t="str">
+        <x:v>Net capacity factor</x:v>
+      </x:c>
+      <x:c r="D41" s="60" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="E41" s="109" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="F41" s="109" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="G41" s="43" t="str">
+        <x:v>Giả định typical để lập mô hình sơ bộ; thay bằng AEP P50 từ báo cáo năng lượng khi có.</x:v>
+      </x:c>
+      <x:c r="H41" s="103"/>
+      <x:c r="I41" s="103"/>
+      <x:c r="J41" s="103"/>
+      <x:c r="K41" s="103"/>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="109" t="str">
+        <x:v>REV-03</x:v>
+      </x:c>
+      <x:c r="B42" s="47" t="str">
         <x:v>Sản lượng điện thương phẩm năm đầu</x:v>
       </x:c>
-      <x:c r="C41" s="102" t="str">
+      <x:c r="C42" s="109" t="str">
         <x:v>AEP net</x:v>
       </x:c>
-      <x:c r="D41" s="75"/>
-      <x:c r="E41" s="102" t="str">
+      <x:c r="D42" s="76" t="n">
+        <x:f>IF(OR(D12="",D41=""),"",D12*8760*D41)</x:f>
+        <x:v>473040</x:v>
+      </x:c>
+      <x:c r="E42" s="109" t="str">
         <x:v>MWh/năm</x:v>
       </x:c>
-      <x:c r="F41" s="102" t="str">
+      <x:c r="F42" s="109" t="str">
+        <x:v>Tự tính</x:v>
+      </x:c>
+      <x:c r="G42" s="43" t="str">
+        <x:v>Công suất × 8.760 giờ × hệ số công suất ròng.</x:v>
+      </x:c>
+      <x:c r="H42" s="103"/>
+      <x:c r="I42" s="103"/>
+      <x:c r="J42" s="103"/>
+      <x:c r="K42" s="103"/>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="109" t="str">
+        <x:v>REV-04</x:v>
+      </x:c>
+      <x:c r="B43" s="43" t="str">
+        <x:v>Tỷ lệ suy giảm sản lượng hằng năm</x:v>
+      </x:c>
+      <x:c r="C43" s="109" t="str">
+        <x:v>Degradation</x:v>
+      </x:c>
+      <x:c r="D43" s="77" t="n">
+        <x:v>0.002</x:v>
+      </x:c>
+      <x:c r="E43" s="109" t="str">
+        <x:v>%/năm</x:v>
+      </x:c>
+      <x:c r="F43" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
-      <x:c r="G41" s="43" t="str">
-        <x:v>Sản lượng thực tế bán được, đã trừ toàn bộ tổn thất.</x:v>
-      </x:c>
-      <x:c r="H41" s="96"/>
-      <x:c r="I41" s="96"/>
-      <x:c r="J41" s="96"/>
-      <x:c r="K41" s="96"/>
-    </x:row>
-    <x:row r="42" ht="15" hidden="0" customHeight="1">
-      <x:c r="A42" s="102" t="str">
-        <x:v>REV-03</x:v>
-      </x:c>
-      <x:c r="B42" s="43" t="str">
-        <x:v>Tỷ lệ suy giảm sản lượng hằng năm</x:v>
-      </x:c>
-      <x:c r="C42" s="102" t="str">
-        <x:v>Degradation</x:v>
-      </x:c>
-      <x:c r="D42" s="76"/>
-      <x:c r="E42" s="102" t="str">
+      <x:c r="G43" s="43" t="str">
+        <x:v>Giả định typical 0,2%/năm.</x:v>
+      </x:c>
+      <x:c r="H43" s="103"/>
+      <x:c r="I43" s="103"/>
+      <x:c r="J43" s="103"/>
+      <x:c r="K43" s="103"/>
+    </x:row>
+    <x:row r="44" ht="24" hidden="0" customHeight="1">
+      <x:c r="A44" s="109" t="str">
+        <x:v>REV-05</x:v>
+      </x:c>
+      <x:c r="B44" s="47" t="str">
+        <x:v>Giá bán điện năm đầu, chưa VAT</x:v>
+      </x:c>
+      <x:c r="C44" s="109" t="str">
+        <x:v>Tariff</x:v>
+      </x:c>
+      <x:c r="D44" s="59" t="n">
+        <x:v>1807.4</x:v>
+      </x:c>
+      <x:c r="E44" s="109" t="str">
+        <x:v>VND/kWh</x:v>
+      </x:c>
+      <x:c r="F44" s="109" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="G44" s="43" t="str">
+        <x:v>Giá tối đa điện gió trên đất liền miền Trung năm 2025 theo QĐ 1508/QĐ-BCT; không mặc nhiên là giá PPA.</x:v>
+      </x:c>
+      <x:c r="H44" s="103"/>
+      <x:c r="I44" s="103"/>
+      <x:c r="J44" s="103"/>
+      <x:c r="K44" s="103"/>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="109" t="str">
+        <x:v>REV-06</x:v>
+      </x:c>
+      <x:c r="B45" s="43" t="str">
+        <x:v>Tỷ lệ tăng giá điện hằng năm</x:v>
+      </x:c>
+      <x:c r="C45" s="109" t="str">
+        <x:v>Tariff escalation</x:v>
+      </x:c>
+      <x:c r="D45" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E45" s="109" t="str">
         <x:v>%/năm</x:v>
       </x:c>
-      <x:c r="F42" s="102" t="str">
+      <x:c r="F45" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
-      <x:c r="G42" s="43" t="str">
-        <x:v>Nhập 0 nếu không xét suy giảm.</x:v>
-      </x:c>
-      <x:c r="H42" s="96"/>
-      <x:c r="I42" s="96"/>
-      <x:c r="J42" s="96"/>
-      <x:c r="K42" s="96"/>
-    </x:row>
-    <x:row r="43" ht="15" hidden="0" customHeight="1">
-      <x:c r="A43" s="102" t="str">
-        <x:v>REV-04</x:v>
-      </x:c>
-      <x:c r="B43" s="47" t="str">
-        <x:v>Giá bán điện năm đầu, chưa VAT</x:v>
-      </x:c>
-      <x:c r="C43" s="102" t="str">
-        <x:v>Tariff</x:v>
-      </x:c>
-      <x:c r="D43" s="58"/>
-      <x:c r="E43" s="102" t="str">
-        <x:v>VND/kWh</x:v>
-      </x:c>
-      <x:c r="F43" s="102" t="str">
-        <x:v>Bắt buộc</x:v>
-      </x:c>
-      <x:c r="G43" s="43" t="str">
-        <x:v>Giá điện chưa bao gồm VAT.</x:v>
-      </x:c>
-      <x:c r="H43" s="96"/>
-      <x:c r="I43" s="96"/>
-      <x:c r="J43" s="96"/>
-      <x:c r="K43" s="96"/>
-    </x:row>
-    <x:row r="44" ht="15" hidden="0" customHeight="1">
-      <x:c r="A44" s="102" t="str">
-        <x:v>REV-05</x:v>
-      </x:c>
-      <x:c r="B44" s="43" t="str">
-        <x:v>Tỷ lệ tăng giá điện hằng năm</x:v>
-      </x:c>
-      <x:c r="C44" s="102" t="str">
-        <x:v>Tariff escalation</x:v>
-      </x:c>
-      <x:c r="D44" s="76"/>
-      <x:c r="E44" s="102" t="str">
-        <x:v>%/năm</x:v>
-      </x:c>
-      <x:c r="F44" s="102" t="str">
-        <x:v>Bắt buộc</x:v>
-      </x:c>
-      <x:c r="G44" s="43" t="str">
-        <x:v>Nhập 0 nếu giá điện cố định.</x:v>
-      </x:c>
-      <x:c r="H44" s="96"/>
-      <x:c r="I44" s="96"/>
-      <x:c r="J44" s="96"/>
-      <x:c r="K44" s="96"/>
-    </x:row>
-    <x:row r="45" ht="15" hidden="0" customHeight="1">
-      <x:c r="A45" s="102" t="str">
-        <x:v>REV-06</x:v>
-      </x:c>
-      <x:c r="B45" s="43" t="str">
+      <x:c r="G45" s="43" t="str">
+        <x:v>Giả định giá cố định; cập nhật theo PPA thực tế.</x:v>
+      </x:c>
+      <x:c r="H45" s="103"/>
+      <x:c r="I45" s="103"/>
+      <x:c r="J45" s="103"/>
+      <x:c r="K45" s="103"/>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="109" t="str">
+        <x:v>REV-07</x:v>
+      </x:c>
+      <x:c r="B46" s="43" t="str">
         <x:v>Doanh thu khác năm đầu</x:v>
       </x:c>
-      <x:c r="C45" s="102" t="str">
+      <x:c r="C46" s="109" t="str">
         <x:v>Other revenue</x:v>
       </x:c>
-      <x:c r="D45" s="63"/>
-      <x:c r="E45" s="102" t="str">
+      <x:c r="D46" s="63" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E46" s="109" t="str">
         <x:v>Tỷ VND/năm</x:v>
       </x:c>
-      <x:c r="F45" s="102" t="str">
+      <x:c r="F46" s="109" t="str">
         <x:v>Tùy chọn</x:v>
       </x:c>
-      <x:c r="G45" s="43" t="str">
-        <x:v>REC, I-REC, tín chỉ carbon hoặc nguồn thu khác.</x:v>
-      </x:c>
-      <x:c r="H45" s="96"/>
-      <x:c r="I45" s="96"/>
-      <x:c r="J45" s="96"/>
-      <x:c r="K45" s="96"/>
-    </x:row>
-    <x:row r="46" ht="15" hidden="0" customHeight="1">
-      <x:c r="A46" s="102" t="str">
-        <x:v>REV-07</x:v>
-      </x:c>
-      <x:c r="B46" s="43" t="str">
-        <x:v>Tỷ lệ tăng doanh thu khác</x:v>
-      </x:c>
-      <x:c r="C46" s="102" t="str">
-        <x:v>Other escalation</x:v>
-      </x:c>
-      <x:c r="D46" s="76"/>
-      <x:c r="E46" s="102" t="str">
-        <x:v>%/năm</x:v>
-      </x:c>
-      <x:c r="F46" s="102" t="str">
-        <x:v>Tùy chọn</x:v>
-      </x:c>
       <x:c r="G46" s="43" t="str">
-        <x:v>Nhập 0 nếu không tăng.</x:v>
-      </x:c>
-      <x:c r="H46" s="96"/>
-      <x:c r="I46" s="96"/>
-      <x:c r="J46" s="96"/>
-      <x:c r="K46" s="96"/>
+        <x:v>Chưa xét REC, I-REC, tín chỉ carbon hoặc nguồn thu khác.</x:v>
+      </x:c>
+      <x:c r="H46" s="103"/>
+      <x:c r="I46" s="103"/>
+      <x:c r="J46" s="103"/>
+      <x:c r="K46" s="103"/>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
-      <x:c r="A47" s="102" t="str">
+      <x:c r="A47" s="109" t="str">
         <x:v>REV-08</x:v>
       </x:c>
       <x:c r="B47" s="47" t="str">
         <x:v>Doanh thu năm vận hành đầu tiên</x:v>
       </x:c>
-      <x:c r="C47" s="102" t="str">
+      <x:c r="C47" s="109" t="str">
         <x:v>Revenue Y1</x:v>
       </x:c>
-      <x:c r="D47" s="62" t="str">
-        <x:f>IF(OR(D41="",D43=""),"",D41*1000*D43/1000000000+IF(D45="",0,D45))</x:f>
-      </x:c>
-      <x:c r="E47" s="102" t="str">
+      <x:c r="D47" s="58" t="n">
+        <x:f>IF(OR(D42="",D44=""),"",D42*1000*D44/1000000000+IF(D46="",0,D46))</x:f>
+        <x:v>854.972496</x:v>
+      </x:c>
+      <x:c r="E47" s="109" t="str">
         <x:v>Tỷ VND</x:v>
       </x:c>
-      <x:c r="F47" s="102" t="str">
+      <x:c r="F47" s="109" t="str">
         <x:v>Tự tính</x:v>
       </x:c>
       <x:c r="G47" s="43" t="str">
         <x:v>Doanh thu điện cộng doanh thu khác.</x:v>
       </x:c>
-      <x:c r="H47" s="96"/>
-      <x:c r="I47" s="96"/>
-      <x:c r="J47" s="96"/>
-      <x:c r="K47" s="96"/>
+      <x:c r="H47" s="103"/>
+      <x:c r="I47" s="103"/>
+      <x:c r="J47" s="103"/>
+      <x:c r="K47" s="103"/>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
-      <x:c r="A48" s="103"/>
-      <x:c r="B48" s="96"/>
-      <x:c r="C48" s="103"/>
-      <x:c r="D48" s="96"/>
-      <x:c r="E48" s="103"/>
-      <x:c r="F48" s="103"/>
-      <x:c r="G48" s="105"/>
-      <x:c r="H48" s="96"/>
-      <x:c r="I48" s="96"/>
-      <x:c r="J48" s="96"/>
-      <x:c r="K48" s="96"/>
+      <x:c r="A48" s="110"/>
+      <x:c r="B48" s="103"/>
+      <x:c r="C48" s="110"/>
+      <x:c r="D48" s="103"/>
+      <x:c r="E48" s="110"/>
+      <x:c r="F48" s="110"/>
+      <x:c r="G48" s="112"/>
+      <x:c r="H48" s="103"/>
+      <x:c r="I48" s="103"/>
+      <x:c r="J48" s="103"/>
+      <x:c r="K48" s="103"/>
     </x:row>
     <x:row r="49" ht="22" hidden="0" customHeight="1">
-      <x:c r="A49" s="98" t="str">
+      <x:c r="A49" s="105" t="str">
         <x:v>5. CHI PHÍ VẬN HÀNH</x:v>
       </x:c>
       <x:c r="B49" s="40"/>
-      <x:c r="C49" s="98"/>
+      <x:c r="C49" s="105"/>
       <x:c r="D49" s="40"/>
-      <x:c r="E49" s="98"/>
-      <x:c r="F49" s="98"/>
-      <x:c r="G49" s="104"/>
-      <x:c r="H49" s="96"/>
-      <x:c r="I49" s="96"/>
-      <x:c r="J49" s="96"/>
-      <x:c r="K49" s="96"/>
+      <x:c r="E49" s="105"/>
+      <x:c r="F49" s="105"/>
+      <x:c r="G49" s="111"/>
+      <x:c r="H49" s="103"/>
+      <x:c r="I49" s="103"/>
+      <x:c r="J49" s="103"/>
+      <x:c r="K49" s="103"/>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
-      <x:c r="A50" s="102" t="str">
+      <x:c r="A50" s="109" t="str">
         <x:v>OPE-01</x:v>
       </x:c>
       <x:c r="B50" s="47" t="str">
         <x:v>Chi phí O&amp;M năm đầu</x:v>
       </x:c>
-      <x:c r="C50" s="102" t="str">
+      <x:c r="C50" s="109" t="str">
         <x:v>O&amp;M Y1</x:v>
       </x:c>
-      <x:c r="D50" s="58"/>
-      <x:c r="E50" s="102" t="str">
+      <x:c r="D50" s="59" t="n">
+        <x:v>111.6</x:v>
+      </x:c>
+      <x:c r="E50" s="109" t="str">
         <x:v>Tỷ VND/năm</x:v>
       </x:c>
-      <x:c r="F50" s="102" t="str">
+      <x:c r="F50" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G50" s="43" t="str">
-        <x:v>Tổng chi phí vận hành, bảo dưỡng và quản lý năm đầu.</x:v>
-      </x:c>
-      <x:c r="H50" s="96"/>
-      <x:c r="I50" s="96"/>
-      <x:c r="J50" s="96"/>
-      <x:c r="K50" s="96"/>
+        <x:v>Giả định typical bằng 2% CAPEX chưa VAT.</x:v>
+      </x:c>
+      <x:c r="H50" s="103"/>
+      <x:c r="I50" s="103"/>
+      <x:c r="J50" s="103"/>
+      <x:c r="K50" s="103"/>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
-      <x:c r="A51" s="102" t="str">
+      <x:c r="A51" s="109" t="str">
         <x:v>OPE-02</x:v>
       </x:c>
       <x:c r="B51" s="43" t="str">
         <x:v>Tỷ lệ tăng O&amp;M hằng năm</x:v>
       </x:c>
-      <x:c r="C51" s="102" t="str">
+      <x:c r="C51" s="109" t="str">
         <x:v>O&amp;M escalation</x:v>
       </x:c>
-      <x:c r="D51" s="76"/>
-      <x:c r="E51" s="102" t="str">
+      <x:c r="D51" s="77" t="n">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="E51" s="109" t="str">
         <x:v>%/năm</x:v>
       </x:c>
-      <x:c r="F51" s="102" t="str">
+      <x:c r="F51" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G51" s="43" t="str">
-        <x:v>Có thể sử dụng tỷ lệ lạm phát O&amp;M.</x:v>
-      </x:c>
-      <x:c r="H51" s="96"/>
-      <x:c r="I51" s="96"/>
-      <x:c r="J51" s="96"/>
-      <x:c r="K51" s="96"/>
+        <x:v>Giả định typical 3%/năm.</x:v>
+      </x:c>
+      <x:c r="H51" s="103"/>
+      <x:c r="I51" s="103"/>
+      <x:c r="J51" s="103"/>
+      <x:c r="K51" s="103"/>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
-      <x:c r="A52" s="102" t="str">
+      <x:c r="A52" s="109" t="str">
         <x:v>OPE-03</x:v>
       </x:c>
       <x:c r="B52" s="47" t="str">
         <x:v>EBITDA năm vận hành đầu tiên</x:v>
       </x:c>
-      <x:c r="C52" s="102" t="str">
+      <x:c r="C52" s="109" t="str">
         <x:v>EBITDA Y1</x:v>
       </x:c>
-      <x:c r="D52" s="62" t="str">
+      <x:c r="D52" s="58" t="n">
         <x:f>IF(OR(D47="",D50=""),"",D47-D50)</x:f>
-      </x:c>
-      <x:c r="E52" s="102" t="str">
+        <x:v>743.372496</x:v>
+      </x:c>
+      <x:c r="E52" s="109" t="str">
         <x:v>Tỷ VND</x:v>
       </x:c>
-      <x:c r="F52" s="102" t="str">
+      <x:c r="F52" s="109" t="str">
         <x:v>Tự tính</x:v>
       </x:c>
       <x:c r="G52" s="43" t="str">
         <x:v>Chưa xét khấu hao, lãi vay và thuế.</x:v>
       </x:c>
-      <x:c r="H52" s="96"/>
-      <x:c r="I52" s="96"/>
-      <x:c r="J52" s="96"/>
-      <x:c r="K52" s="96"/>
+      <x:c r="H52" s="103"/>
+      <x:c r="I52" s="103"/>
+      <x:c r="J52" s="103"/>
+      <x:c r="K52" s="103"/>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
-      <x:c r="A53" s="103"/>
-      <x:c r="B53" s="96"/>
-      <x:c r="C53" s="103"/>
-      <x:c r="D53" s="96"/>
-      <x:c r="E53" s="103"/>
-      <x:c r="F53" s="103"/>
-      <x:c r="G53" s="105"/>
-      <x:c r="H53" s="96"/>
-      <x:c r="I53" s="96"/>
-      <x:c r="J53" s="96"/>
-      <x:c r="K53" s="96"/>
+      <x:c r="A53" s="110"/>
+      <x:c r="B53" s="103"/>
+      <x:c r="C53" s="110"/>
+      <x:c r="D53" s="103"/>
+      <x:c r="E53" s="110"/>
+      <x:c r="F53" s="110"/>
+      <x:c r="G53" s="112"/>
+      <x:c r="H53" s="103"/>
+      <x:c r="I53" s="103"/>
+      <x:c r="J53" s="103"/>
+      <x:c r="K53" s="103"/>
     </x:row>
     <x:row r="54" ht="22" hidden="0" customHeight="1">
-      <x:c r="A54" s="98" t="str">
+      <x:c r="A54" s="105" t="str">
         <x:v>6. CƠ CẤU VỐN VÀ KHOẢN VAY</x:v>
       </x:c>
       <x:c r="B54" s="40"/>
-      <x:c r="C54" s="98"/>
+      <x:c r="C54" s="105"/>
       <x:c r="D54" s="40"/>
-      <x:c r="E54" s="98"/>
-      <x:c r="F54" s="98"/>
-      <x:c r="G54" s="104"/>
-      <x:c r="H54" s="96"/>
-      <x:c r="I54" s="96"/>
-      <x:c r="J54" s="96"/>
-      <x:c r="K54" s="96"/>
+      <x:c r="E54" s="105"/>
+      <x:c r="F54" s="105"/>
+      <x:c r="G54" s="111"/>
+      <x:c r="H54" s="103"/>
+      <x:c r="I54" s="103"/>
+      <x:c r="J54" s="103"/>
+      <x:c r="K54" s="103"/>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
-      <x:c r="A55" s="102" t="str">
+      <x:c r="A55" s="109" t="str">
         <x:v>FIN-01</x:v>
       </x:c>
       <x:c r="B55" s="47" t="str">
         <x:v>Tỷ lệ vốn vay</x:v>
       </x:c>
-      <x:c r="C55" s="102" t="str">
+      <x:c r="C55" s="109" t="str">
         <x:v>Debt ratio</x:v>
       </x:c>
-      <x:c r="D55" s="59"/>
-      <x:c r="E55" s="102" t="str">
+      <x:c r="D55" s="60" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="E55" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F55" s="102" t="str">
+      <x:c r="F55" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G55" s="43" t="str">
-        <x:v>Tỷ lệ khoản vay trên cơ sở vốn đầu tư kinh tế.</x:v>
-      </x:c>
-      <x:c r="H55" s="96"/>
-      <x:c r="I55" s="96"/>
-      <x:c r="J55" s="96"/>
-      <x:c r="K55" s="96"/>
+        <x:v>Giả định typical 70% vốn vay.</x:v>
+      </x:c>
+      <x:c r="H55" s="103"/>
+      <x:c r="I55" s="103"/>
+      <x:c r="J55" s="103"/>
+      <x:c r="K55" s="103"/>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
-      <x:c r="A56" s="102" t="str">
+      <x:c r="A56" s="109" t="str">
         <x:v>FIN-02</x:v>
       </x:c>
       <x:c r="B56" s="47" t="str">
         <x:v>Tỷ lệ vốn chủ sở hữu</x:v>
       </x:c>
-      <x:c r="C56" s="102" t="str">
+      <x:c r="C56" s="109" t="str">
         <x:v>Equity ratio</x:v>
       </x:c>
-      <x:c r="D56" s="74" t="str">
+      <x:c r="D56" s="74" t="n">
         <x:f>IF(D55="","",1-D55)</x:f>
-      </x:c>
-      <x:c r="E56" s="102" t="str">
+        <x:v>0.30000000000000004</x:v>
+      </x:c>
+      <x:c r="E56" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F56" s="102" t="str">
+      <x:c r="F56" s="109" t="str">
         <x:v>Tự tính</x:v>
       </x:c>
       <x:c r="G56" s="43" t="str">
         <x:v>Bằng 100% trừ tỷ lệ vốn vay.</x:v>
       </x:c>
-      <x:c r="H56" s="96"/>
-      <x:c r="I56" s="96"/>
-      <x:c r="J56" s="96"/>
-      <x:c r="K56" s="96"/>
+      <x:c r="H56" s="103"/>
+      <x:c r="I56" s="103"/>
+      <x:c r="J56" s="103"/>
+      <x:c r="K56" s="103"/>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
-      <x:c r="A57" s="102" t="str">
+      <x:c r="A57" s="109" t="str">
         <x:v>FIN-03</x:v>
       </x:c>
       <x:c r="B57" s="47" t="str">
         <x:v>Lãi suất vay</x:v>
       </x:c>
-      <x:c r="C57" s="102" t="str">
+      <x:c r="C57" s="109" t="str">
         <x:v>Interest rate</x:v>
       </x:c>
-      <x:c r="D57" s="77"/>
-      <x:c r="E57" s="102" t="str">
+      <x:c r="D57" s="78" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="E57" s="109" t="str">
         <x:v>%/năm</x:v>
       </x:c>
-      <x:c r="F57" s="102" t="str">
+      <x:c r="F57" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G57" s="43" t="str">
-        <x:v>Lãi suất cố định trong Ver1.</x:v>
-      </x:c>
-      <x:c r="H57" s="96"/>
-      <x:c r="I57" s="96"/>
-      <x:c r="J57" s="96"/>
-      <x:c r="K57" s="96"/>
+        <x:v>Giả định typical 10%/năm, lãi suất cố định trong Ver1.</x:v>
+      </x:c>
+      <x:c r="H57" s="103"/>
+      <x:c r="I57" s="103"/>
+      <x:c r="J57" s="103"/>
+      <x:c r="K57" s="103"/>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
-      <x:c r="A58" s="102" t="str">
+      <x:c r="A58" s="109" t="str">
         <x:v>FIN-04</x:v>
       </x:c>
       <x:c r="B58" s="47" t="str">
         <x:v>Thời hạn vay</x:v>
       </x:c>
-      <x:c r="C58" s="102" t="str">
+      <x:c r="C58" s="109" t="str">
         <x:v>Debt tenor</x:v>
       </x:c>
-      <x:c r="D58" s="53"/>
-      <x:c r="E58" s="102" t="str">
+      <x:c r="D58" s="53" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E58" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F58" s="102" t="str">
+      <x:c r="F58" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G58" s="43" t="str">
-        <x:v>Tính từ thời điểm bắt đầu trả nợ.</x:v>
-      </x:c>
-      <x:c r="H58" s="96"/>
-      <x:c r="I58" s="96"/>
-      <x:c r="J58" s="96"/>
-      <x:c r="K58" s="96"/>
+        <x:v>Giả định typical, tính từ thời điểm bắt đầu trả nợ.</x:v>
+      </x:c>
+      <x:c r="H58" s="103"/>
+      <x:c r="I58" s="103"/>
+      <x:c r="J58" s="103"/>
+      <x:c r="K58" s="103"/>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
-      <x:c r="A59" s="102" t="str">
+      <x:c r="A59" s="109" t="str">
         <x:v>FIN-05</x:v>
       </x:c>
       <x:c r="B59" s="43" t="str">
         <x:v>Thời gian ân hạn gốc</x:v>
       </x:c>
-      <x:c r="C59" s="102" t="str">
+      <x:c r="C59" s="109" t="str">
         <x:v>Grace period</x:v>
       </x:c>
-      <x:c r="D59" s="61"/>
-      <x:c r="E59" s="102" t="str">
+      <x:c r="D59" s="62" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E59" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F59" s="102" t="str">
+      <x:c r="F59" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G59" s="43" t="str">
-        <x:v>Không vượt quá thời hạn vay.</x:v>
-      </x:c>
-      <x:c r="H59" s="96"/>
-      <x:c r="I59" s="96"/>
-      <x:c r="J59" s="96"/>
-      <x:c r="K59" s="96"/>
+        <x:v>Giả định bằng thời gian xây dựng.</x:v>
+      </x:c>
+      <x:c r="H59" s="103"/>
+      <x:c r="I59" s="103"/>
+      <x:c r="J59" s="103"/>
+      <x:c r="K59" s="103"/>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
-      <x:c r="A60" s="102" t="str">
+      <x:c r="A60" s="109" t="str">
         <x:v>FIN-06</x:v>
       </x:c>
       <x:c r="B60" s="43" t="str">
         <x:v>Phương thức trả gốc</x:v>
       </x:c>
-      <x:c r="C60" s="102" t="str">
+      <x:c r="C60" s="109" t="str">
         <x:v>Repayment</x:v>
       </x:c>
-      <x:c r="D60" s="49" t="str">
+      <x:c r="D60" s="75" t="str">
         <x:v>Gốc đều</x:v>
       </x:c>
-      <x:c r="E60" s="102" t="str">
+      <x:c r="E60" s="109" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="F60" s="102" t="str">
+      <x:c r="F60" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G60" s="43" t="str">
         <x:v>Chọn Gốc đều hoặc Niên kim.</x:v>
       </x:c>
-      <x:c r="H60" s="96"/>
-      <x:c r="I60" s="96"/>
-      <x:c r="J60" s="96"/>
-      <x:c r="K60" s="96"/>
+      <x:c r="H60" s="103"/>
+      <x:c r="I60" s="103"/>
+      <x:c r="J60" s="103"/>
+      <x:c r="K60" s="103"/>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
-      <x:c r="A61" s="102" t="str">
+      <x:c r="A61" s="109" t="str">
         <x:v>FIN-07</x:v>
       </x:c>
       <x:c r="B61" s="43" t="str">
         <x:v>Phí thu xếp khoản vay</x:v>
       </x:c>
-      <x:c r="C61" s="102" t="str">
+      <x:c r="C61" s="109" t="str">
         <x:v>Upfront fee</x:v>
       </x:c>
-      <x:c r="D61" s="76"/>
-      <x:c r="E61" s="102" t="str">
+      <x:c r="D61" s="77" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="E61" s="109" t="str">
         <x:v>% khoản vay</x:v>
       </x:c>
-      <x:c r="F61" s="102" t="str">
+      <x:c r="F61" s="109" t="str">
         <x:v>Tùy chọn</x:v>
       </x:c>
       <x:c r="G61" s="43" t="str">
-        <x:v>Nhập 0 nếu không áp dụng.</x:v>
-      </x:c>
-      <x:c r="H61" s="96"/>
-      <x:c r="I61" s="96"/>
-      <x:c r="J61" s="96"/>
-      <x:c r="K61" s="96"/>
+        <x:v>Giả định typical 1% giá trị khoản vay.</x:v>
+      </x:c>
+      <x:c r="H61" s="103"/>
+      <x:c r="I61" s="103"/>
+      <x:c r="J61" s="103"/>
+      <x:c r="K61" s="103"/>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
-      <x:c r="A62" s="102" t="str">
+      <x:c r="A62" s="109" t="str">
         <x:v>FIN-08</x:v>
       </x:c>
       <x:c r="B62" s="43" t="str">
         <x:v>DSCR tối thiểu yêu cầu</x:v>
       </x:c>
-      <x:c r="C62" s="102" t="str">
+      <x:c r="C62" s="109" t="str">
         <x:v>Minimum DSCR</x:v>
       </x:c>
-      <x:c r="D62" s="78"/>
-      <x:c r="E62" s="102" t="str">
+      <x:c r="D62" s="79" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="E62" s="109" t="str">
         <x:v>Lần</x:v>
       </x:c>
-      <x:c r="F62" s="102" t="str">
+      <x:c r="F62" s="109" t="str">
         <x:v>Tùy chọn</x:v>
       </x:c>
       <x:c r="G62" s="43" t="str">
-        <x:v>Dùng để kiểm tra khả năng trả nợ.</x:v>
-      </x:c>
-      <x:c r="H62" s="96"/>
-      <x:c r="I62" s="96"/>
-      <x:c r="J62" s="96"/>
-      <x:c r="K62" s="96"/>
+        <x:v>Giả định ngưỡng kiểm tra khả năng trả nợ.</x:v>
+      </x:c>
+      <x:c r="H62" s="103"/>
+      <x:c r="I62" s="103"/>
+      <x:c r="J62" s="103"/>
+      <x:c r="K62" s="103"/>
     </x:row>
     <x:row r="63" ht="15" hidden="0" customHeight="1">
-      <x:c r="A63" s="102" t="str">
+      <x:c r="A63" s="109" t="str">
         <x:v>FIN-09</x:v>
       </x:c>
       <x:c r="B63" s="47" t="str">
         <x:v>Giá trị khoản vay</x:v>
       </x:c>
-      <x:c r="C63" s="102" t="str">
+      <x:c r="C63" s="109" t="str">
         <x:v>Debt amount</x:v>
       </x:c>
-      <x:c r="D63" s="62" t="str">
+      <x:c r="D63" s="58" t="n">
         <x:f>IF(OR(D26="",D55=""),"",D26*D55)</x:f>
-      </x:c>
-      <x:c r="E63" s="102" t="str">
+        <x:v>3905.9999999999995</x:v>
+      </x:c>
+      <x:c r="E63" s="109" t="str">
         <x:v>Tỷ VND</x:v>
       </x:c>
-      <x:c r="F63" s="102" t="str">
+      <x:c r="F63" s="109" t="str">
         <x:v>Tự tính</x:v>
       </x:c>
       <x:c r="G63" s="43" t="str">
         <x:v>Chưa bao gồm lãi vay trong xây dựng và phí thu xếp vốn.</x:v>
       </x:c>
-      <x:c r="H63" s="96"/>
-      <x:c r="I63" s="96"/>
-      <x:c r="J63" s="96"/>
-      <x:c r="K63" s="96"/>
+      <x:c r="H63" s="103"/>
+      <x:c r="I63" s="103"/>
+      <x:c r="J63" s="103"/>
+      <x:c r="K63" s="103"/>
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
-      <x:c r="A64" s="102" t="str">
+      <x:c r="A64" s="109" t="str">
         <x:v>FIN-10</x:v>
       </x:c>
       <x:c r="B64" s="47" t="str">
         <x:v>Vốn chủ sở hữu ban đầu</x:v>
       </x:c>
-      <x:c r="C64" s="102" t="str">
+      <x:c r="C64" s="109" t="str">
         <x:v>Equity amount</x:v>
       </x:c>
-      <x:c r="D64" s="62" t="str">
+      <x:c r="D64" s="58" t="n">
         <x:f>IF(OR(D26="",D63=""),"",D26-D63)</x:f>
-      </x:c>
-      <x:c r="E64" s="102" t="str">
+        <x:v>1674.0000000000005</x:v>
+      </x:c>
+      <x:c r="E64" s="109" t="str">
         <x:v>Tỷ VND</x:v>
       </x:c>
-      <x:c r="F64" s="102" t="str">
+      <x:c r="F64" s="109" t="str">
         <x:v>Tự tính</x:v>
       </x:c>
       <x:c r="G64" s="43" t="str">
         <x:v>Phần cơ sở vốn đầu tư kinh tế không được tài trợ bằng khoản vay.</x:v>
       </x:c>
-      <x:c r="H64" s="96"/>
-      <x:c r="I64" s="96"/>
-      <x:c r="J64" s="96"/>
-      <x:c r="K64" s="96"/>
+      <x:c r="H64" s="103"/>
+      <x:c r="I64" s="103"/>
+      <x:c r="J64" s="103"/>
+      <x:c r="K64" s="103"/>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
-      <x:c r="A65" s="103"/>
-      <x:c r="B65" s="96"/>
-      <x:c r="C65" s="103"/>
-      <x:c r="D65" s="96"/>
-      <x:c r="E65" s="103"/>
-      <x:c r="F65" s="103"/>
-      <x:c r="G65" s="105"/>
-      <x:c r="H65" s="96"/>
-      <x:c r="I65" s="96"/>
-      <x:c r="J65" s="96"/>
-      <x:c r="K65" s="96"/>
+      <x:c r="A65" s="110"/>
+      <x:c r="B65" s="103"/>
+      <x:c r="C65" s="110"/>
+      <x:c r="D65" s="103"/>
+      <x:c r="E65" s="110"/>
+      <x:c r="F65" s="110"/>
+      <x:c r="G65" s="112"/>
+      <x:c r="H65" s="103"/>
+      <x:c r="I65" s="103"/>
+      <x:c r="J65" s="103"/>
+      <x:c r="K65" s="103"/>
     </x:row>
     <x:row r="66" ht="22" hidden="0" customHeight="1">
-      <x:c r="A66" s="98" t="str">
+      <x:c r="A66" s="105" t="str">
         <x:v>7. THUẾ, KHẤU HAO VÀ TỶ LỆ CHIẾT KHẤU</x:v>
       </x:c>
       <x:c r="B66" s="40"/>
-      <x:c r="C66" s="98"/>
+      <x:c r="C66" s="105"/>
       <x:c r="D66" s="40"/>
-      <x:c r="E66" s="98"/>
-      <x:c r="F66" s="98"/>
-      <x:c r="G66" s="104"/>
-      <x:c r="H66" s="96"/>
-      <x:c r="I66" s="96"/>
-      <x:c r="J66" s="96"/>
-      <x:c r="K66" s="96"/>
+      <x:c r="E66" s="105"/>
+      <x:c r="F66" s="105"/>
+      <x:c r="G66" s="111"/>
+      <x:c r="H66" s="103"/>
+      <x:c r="I66" s="103"/>
+      <x:c r="J66" s="103"/>
+      <x:c r="K66" s="103"/>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
-      <x:c r="A67" s="102" t="str">
+      <x:c r="A67" s="109" t="str">
         <x:v>TAX-01</x:v>
       </x:c>
       <x:c r="B67" s="47" t="str">
         <x:v>Thuế suất thuế TNDN thông thường</x:v>
       </x:c>
-      <x:c r="C67" s="102" t="str">
+      <x:c r="C67" s="109" t="str">
         <x:v>CIT standard</x:v>
       </x:c>
-      <x:c r="D67" s="59"/>
-      <x:c r="E67" s="102" t="str">
+      <x:c r="D67" s="60" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="E67" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F67" s="102" t="str">
+      <x:c r="F67" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G67" s="43" t="str">
-        <x:v>Nhập theo quy định áp dụng cho dự án.</x:v>
-      </x:c>
-      <x:c r="H67" s="96"/>
-      <x:c r="I67" s="96"/>
-      <x:c r="J67" s="96"/>
-      <x:c r="K67" s="96"/>
-    </x:row>
-    <x:row r="68" ht="15" hidden="0" customHeight="1">
-      <x:c r="A68" s="102" t="str">
+        <x:v>Thuế suất phổ thông dùng làm giả định cơ sở.</x:v>
+      </x:c>
+      <x:c r="H67" s="103"/>
+      <x:c r="I67" s="103"/>
+      <x:c r="J67" s="103"/>
+      <x:c r="K67" s="103"/>
+    </x:row>
+    <x:row r="68" ht="24" hidden="0" customHeight="1">
+      <x:c r="A68" s="109" t="str">
         <x:v>TAX-02</x:v>
       </x:c>
       <x:c r="B68" s="43" t="str">
         <x:v>Thuế suất thuế TNDN ưu đãi</x:v>
       </x:c>
-      <x:c r="C68" s="102" t="str">
+      <x:c r="C68" s="109" t="str">
         <x:v>CIT incentive</x:v>
       </x:c>
-      <x:c r="D68" s="60"/>
-      <x:c r="E68" s="102" t="str">
+      <x:c r="D68" s="61" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="E68" s="109" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F68" s="102" t="str">
+      <x:c r="F68" s="109" t="str">
         <x:v>Tùy chọn</x:v>
       </x:c>
       <x:c r="G68" s="43" t="str">
-        <x:v>Để trống nếu không được hưởng ưu đãi.</x:v>
-      </x:c>
-      <x:c r="H68" s="96"/>
-      <x:c r="I68" s="96"/>
-      <x:c r="J68" s="96"/>
-      <x:c r="K68" s="96"/>
+        <x:v>Giả định dự án đầu tư mới năng lượng tái tạo đủ điều kiện; cần xác minh pháp lý.</x:v>
+      </x:c>
+      <x:c r="H68" s="103"/>
+      <x:c r="I68" s="103"/>
+      <x:c r="J68" s="103"/>
+      <x:c r="K68" s="103"/>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
-      <x:c r="A69" s="102" t="str">
+      <x:c r="A69" s="109" t="str">
         <x:v>TAX-03</x:v>
       </x:c>
       <x:c r="B69" s="43" t="str">
         <x:v>Thời gian áp dụng thuế suất ưu đãi</x:v>
       </x:c>
-      <x:c r="C69" s="102" t="str">
+      <x:c r="C69" s="109" t="str">
         <x:v>Incentive period</x:v>
       </x:c>
-      <x:c r="D69" s="51"/>
-      <x:c r="E69" s="102" t="str">
+      <x:c r="D69" s="52" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E69" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F69" s="102" t="str">
+      <x:c r="F69" s="109" t="str">
         <x:v>Tùy chọn</x:v>
       </x:c>
       <x:c r="G69" s="43" t="str">
-        <x:v>Nhập 0 nếu không áp dụng.</x:v>
-      </x:c>
-      <x:c r="H69" s="96"/>
-      <x:c r="I69" s="96"/>
-      <x:c r="J69" s="96"/>
-      <x:c r="K69" s="96"/>
+        <x:v>Giả định ưu đãi 10% trong 15 năm.</x:v>
+      </x:c>
+      <x:c r="H69" s="103"/>
+      <x:c r="I69" s="103"/>
+      <x:c r="J69" s="103"/>
+      <x:c r="K69" s="103"/>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
-      <x:c r="A70" s="102" t="str">
+      <x:c r="A70" s="109" t="str">
         <x:v>TAX-04</x:v>
       </x:c>
       <x:c r="B70" s="43" t="str">
         <x:v>Thời gian miễn thuế</x:v>
       </x:c>
-      <x:c r="C70" s="102" t="str">
+      <x:c r="C70" s="109" t="str">
         <x:v>Tax holiday</x:v>
       </x:c>
-      <x:c r="D70" s="51"/>
-      <x:c r="E70" s="102" t="str">
+      <x:c r="D70" s="52" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E70" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F70" s="102" t="str">
+      <x:c r="F70" s="109" t="str">
         <x:v>Tùy chọn</x:v>
       </x:c>
       <x:c r="G70" s="43" t="str">
-        <x:v>Tính từ năm phát sinh thu nhập chịu thuế theo quy định áp dụng.</x:v>
-      </x:c>
-      <x:c r="H70" s="96"/>
-      <x:c r="I70" s="96"/>
-      <x:c r="J70" s="96"/>
-      <x:c r="K70" s="96"/>
+        <x:v>Giả định miễn thuế 4 năm; cần xác minh thời điểm bắt đầu ưu đãi.</x:v>
+      </x:c>
+      <x:c r="H70" s="103"/>
+      <x:c r="I70" s="103"/>
+      <x:c r="J70" s="103"/>
+      <x:c r="K70" s="103"/>
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
-      <x:c r="A71" s="102" t="str">
+      <x:c r="A71" s="109" t="str">
         <x:v>TAX-05</x:v>
       </x:c>
       <x:c r="B71" s="43" t="str">
         <x:v>Thời gian giảm 50% thuế</x:v>
       </x:c>
-      <x:c r="C71" s="102" t="str">
+      <x:c r="C71" s="109" t="str">
         <x:v>Tax reduction</x:v>
       </x:c>
-      <x:c r="D71" s="51"/>
-      <x:c r="E71" s="102" t="str">
+      <x:c r="D71" s="52" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E71" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F71" s="102" t="str">
+      <x:c r="F71" s="109" t="str">
         <x:v>Tùy chọn</x:v>
       </x:c>
       <x:c r="G71" s="43" t="str">
-        <x:v>Giai đoạn sau thời gian miễn thuế.</x:v>
-      </x:c>
-      <x:c r="H71" s="96"/>
-      <x:c r="I71" s="96"/>
-      <x:c r="J71" s="96"/>
-      <x:c r="K71" s="96"/>
+        <x:v>Giả định giảm 50% thuế trong 9 năm tiếp theo.</x:v>
+      </x:c>
+      <x:c r="H71" s="103"/>
+      <x:c r="I71" s="103"/>
+      <x:c r="J71" s="103"/>
+      <x:c r="K71" s="103"/>
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
-      <x:c r="A72" s="102" t="str">
+      <x:c r="A72" s="109" t="str">
         <x:v>TAX-06</x:v>
       </x:c>
       <x:c r="B72" s="47" t="str">
         <x:v>Thời gian khấu hao tài sản</x:v>
       </x:c>
-      <x:c r="C72" s="102" t="str">
+      <x:c r="C72" s="109" t="str">
         <x:v>Depreciation life</x:v>
       </x:c>
-      <x:c r="D72" s="53"/>
-      <x:c r="E72" s="102" t="str">
+      <x:c r="D72" s="53" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E72" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F72" s="102" t="str">
+      <x:c r="F72" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G72" s="43" t="str">
-        <x:v>Ver1 áp dụng phương pháp đường thẳng.</x:v>
-      </x:c>
-      <x:c r="H72" s="96"/>
-      <x:c r="I72" s="96"/>
-      <x:c r="J72" s="96"/>
-      <x:c r="K72" s="96"/>
+        <x:v>Giả định khấu hao đường thẳng theo thời gian vận hành.</x:v>
+      </x:c>
+      <x:c r="H72" s="103"/>
+      <x:c r="I72" s="103"/>
+      <x:c r="J72" s="103"/>
+      <x:c r="K72" s="103"/>
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
-      <x:c r="A73" s="102" t="str">
+      <x:c r="A73" s="109" t="str">
         <x:v>TAX-07</x:v>
       </x:c>
       <x:c r="B73" s="43" t="str">
         <x:v>Thời gian chuyển lỗ tối đa</x:v>
       </x:c>
-      <x:c r="C73" s="102" t="str">
+      <x:c r="C73" s="109" t="str">
         <x:v>Loss carryforward</x:v>
       </x:c>
-      <x:c r="D73" s="51"/>
-      <x:c r="E73" s="102" t="str">
+      <x:c r="D73" s="52" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E73" s="109" t="str">
         <x:v>Năm</x:v>
       </x:c>
-      <x:c r="F73" s="102" t="str">
+      <x:c r="F73" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G73" s="43" t="str">
-        <x:v>Nhập theo quy định áp dụng tại thời điểm tính toán.</x:v>
-      </x:c>
-      <x:c r="H73" s="96"/>
-      <x:c r="I73" s="96"/>
-      <x:c r="J73" s="96"/>
-      <x:c r="K73" s="96"/>
+        <x:v>Giả định cơ sở; cần cập nhật theo quy định áp dụng.</x:v>
+      </x:c>
+      <x:c r="H73" s="103"/>
+      <x:c r="I73" s="103"/>
+      <x:c r="J73" s="103"/>
+      <x:c r="K73" s="103"/>
     </x:row>
     <x:row r="74" ht="15" hidden="0" customHeight="1">
-      <x:c r="A74" s="102" t="str">
+      <x:c r="A74" s="109" t="str">
         <x:v>VAL-01</x:v>
       </x:c>
       <x:c r="B74" s="47" t="str">
         <x:v>Tỷ lệ chiết khấu dự án</x:v>
       </x:c>
-      <x:c r="C74" s="102" t="str">
+      <x:c r="C74" s="109" t="str">
         <x:v>Project discount</x:v>
       </x:c>
-      <x:c r="D74" s="77"/>
-      <x:c r="E74" s="102" t="str">
+      <x:c r="D74" s="78" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="E74" s="109" t="str">
         <x:v>%/năm</x:v>
       </x:c>
-      <x:c r="F74" s="102" t="str">
+      <x:c r="F74" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G74" s="43" t="str">
-        <x:v>Dùng tính Project NPV.</x:v>
-      </x:c>
-      <x:c r="H74" s="96"/>
-      <x:c r="I74" s="96"/>
-      <x:c r="J74" s="96"/>
-      <x:c r="K74" s="96"/>
+        <x:v>Giả định typical dùng tính Project NPV.</x:v>
+      </x:c>
+      <x:c r="H74" s="103"/>
+      <x:c r="I74" s="103"/>
+      <x:c r="J74" s="103"/>
+      <x:c r="K74" s="103"/>
     </x:row>
     <x:row r="75" ht="15" hidden="0" customHeight="1">
-      <x:c r="A75" s="102" t="str">
+      <x:c r="A75" s="109" t="str">
         <x:v>VAL-02</x:v>
       </x:c>
       <x:c r="B75" s="47" t="str">
         <x:v>Tỷ lệ chiết khấu vốn chủ sở hữu</x:v>
       </x:c>
-      <x:c r="C75" s="102" t="str">
+      <x:c r="C75" s="109" t="str">
         <x:v>Equity discount</x:v>
       </x:c>
-      <x:c r="D75" s="77"/>
-      <x:c r="E75" s="102" t="str">
+      <x:c r="D75" s="78" t="n">
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="E75" s="109" t="str">
         <x:v>%/năm</x:v>
       </x:c>
-      <x:c r="F75" s="102" t="str">
+      <x:c r="F75" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G75" s="43" t="str">
-        <x:v>Dùng tính Equity NPV.</x:v>
-      </x:c>
-      <x:c r="H75" s="96"/>
-      <x:c r="I75" s="96"/>
-      <x:c r="J75" s="96"/>
-      <x:c r="K75" s="96"/>
+        <x:v>Giả định typical dùng tính Equity NPV.</x:v>
+      </x:c>
+      <x:c r="H75" s="103"/>
+      <x:c r="I75" s="103"/>
+      <x:c r="J75" s="103"/>
+      <x:c r="K75" s="103"/>
     </x:row>
     <x:row r="76" ht="15" hidden="0" customHeight="1">
-      <x:c r="A76" s="96"/>
-      <x:c r="B76" s="96"/>
-      <x:c r="C76" s="96"/>
-      <x:c r="D76" s="96"/>
-      <x:c r="E76" s="96"/>
-      <x:c r="F76" s="96"/>
-      <x:c r="G76" s="105"/>
-      <x:c r="H76" s="96"/>
-      <x:c r="I76" s="96"/>
-      <x:c r="J76" s="96"/>
-      <x:c r="K76" s="96"/>
+      <x:c r="A76" s="103"/>
+      <x:c r="B76" s="103"/>
+      <x:c r="C76" s="103"/>
+      <x:c r="D76" s="103"/>
+      <x:c r="E76" s="103"/>
+      <x:c r="F76" s="103"/>
+      <x:c r="G76" s="112"/>
+      <x:c r="H76" s="103"/>
+      <x:c r="I76" s="103"/>
+      <x:c r="J76" s="103"/>
+      <x:c r="K76" s="103"/>
     </x:row>
     <x:row r="77" ht="15" hidden="0" customHeight="1">
-      <x:c r="A77" s="96"/>
-      <x:c r="B77" s="96"/>
-      <x:c r="C77" s="96"/>
-      <x:c r="D77" s="96"/>
-      <x:c r="E77" s="96"/>
-      <x:c r="F77" s="96"/>
-      <x:c r="G77" s="105"/>
-      <x:c r="H77" s="96"/>
-      <x:c r="I77" s="96"/>
-      <x:c r="J77" s="96"/>
-      <x:c r="K77" s="96"/>
+      <x:c r="A77" s="103"/>
+      <x:c r="B77" s="103"/>
+      <x:c r="C77" s="103"/>
+      <x:c r="D77" s="103"/>
+      <x:c r="E77" s="103"/>
+      <x:c r="F77" s="103"/>
+      <x:c r="G77" s="112"/>
+      <x:c r="H77" s="103"/>
+      <x:c r="I77" s="103"/>
+      <x:c r="J77" s="103"/>
+      <x:c r="K77" s="103"/>
     </x:row>
     <x:row r="78" ht="15" hidden="0" customHeight="1">
-      <x:c r="A78" s="82" t="str">
+      <x:c r="A78" s="83" t="str">
         <x:v>Ghi chú: các giả định pháp lý, thuế, giá điện và ưu đãi phải được cập nhật theo hồ sơ và quy định áp dụng cho từng dự án.</x:v>
       </x:c>
-      <x:c r="B78" s="82"/>
-      <x:c r="C78" s="82"/>
-      <x:c r="D78" s="82"/>
-      <x:c r="E78" s="82"/>
-      <x:c r="F78" s="82"/>
-      <x:c r="G78" s="82"/>
-      <x:c r="H78" s="96"/>
-      <x:c r="I78" s="96"/>
-      <x:c r="J78" s="96"/>
-      <x:c r="K78" s="96"/>
+      <x:c r="B78" s="83"/>
+      <x:c r="C78" s="83"/>
+      <x:c r="D78" s="83"/>
+      <x:c r="E78" s="83"/>
+      <x:c r="F78" s="83"/>
+      <x:c r="G78" s="83"/>
+      <x:c r="H78" s="103"/>
+      <x:c r="I78" s="103"/>
+      <x:c r="J78" s="103"/>
+      <x:c r="K78" s="103"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="1"/>
@@ -2575,21 +2808,18 @@
       <x:formula>1</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J20:J20">
+  <x:conditionalFormatting sqref="J23:J23">
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="OK"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="CHƯA"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="17">
-    <x:dataValidation type="list" sqref="D12">
-      <x:formula1>"VND"</x:formula1>
-    </x:dataValidation>
+  <x:dataValidations count="18">
     <x:dataValidation type="list" sqref="D40">
       <x:formula1>"P50,P75,P90,Khác"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D60">
       <x:formula1>"Gốc đều,Niên kim"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="decimal" operator="between" sqref="D22:D23">
+    <x:dataValidation type="decimal" operator="between" sqref="D23:D24">
       <x:formula1>0</x:formula1>
       <x:formula2>1</x:formula2>
     </x:dataValidation>
@@ -2597,11 +2827,15 @@
       <x:formula1>0</x:formula1>
       <x:formula2>1</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="decimal" operator="between" sqref="D42:D44">
+    <x:dataValidation type="decimal" operator="between" sqref="D41">
       <x:formula1>0</x:formula1>
       <x:formula2>1</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="decimal" operator="between" sqref="D46">
+    <x:dataValidation type="decimal" operator="between" sqref="D43">
+      <x:formula1>0</x:formula1>
+      <x:formula2>1</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="D45">
       <x:formula1>0</x:formula1>
       <x:formula2>1</x:formula2>
     </x:dataValidation>
@@ -2629,6 +2863,10 @@
       <x:formula1>0</x:formula1>
       <x:formula2>1</x:formula2>
     </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="D12">
+      <x:formula1>0</x:formula1>
+      <x:formula2>10000</x:formula2>
+    </x:dataValidation>
     <x:dataValidation type="whole" operator="between" sqref="D15">
       <x:formula1>0</x:formula1>
       <x:formula2>100</x:formula2>
@@ -2647,5 +2885,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0c12f2004574987"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Làm dịu màu nền sheet Input
</commit_message>
<xml_diff>
--- a/PTKTTC_Ver1.xlsx
+++ b/PTKTTC_Ver1.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" r:id="R1de55419e3224262"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" r:id="Reaed320938c2499a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10,11 +10,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={11F66432-3307-873B-12A7-4C732E0186EA}</x:author>
-    <x:author>tc={F3757FEC-73D4-ABA4-0914-CE3007BB35CA}</x:author>
-    <x:author>tc={F2BADE1D-790A-3D7B-F48A-7A5B2281F0C8}</x:author>
-    <x:author>tc={D528358C-641E-4296-3905-F551C67979C5}</x:author>
-    <x:author>tc={C36BD088-EB2C-AE04-C47F-4F689DECD2D5}</x:author>
+    <x:author>tc={B7BFDAC7-1D29-6E41-163F-B290611BE5CD}</x:author>
+    <x:author>tc={9875F86A-E2BE-88A0-4D54-84FA999D4C19}</x:author>
+    <x:author>tc={8F46B198-BF1E-BE29-6718-D6EE5BD5C993}</x:author>
+    <x:author>tc={31AF7879-C221-0607-98D5-BB3DE4317D9D}</x:author>
+    <x:author>tc={2A959A44-9F3A-8259-3143-8D1603DF8060}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="D22" authorId="0">
@@ -91,7 +91,7 @@
     <x:numFmt numFmtId="210" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="211" formatCode="@"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -121,7 +121,7 @@
     <x:font>
       <x:b/>
       <x:sz val="10"/>
-      <x:color rgb="FFFFFFFF"/>
+      <x:color rgb="FF4F6D8A"/>
       <x:name val="Arial"/>
     </x:font>
     <x:font>
@@ -143,6 +143,12 @@
       <x:name val="Arial"/>
     </x:font>
     <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
       <x:sz val="10"/>
       <x:color rgb="FFFF0000"/>
       <x:name val="Arial"/>
@@ -157,7 +163,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF17365D"/>
+        <x:fgColor rgb="FF4F6D8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF5FA"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -167,17 +178,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF1F4E78"/>
+        <x:fgColor rgb="FFFFF9E8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF2CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFEAF2F8"/>
+        <x:fgColor rgb="FFF1F6FA"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -190,32 +196,32 @@
     <x:border/>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFB8C6D1"/>
+        <x:color rgb="FFCEDAE3"/>
       </x:left>
       <x:top style="thin">
-        <x:color rgb="FFB8C6D1"/>
+        <x:color rgb="FFCEDAE3"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFB8C6D1"/>
+        <x:color rgb="FFCEDAE3"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:top style="thin">
-        <x:color rgb="FFB8C6D1"/>
+        <x:color rgb="FFCEDAE3"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFB8C6D1"/>
+        <x:color rgb="FFCEDAE3"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:right style="thin">
-        <x:color rgb="FFB8C6D1"/>
+        <x:color rgb="FFCEDAE3"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFB8C6D1"/>
+        <x:color rgb="FFCEDAE3"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFB8C6D1"/>
+        <x:color rgb="FFCEDAE3"/>
       </x:bottom>
     </x:border>
     <x:border>
@@ -276,35 +282,35 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -338,13 +344,13 @@
     <x:xf numFmtId="200" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -371,13 +377,13 @@
     <x:xf numFmtId="203" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="203" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="203" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="204" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="204" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="202" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -405,19 +411,19 @@
     <x:xf numFmtId="203" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="205" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="206" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="206" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="206" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="207" fontId="9" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -428,7 +434,7 @@
     <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -494,7 +500,7 @@
     <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -530,7 +536,7 @@
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFEDF6E9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -541,7 +547,7 @@
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFFCEFE8"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -552,7 +558,7 @@
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFEDF6E9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -563,7 +569,7 @@
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFFCEFE8"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -573,7 +579,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Hoang" id="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}"/>
+  <xltc:person displayName="Hoang" id="{5399D1AD-F6B8-4E79-95C8-42830BC6C90C}"/>
 </xltc:personList>
 </file>
 
@@ -770,19 +776,19 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="D22" dT="2026-07-27T08:40:11.144" personId="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}" id="{11F66432-3307-873B-12A7-4C732E0186EA}">
+  <xltc:threadedComment ref="D22" dT="2026-07-27T08:50:21.525" personId="{5399D1AD-F6B8-4E79-95C8-42830BC6C90C}" id="{B7BFDAC7-1D29-6E41-163F-B290611BE5CD}">
     <xltc:text>Nguồn: thông tin do người dùng cung cấp — suất vốn đầu tư 31 tỷ VND/MW.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="D41" dT="2026-07-27T08:40:11.145" personId="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}" id="{F3757FEC-73D4-ABA4-0914-CE3007BB35CA}">
+  <xltc:threadedComment ref="D41" dT="2026-07-27T08:50:21.525" personId="{5399D1AD-F6B8-4E79-95C8-42830BC6C90C}" id="{9875F86A-E2BE-88A0-4D54-84FA999D4C19}">
     <xltc:text>Giả định typical 30% dùng cho mô hình sơ bộ. Đây không phải kết quả nghiên cứu năng lượng; cần thay bằng AEP P50/P90 từ WindPRO hoặc báo cáo đánh giá năng lượng.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="D44" dT="2026-07-27T08:40:11.145" personId="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}" id="{F2BADE1D-790A-3D7B-F48A-7A5B2281F0C8}">
+  <xltc:threadedComment ref="D44" dT="2026-07-27T08:50:21.525" personId="{5399D1AD-F6B8-4E79-95C8-42830BC6C90C}" id="{8F46B198-BF1E-BE29-6718-D6EE5BD5C993}">
     <xltc:text>Nguồn: Quyết định 1508/QĐ-BCT ngày 30/05/2025 của Bộ Công Thương. Giá tối đa điện gió trên đất liền khu vực miền Trung: 1.807,4 VND/kWh, chưa VAT. https://moit.gov.vn/van-ban-phap-luat/quyet-dinh-phe-duyet-khung-gia-phat-dien-loai-hinh-nha-may-dien-gio-nam-2025.html</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="D50" dT="2026-07-27T08:40:11.145" personId="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}" id="{D528358C-641E-4296-3905-F551C67979C5}">
+  <xltc:threadedComment ref="D50" dT="2026-07-27T08:50:21.525" personId="{5399D1AD-F6B8-4E79-95C8-42830BC6C90C}" id="{31AF7879-C221-0607-98D5-BB3DE4317D9D}">
     <xltc:text>Giả định typical: O&amp;M năm đầu bằng 2% CAPEX chưa VAT = 111,6 tỷ VND/năm. Cần thay bằng báo giá O&amp;M và ngân sách vận hành thực tế.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="D68" dT="2026-07-27T08:40:11.145" personId="{BD68F277-147F-47CB-A8ED-08E9266B3DA7}" id="{C36BD088-EB2C-AE04-C47F-4F689DECD2D5}">
+  <xltc:threadedComment ref="D68" dT="2026-07-27T08:50:21.525" personId="{5399D1AD-F6B8-4E79-95C8-42830BC6C90C}" id="{2A959A44-9F3A-8259-3143-8D1603DF8060}">
     <xltc:text>Giả định dự án đầu tư mới trong lĩnh vực sản xuất năng lượng tái tạo đủ điều kiện ưu đãi: thuế suất 10% trong 15 năm, miễn 4 năm và giảm 50% trong 9 năm tiếp theo. Phải xác minh điều kiện áp dụng theo Luật Thuế TNDN 2025 và Nghị định 320/2025/NĐ-CP. https://vanban.chinhphu.vn/?classid=0&amp;docid=217301&amp;pageid=27160</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -837,7 +843,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="104" t="str">
-        <x:v>Phiên bản: Ver1.1  |  Cập nhật: 27/07/2026  |  Đơn vị tiền tệ mặc định: tỷ VND</x:v>
+        <x:v>Phiên bản: Ver1.2  |  Cập nhật: 27/07/2026  |  Đơn vị tiền tệ mặc định: tỷ VND</x:v>
       </x:c>
       <x:c r="B3" s="104"/>
       <x:c r="C3" s="104"/>
@@ -2885,6 +2891,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0c12f2004574987"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02aef2b4977b4ea1"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Đổi đầu vào O&M sang tỷ lệ phần trăm
</commit_message>
<xml_diff>
--- a/PTKTTC_Ver1.xlsx
+++ b/PTKTTC_Ver1.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" r:id="R7271295a915e49d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8095c89160d54f1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX" sheetId="3" r:id="R642e7173973a411b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy_Revenue" sheetId="4" r:id="Rc4172869388249ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" r:id="R066797bb175d4a61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dep_Tax" sheetId="6" r:id="R0d4ea2a3842b464e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income_Statement" sheetId="7" r:id="R99b0d551c4a249bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_CF" sheetId="8" r:id="Ra0762a9c63944e9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity_CF" sheetId="9" r:id="Rce55335ccd164bcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="10" r:id="R56adc6b70baa4f51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" r:id="Rc310633ffde44cec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R061370693bf6492e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX" sheetId="3" r:id="Reb06c5ec79324dd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy_Revenue" sheetId="4" r:id="R0cc2f33818df45df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" r:id="Rea1521bda04f41ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dep_Tax" sheetId="6" r:id="R76dfcb523ed9434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income_Statement" sheetId="7" r:id="Rda7ac03acc1d4187"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_CF" sheetId="8" r:id="R9abbdf0a67804dec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity_CF" sheetId="9" r:id="R1e06b0648fc44981"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="10" r:id="R22615fcf2ae643c2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -923,7 +923,7 @@
         <x:color rgb="FF0000FF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDF6E9"/>
         </x:patternFill>
       </x:fill>
@@ -934,7 +934,7 @@
         <x:color rgb="FF0000FF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCEFE8"/>
         </x:patternFill>
       </x:fill>
@@ -945,7 +945,7 @@
         <x:color rgb="FF0000FF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDF6E9"/>
         </x:patternFill>
       </x:fill>
@@ -956,7 +956,7 @@
         <x:color rgb="FF0000FF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCEFE8"/>
         </x:patternFill>
       </x:fill>
@@ -967,7 +967,7 @@
         <x:color rgb="FF0000FF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDF6E9"/>
         </x:patternFill>
       </x:fill>
@@ -978,7 +978,7 @@
         <x:color rgb="FF0000FF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCEFE8"/>
         </x:patternFill>
       </x:fill>
@@ -989,7 +989,7 @@
         <x:color rgb="FF0000FF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDF6E9"/>
         </x:patternFill>
       </x:fill>
@@ -1000,7 +1000,7 @@
         <x:color rgb="FF0000FF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCEFE8"/>
         </x:patternFill>
       </x:fill>
@@ -1011,7 +1011,7 @@
         <x:color rgb="FF0000FF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCEFE8"/>
         </x:patternFill>
       </x:fill>
@@ -1217,26 +1217,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
-<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="D22" dT="2026-07-27T09:21:44.555" personId="{A7C94DE6-BFEF-4531-80F3-2D14DAFDEC46}" id="{6A2E3B1B-9407-B749-7A6F-5B7C53F5F3C9}">
-    <xltc:text>Nguồn: thông tin do người dùng cung cấp — suất vốn đầu tư 31 tỷ VND/MW.</xltc:text>
-  </xltc:threadedComment>
-  <xltc:threadedComment ref="D41" dT="2026-07-27T09:21:44.555" personId="{A7C94DE6-BFEF-4531-80F3-2D14DAFDEC46}" id="{FDA12B2D-7334-BD06-EE56-079B86C335DF}">
-    <xltc:text>Giả định typical 30% dùng cho mô hình sơ bộ. Đây không phải kết quả nghiên cứu năng lượng; cần thay bằng AEP P50/P90 từ WindPRO hoặc báo cáo đánh giá năng lượng.</xltc:text>
-  </xltc:threadedComment>
-  <xltc:threadedComment ref="D44" dT="2026-07-27T09:21:44.555" personId="{A7C94DE6-BFEF-4531-80F3-2D14DAFDEC46}" id="{B278CF10-436C-DECA-7701-3C37B52FA94C}">
-    <xltc:text>Nguồn: Quyết định 1508/QĐ-BCT ngày 30/05/2025 của Bộ Công Thương. Giá tối đa điện gió trên đất liền khu vực miền Trung: 1.807,4 VND/kWh, chưa VAT. https://moit.gov.vn/van-ban-phap-luat/quyet-dinh-phe-duyet-khung-gia-phat-dien-loai-hinh-nha-may-dien-gio-nam-2025.html</xltc:text>
-  </xltc:threadedComment>
-  <xltc:threadedComment ref="D50" dT="2026-07-27T09:21:44.555" personId="{A7C94DE6-BFEF-4531-80F3-2D14DAFDEC46}" id="{79DE71C1-AC21-2323-5D41-24758D7A6A98}">
-    <xltc:text>Giả định typical: O&amp;M năm đầu bằng 2% CAPEX chưa VAT = 111,6 tỷ VND/năm. Cần thay bằng báo giá O&amp;M và ngân sách vận hành thực tế.</xltc:text>
-  </xltc:threadedComment>
-  <xltc:threadedComment ref="D68" dT="2026-07-27T09:21:44.555" personId="{A7C94DE6-BFEF-4531-80F3-2D14DAFDEC46}" id="{2201F049-C49D-F388-2DB2-A6B4639059FA}">
-    <xltc:text>Giả định dự án đầu tư mới trong lĩnh vực sản xuất năng lượng tái tạo đủ điều kiện ưu đãi: thuế suất 10% trong 15 năm, miễn 4 năm và giảm 50% trong 9 năm tiếp theo. Phải xác minh điều kiện áp dụng theo Luật Thuế TNDN 2025 và Nghị định 320/2025/NĐ-CP. https://vanban.chinhphu.vn/?classid=0&amp;docid=217301&amp;pageid=27160</xltc:text>
-  </xltc:threadedComment>
-</xltc:ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1730,8 +1710,8 @@
         <x:v>Chi phí O&amp;M năm đầu</x:v>
       </x:c>
       <x:c r="J19" s="93" t="n">
-        <x:f>IF(D50="","",D50)</x:f>
-        <x:v>111.6</x:v>
+        <x:f>IF(OR(D21="",D50=""),"",D21*D50)</x:f>
+        <x:v>111.60000000000001</x:v>
       </x:c>
       <x:c r="K19" s="85" t="str">
         <x:v>Tỷ VND</x:v>
@@ -2489,22 +2469,22 @@
         <x:v>OPE-01</x:v>
       </x:c>
       <x:c r="B50" s="47" t="str">
-        <x:v>Chi phí O&amp;M năm đầu</x:v>
+        <x:v>Tỷ lệ chi phí O&amp;M năm đầu trên CAPEX</x:v>
       </x:c>
       <x:c r="C50" s="109" t="str">
-        <x:v>O&amp;M Y1</x:v>
-      </x:c>
-      <x:c r="D50" s="59" t="n">
-        <x:v>111.6</x:v>
+        <x:v>O&amp;M / CAPEX</x:v>
+      </x:c>
+      <x:c r="D50" s="78" t="n">
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="E50" s="109" t="str">
-        <x:v>Tỷ VND/năm</x:v>
+        <x:v>% CAPEX/năm</x:v>
       </x:c>
       <x:c r="F50" s="109" t="str">
         <x:v>Bắt buộc</x:v>
       </x:c>
       <x:c r="G50" s="43" t="str">
-        <x:v>Giả định typical bằng 2% CAPEX chưa VAT.</x:v>
+        <x:v>Giả định typical 2% CAPEX/năm; thay bằng tỷ lệ O&amp;M thực tế.</x:v>
       </x:c>
       <x:c r="H50" s="103"/>
       <x:c r="I50" s="103"/>
@@ -2549,7 +2529,7 @@
         <x:v>EBITDA Y1</x:v>
       </x:c>
       <x:c r="D52" s="58" t="n">
-        <x:f>IF(OR(D47="",D50=""),"",D47-D50)</x:f>
+        <x:f>IF(OR(D47="",D21="",D50=""),"",D47-D21*D50)</x:f>
         <x:v>743.372496</x:v>
       </x:c>
       <x:c r="E52" s="109" t="str">
@@ -3338,7 +3318,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R580fe444a0624e66"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7940091c99940a9"/>
 </x:worksheet>
 </file>
 
@@ -3631,7 +3611,7 @@
       </x:c>
       <x:c r="G7" s="183" t="n">
         <x:f>IF(COUNTIF(C44:AF44,"&lt;0")*COUNTIF(C44:AF44,"&gt;0")=0,0,IRR(C44:AF44))</x:f>
-        <x:v>0.11643290283674468</x:v>
+        <x:v>0.11643290283674458</x:v>
       </x:c>
       <x:c r="H7" s="128"/>
       <x:c r="I7" s="128"/>
@@ -3684,7 +3664,7 @@
       </x:c>
       <x:c r="G8" s="183" t="n">
         <x:f>IF(COUNTIF(C49:AF49,"&lt;0")*COUNTIF(C49:AF49,"&gt;0")=0,0,IRR(C49:AF49))</x:f>
-        <x:v>0.11643290283674468</x:v>
+        <x:v>0.11643290283674458</x:v>
       </x:c>
       <x:c r="H8" s="128"/>
       <x:c r="I8" s="128"/>
@@ -3721,7 +3701,7 @@
       </x:c>
       <x:c r="C9" s="183" t="n">
         <x:f>IF(COUNTIF(C50:AF50,"&lt;0")*COUNTIF(C50:AF50,"&gt;0")=0,0,IRR(C50:AF50))</x:f>
-        <x:v>0.11538357743844008</x:v>
+        <x:v>0.11538357743844084</x:v>
       </x:c>
       <x:c r="D9" s="183" t="n">
         <x:f>IF(COUNTIF(C51:AF51,"&lt;0")*COUNTIF(C51:AF51,"&gt;0")=0,0,IRR(C51:AF51))</x:f>
@@ -3737,7 +3717,7 @@
       </x:c>
       <x:c r="G9" s="183" t="n">
         <x:f>IF(COUNTIF(C54:AF54,"&lt;0")*COUNTIF(C54:AF54,"&gt;0")=0,0,IRR(C54:AF54))</x:f>
-        <x:v>0.08698929456650045</x:v>
+        <x:v>0.08698929456650216</x:v>
       </x:c>
       <x:c r="H9" s="128"/>
       <x:c r="I9" s="128"/>
@@ -3774,11 +3754,11 @@
       </x:c>
       <x:c r="C10" s="183" t="n">
         <x:f>IF(COUNTIF(C55:AF55,"&lt;0")*COUNTIF(C55:AF55,"&gt;0")=0,0,IRR(C55:AF55))</x:f>
-        <x:v>0.10271529399494407</x:v>
+        <x:v>0.10271529399494406</x:v>
       </x:c>
       <x:c r="D10" s="183" t="n">
         <x:f>IF(COUNTIF(C56:AF56,"&lt;0")*COUNTIF(C56:AF56,"&gt;0")=0,0,IRR(C56:AF56))</x:f>
-        <x:v>0.10137843441184939</x:v>
+        <x:v>0.10137843441184922</x:v>
       </x:c>
       <x:c r="E10" s="183" t="n">
         <x:f>IF(COUNTIF(C57:AF57,"&lt;0")*COUNTIF(C57:AF57,"&gt;0")=0,0,IRR(C57:AF57))</x:f>
@@ -4032,23 +4012,23 @@
       </x:c>
       <x:c r="C16" s="183" t="n">
         <x:f>IF(COUNTIF(C70:AF70,"&lt;0")*COUNTIF(C70:AF70,"&gt;0")=0,0,IRR(C70:AF70))</x:f>
-        <x:v>0.06217715345123813</x:v>
+        <x:v>0.06217715345125385</x:v>
       </x:c>
       <x:c r="D16" s="183" t="n">
         <x:f>IF(COUNTIF(C71:AF71,"&lt;0")*COUNTIF(C71:AF71,"&gt;0")=0,0,IRR(C71:AF71))</x:f>
-        <x:v>0.07664308412616601</x:v>
+        <x:v>0.07664308412616276</x:v>
       </x:c>
       <x:c r="E16" s="183" t="n">
         <x:f>IF(COUNTIF(C72:AF72,"&lt;0")*COUNTIF(C72:AF72,"&gt;0")=0,0,IRR(C72:AF72))</x:f>
-        <x:v>0.09099776668955893</x:v>
+        <x:v>0.09099776668955771</x:v>
       </x:c>
       <x:c r="F16" s="183" t="n">
         <x:f>IF(COUNTIF(C73:AF73,"&lt;0")*COUNTIF(C73:AF73,"&gt;0")=0,0,IRR(C73:AF73))</x:f>
-        <x:v>0.10527314812925224</x:v>
+        <x:v>0.10527314812925223</x:v>
       </x:c>
       <x:c r="G16" s="183" t="n">
         <x:f>IF(COUNTIF(C74:AF74,"&lt;0")*COUNTIF(C74:AF74,"&gt;0")=0,0,IRR(C74:AF74))</x:f>
-        <x:v>0.11949321417132609</x:v>
+        <x:v>0.11949321417132476</x:v>
       </x:c>
       <x:c r="H16" s="128"/>
       <x:c r="I16" s="128"/>
@@ -4085,23 +4065,23 @@
       </x:c>
       <x:c r="C17" s="183" t="n">
         <x:f>IF(COUNTIF(C75:AF75,"&lt;0")*COUNTIF(C75:AF75,"&gt;0")=0,0,IRR(C75:AF75))</x:f>
-        <x:v>0.06217715345123813</x:v>
+        <x:v>0.06217715345125385</x:v>
       </x:c>
       <x:c r="D17" s="183" t="n">
         <x:f>IF(COUNTIF(C76:AF76,"&lt;0")*COUNTIF(C76:AF76,"&gt;0")=0,0,IRR(C76:AF76))</x:f>
-        <x:v>0.07664308412616601</x:v>
+        <x:v>0.07664308412616276</x:v>
       </x:c>
       <x:c r="E17" s="183" t="n">
         <x:f>IF(COUNTIF(C77:AF77,"&lt;0")*COUNTIF(C77:AF77,"&gt;0")=0,0,IRR(C77:AF77))</x:f>
-        <x:v>0.09099776668955893</x:v>
+        <x:v>0.09099776668955771</x:v>
       </x:c>
       <x:c r="F17" s="183" t="n">
         <x:f>IF(COUNTIF(C78:AF78,"&lt;0")*COUNTIF(C78:AF78,"&gt;0")=0,0,IRR(C78:AF78))</x:f>
-        <x:v>0.10527314812925224</x:v>
+        <x:v>0.10527314812925223</x:v>
       </x:c>
       <x:c r="G17" s="183" t="n">
         <x:f>IF(COUNTIF(C79:AF79,"&lt;0")*COUNTIF(C79:AF79,"&gt;0")=0,0,IRR(C79:AF79))</x:f>
-        <x:v>0.11949321417132609</x:v>
+        <x:v>0.11949321417132476</x:v>
       </x:c>
       <x:c r="H17" s="128"/>
       <x:c r="I17" s="128"/>
@@ -4138,23 +4118,23 @@
       </x:c>
       <x:c r="C18" s="183" t="n">
         <x:f>IF(COUNTIF(C80:AF80,"&lt;0")*COUNTIF(C80:AF80,"&gt;0")=0,0,IRR(C80:AF80))</x:f>
-        <x:v>0.0984223187458286</x:v>
+        <x:v>0.09842231874582841</x:v>
       </x:c>
       <x:c r="D18" s="183" t="n">
         <x:f>IF(COUNTIF(C81:AF81,"&lt;0")*COUNTIF(C81:AF81,"&gt;0")=0,0,IRR(C81:AF81))</x:f>
-        <x:v>0.09461115126438392</x:v>
+        <x:v>0.0946111512643832</x:v>
       </x:c>
       <x:c r="E18" s="183" t="n">
         <x:f>IF(COUNTIF(C82:AF82,"&lt;0")*COUNTIF(C82:AF82,"&gt;0")=0,0,IRR(C82:AF82))</x:f>
-        <x:v>0.09099776668955893</x:v>
+        <x:v>0.09099776668955771</x:v>
       </x:c>
       <x:c r="F18" s="183" t="n">
         <x:f>IF(COUNTIF(C83:AF83,"&lt;0")*COUNTIF(C83:AF83,"&gt;0")=0,0,IRR(C83:AF83))</x:f>
-        <x:v>0.08756382129001206</x:v>
+        <x:v>0.0875638212900106</x:v>
       </x:c>
       <x:c r="G18" s="183" t="n">
         <x:f>IF(COUNTIF(C84:AF84,"&lt;0")*COUNTIF(C84:AF84,"&gt;0")=0,0,IRR(C84:AF84))</x:f>
-        <x:v>0.0842933510839552</x:v>
+        <x:v>0.08429335108395536</x:v>
       </x:c>
       <x:c r="H18" s="128"/>
       <x:c r="I18" s="128"/>
@@ -4191,23 +4171,23 @@
       </x:c>
       <x:c r="C19" s="183" t="n">
         <x:f>IF(COUNTIF(C85:AF85,"&lt;0")*COUNTIF(C85:AF85,"&gt;0")=0,0,IRR(C85:AF85))</x:f>
-        <x:v>0.09560963889120139</x:v>
+        <x:v>0.09560963889120186</x:v>
       </x:c>
       <x:c r="D19" s="183" t="n">
         <x:f>IF(COUNTIF(C86:AF86,"&lt;0")*COUNTIF(C86:AF86,"&gt;0")=0,0,IRR(C86:AF86))</x:f>
-        <x:v>0.09330898418856182</x:v>
+        <x:v>0.09330898418856183</x:v>
       </x:c>
       <x:c r="E19" s="183" t="n">
         <x:f>IF(COUNTIF(C87:AF87,"&lt;0")*COUNTIF(C87:AF87,"&gt;0")=0,0,IRR(C87:AF87))</x:f>
-        <x:v>0.09099776668955893</x:v>
+        <x:v>0.09099776668955771</x:v>
       </x:c>
       <x:c r="F19" s="183" t="n">
         <x:f>IF(COUNTIF(C88:AF88,"&lt;0")*COUNTIF(C88:AF88,"&gt;0")=0,0,IRR(C88:AF88))</x:f>
-        <x:v>0.08867565224581594</x:v>
+        <x:v>0.08867565224581625</x:v>
       </x:c>
       <x:c r="G19" s="183" t="n">
         <x:f>IF(COUNTIF(C89:AF89,"&lt;0")*COUNTIF(C89:AF89,"&gt;0")=0,0,IRR(C89:AF89))</x:f>
-        <x:v>0.08634229225087042</x:v>
+        <x:v>0.08634229225087053</x:v>
       </x:c>
       <x:c r="H19" s="128"/>
       <x:c r="I19" s="128"/>
@@ -4244,23 +4224,23 @@
       </x:c>
       <x:c r="C20" s="183" t="n">
         <x:f>IF(COUNTIF(C90:AF90,"&lt;0")*COUNTIF(C90:AF90,"&gt;0")=0,0,IRR(C90:AF90))</x:f>
-        <x:v>0.09942615561012688</x:v>
+        <x:v>0.09942615561012694</x:v>
       </x:c>
       <x:c r="D20" s="183" t="n">
         <x:f>IF(COUNTIF(C91:AF91,"&lt;0")*COUNTIF(C91:AF91,"&gt;0")=0,0,IRR(C91:AF91))</x:f>
-        <x:v>0.0951487194097706</x:v>
+        <x:v>0.09514871940977168</x:v>
       </x:c>
       <x:c r="E20" s="183" t="n">
         <x:f>IF(COUNTIF(C92:AF92,"&lt;0")*COUNTIF(C92:AF92,"&gt;0")=0,0,IRR(C92:AF92))</x:f>
-        <x:v>0.09099776668955893</x:v>
+        <x:v>0.09099776668955771</x:v>
       </x:c>
       <x:c r="F20" s="183" t="n">
         <x:f>IF(COUNTIF(C93:AF93,"&lt;0")*COUNTIF(C93:AF93,"&gt;0")=0,0,IRR(C93:AF93))</x:f>
-        <x:v>0.08696841031670174</x:v>
+        <x:v>0.08696841031670186</x:v>
       </x:c>
       <x:c r="G20" s="183" t="n">
         <x:f>IF(COUNTIF(C94:AF94,"&lt;0")*COUNTIF(C94:AF94,"&gt;0")=0,0,IRR(C94:AF94))</x:f>
-        <x:v>0.08305590900880544</x:v>
+        <x:v>0.08305590900880559</x:v>
       </x:c>
       <x:c r="H20" s="128"/>
       <x:c r="I20" s="128"/>
@@ -4979,7 +4959,7 @@
       </x:c>
       <x:c r="K40" s="188" t="n">
         <x:f>'Project_CF'!K24+('Energy_Revenue'!K14*-0.09999999999999998)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>610.508635097143</x:v>
+        <x:v>610.5086350971429</x:v>
       </x:c>
       <x:c r="L40" s="188" t="n">
         <x:f>'Project_CF'!L24+('Energy_Revenue'!L14*-0.09999999999999998)*(1-'Dep_Tax'!L24)</x:f>
@@ -5107,7 +5087,7 @@
       </x:c>
       <x:c r="K41" s="188" t="n">
         <x:f>'Project_CF'!K24+('Energy_Revenue'!K14*-0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>650.6349245179846</x:v>
+        <x:v>650.6349245179845</x:v>
       </x:c>
       <x:c r="L41" s="188" t="n">
         <x:f>'Project_CF'!L24+('Energy_Revenue'!L14*-0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -5235,7 +5215,7 @@
       </x:c>
       <x:c r="K42" s="188" t="n">
         <x:f>'Project_CF'!K24+('Energy_Revenue'!K14*0)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L42" s="188" t="n">
         <x:f>'Project_CF'!L24+('Energy_Revenue'!L14*0)*(1-'Dep_Tax'!L24)</x:f>
@@ -5363,7 +5343,7 @@
       </x:c>
       <x:c r="K43" s="188" t="n">
         <x:f>'Project_CF'!K24+('Energy_Revenue'!K14*0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>730.8875033596677</x:v>
+        <x:v>730.8875033596676</x:v>
       </x:c>
       <x:c r="L43" s="188" t="n">
         <x:f>'Project_CF'!L24+('Energy_Revenue'!L14*0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -5491,7 +5471,7 @@
       </x:c>
       <x:c r="K44" s="188" t="n">
         <x:f>'Project_CF'!K24+('Energy_Revenue'!K14*0.10000000000000009)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>771.0137927805092</x:v>
+        <x:v>771.0137927805091</x:v>
       </x:c>
       <x:c r="L44" s="188" t="n">
         <x:f>'Project_CF'!L24+('Energy_Revenue'!L14*0.10000000000000009)*(1-'Dep_Tax'!L24)</x:f>
@@ -5619,7 +5599,7 @@
       </x:c>
       <x:c r="K45" s="188" t="n">
         <x:f>'Project_CF'!K24+('Energy_Revenue'!K14*-0.09999999999999998)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>610.508635097143</x:v>
+        <x:v>610.5086350971429</x:v>
       </x:c>
       <x:c r="L45" s="188" t="n">
         <x:f>'Project_CF'!L24+('Energy_Revenue'!L14*-0.09999999999999998)*(1-'Dep_Tax'!L24)</x:f>
@@ -5747,7 +5727,7 @@
       </x:c>
       <x:c r="K46" s="188" t="n">
         <x:f>'Project_CF'!K24+('Energy_Revenue'!K14*-0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>650.6349245179846</x:v>
+        <x:v>650.6349245179845</x:v>
       </x:c>
       <x:c r="L46" s="188" t="n">
         <x:f>'Project_CF'!L24+('Energy_Revenue'!L14*-0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -5875,7 +5855,7 @@
       </x:c>
       <x:c r="K47" s="188" t="n">
         <x:f>'Project_CF'!K24+('Energy_Revenue'!K14*0)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L47" s="188" t="n">
         <x:f>'Project_CF'!L24+('Energy_Revenue'!L14*0)*(1-'Dep_Tax'!L24)</x:f>
@@ -6003,7 +5983,7 @@
       </x:c>
       <x:c r="K48" s="188" t="n">
         <x:f>'Project_CF'!K24+('Energy_Revenue'!K14*0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>730.8875033596677</x:v>
+        <x:v>730.8875033596676</x:v>
       </x:c>
       <x:c r="L48" s="188" t="n">
         <x:f>'Project_CF'!L24+('Energy_Revenue'!L14*0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -6131,7 +6111,7 @@
       </x:c>
       <x:c r="K49" s="188" t="n">
         <x:f>'Project_CF'!K24+('Energy_Revenue'!K14*0.10000000000000009)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>771.0137927805092</x:v>
+        <x:v>771.0137927805091</x:v>
       </x:c>
       <x:c r="L49" s="188" t="n">
         <x:f>'Project_CF'!L24+('Energy_Revenue'!L14*0.10000000000000009)*(1-'Dep_Tax'!L24)</x:f>
@@ -6259,7 +6239,7 @@
       </x:c>
       <x:c r="K50" s="188" t="n">
         <x:f>'Project_CF'!K24-('CAPEX'!K15-'CAPEX'!K17)*-0.09999999999999998+'Dep_Tax'!K12*-0.09999999999999998*'Dep_Tax'!K24</x:f>
-        <x:v>689.2783289388261</x:v>
+        <x:v>689.278328938826</x:v>
       </x:c>
       <x:c r="L50" s="188" t="n">
         <x:f>'Project_CF'!L24-('CAPEX'!L15-'CAPEX'!L17)*-0.09999999999999998+'Dep_Tax'!L12*-0.09999999999999998*'Dep_Tax'!L24</x:f>
@@ -6387,7 +6367,7 @@
       </x:c>
       <x:c r="K51" s="188" t="n">
         <x:f>'Project_CF'!K24-('CAPEX'!K15-'CAPEX'!K17)*-0.050000000000000044+'Dep_Tax'!K12*-0.050000000000000044*'Dep_Tax'!K24</x:f>
-        <x:v>690.0197714388262</x:v>
+        <x:v>690.0197714388261</x:v>
       </x:c>
       <x:c r="L51" s="188" t="n">
         <x:f>'Project_CF'!L24-('CAPEX'!L15-'CAPEX'!L17)*-0.050000000000000044+'Dep_Tax'!L12*-0.050000000000000044*'Dep_Tax'!L24</x:f>
@@ -6515,7 +6495,7 @@
       </x:c>
       <x:c r="K52" s="188" t="n">
         <x:f>'Project_CF'!K24-('CAPEX'!K15-'CAPEX'!K17)*0+'Dep_Tax'!K12*0*'Dep_Tax'!K24</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L52" s="188" t="n">
         <x:f>'Project_CF'!L24-('CAPEX'!L15-'CAPEX'!L17)*0+'Dep_Tax'!L12*0*'Dep_Tax'!L24</x:f>
@@ -6643,7 +6623,7 @@
       </x:c>
       <x:c r="K53" s="188" t="n">
         <x:f>'Project_CF'!K24-('CAPEX'!K15-'CAPEX'!K17)*0.050000000000000044+'Dep_Tax'!K12*0.050000000000000044*'Dep_Tax'!K24</x:f>
-        <x:v>691.5026564388261</x:v>
+        <x:v>691.502656438826</x:v>
       </x:c>
       <x:c r="L53" s="188" t="n">
         <x:f>'Project_CF'!L24-('CAPEX'!L15-'CAPEX'!L17)*0.050000000000000044+'Dep_Tax'!L12*0.050000000000000044*'Dep_Tax'!L24</x:f>
@@ -6771,7 +6751,7 @@
       </x:c>
       <x:c r="K54" s="188" t="n">
         <x:f>'Project_CF'!K24-('CAPEX'!K15-'CAPEX'!K17)*0.10000000000000009+'Dep_Tax'!K12*0.10000000000000009*'Dep_Tax'!K24</x:f>
-        <x:v>692.2440989388261</x:v>
+        <x:v>692.244098938826</x:v>
       </x:c>
       <x:c r="L54" s="188" t="n">
         <x:f>'Project_CF'!L24-('CAPEX'!L15-'CAPEX'!L17)*0.10000000000000009+'Dep_Tax'!L12*0.10000000000000009*'Dep_Tax'!L24</x:f>
@@ -6879,7 +6859,7 @@
       </x:c>
       <x:c r="F55" s="188" t="n">
         <x:f>'Project_CF'!F24-('Energy_Revenue'!F19*-0.09999999999999998)*(1-'Dep_Tax'!F24)</x:f>
-        <x:v>749.8093510079999</x:v>
+        <x:v>749.809351008</x:v>
       </x:c>
       <x:c r="G55" s="188" t="n">
         <x:f>'Project_CF'!G24-('Energy_Revenue'!G19*-0.09999999999999998)*(1-'Dep_Tax'!G24)</x:f>
@@ -6899,7 +6879,7 @@
       </x:c>
       <x:c r="K55" s="188" t="n">
         <x:f>'Project_CF'!K24-('Energy_Revenue'!K19*-0.09999999999999998)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>703.4205563866266</x:v>
+        <x:v>703.4205563866265</x:v>
       </x:c>
       <x:c r="L55" s="188" t="n">
         <x:f>'Project_CF'!L24-('Energy_Revenue'!L19*-0.09999999999999998)*(1-'Dep_Tax'!L24)</x:f>
@@ -7027,7 +7007,7 @@
       </x:c>
       <x:c r="K56" s="188" t="n">
         <x:f>'Project_CF'!K24-('Energy_Revenue'!K19*-0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>697.0908851627264</x:v>
+        <x:v>697.0908851627263</x:v>
       </x:c>
       <x:c r="L56" s="188" t="n">
         <x:f>'Project_CF'!L24-('Energy_Revenue'!L19*-0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -7075,7 +7055,7 @@
       </x:c>
       <x:c r="W56" s="188" t="n">
         <x:f>'Project_CF'!W24-('Energy_Revenue'!W19*-0.050000000000000044)*(1-'Dep_Tax'!W24)</x:f>
-        <x:v>574.6907892195969</x:v>
+        <x:v>574.690789219597</x:v>
       </x:c>
       <x:c r="X56" s="188" t="n">
         <x:f>'Project_CF'!X24-('Energy_Revenue'!X19*-0.050000000000000044)*(1-'Dep_Tax'!X24)</x:f>
@@ -7155,7 +7135,7 @@
       </x:c>
       <x:c r="K57" s="188" t="n">
         <x:f>'Project_CF'!K24-('Energy_Revenue'!K19*0)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L57" s="188" t="n">
         <x:f>'Project_CF'!L24-('Energy_Revenue'!L19*0)*(1-'Dep_Tax'!L24)</x:f>
@@ -7283,7 +7263,7 @@
       </x:c>
       <x:c r="K58" s="188" t="n">
         <x:f>'Project_CF'!K24-('Energy_Revenue'!K19*0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>684.4315427149259</x:v>
+        <x:v>684.4315427149257</x:v>
       </x:c>
       <x:c r="L58" s="188" t="n">
         <x:f>'Project_CF'!L24-('Energy_Revenue'!L19*0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -7331,7 +7311,7 @@
       </x:c>
       <x:c r="W58" s="188" t="n">
         <x:f>'Project_CF'!W24-('Energy_Revenue'!W19*0.050000000000000044)*(1-'Dep_Tax'!W24)</x:f>
-        <x:v>559.4914668488472</x:v>
+        <x:v>559.491466848847</x:v>
       </x:c>
       <x:c r="X58" s="188" t="n">
         <x:f>'Project_CF'!X24-('Energy_Revenue'!X19*0.050000000000000044)*(1-'Dep_Tax'!X24)</x:f>
@@ -7411,7 +7391,7 @@
       </x:c>
       <x:c r="K59" s="188" t="n">
         <x:f>'Project_CF'!K24-('Energy_Revenue'!K19*0.10000000000000009)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>678.1018714910257</x:v>
+        <x:v>678.1018714910256</x:v>
       </x:c>
       <x:c r="L59" s="188" t="n">
         <x:f>'Project_CF'!L24-('Energy_Revenue'!L19*0.10000000000000009)*(1-'Dep_Tax'!L24)</x:f>
@@ -7539,7 +7519,7 @@
       </x:c>
       <x:c r="K60" s="188" t="n">
         <x:f>'Project_CF'!K24</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L60" s="188" t="n">
         <x:f>'Project_CF'!L24</x:f>
@@ -7667,7 +7647,7 @@
       </x:c>
       <x:c r="K61" s="188" t="n">
         <x:f>'Project_CF'!K24</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L61" s="188" t="n">
         <x:f>'Project_CF'!L24</x:f>
@@ -7795,7 +7775,7 @@
       </x:c>
       <x:c r="K62" s="188" t="n">
         <x:f>'Project_CF'!K24</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L62" s="188" t="n">
         <x:f>'Project_CF'!L24</x:f>
@@ -7923,7 +7903,7 @@
       </x:c>
       <x:c r="K63" s="188" t="n">
         <x:f>'Project_CF'!K24</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L63" s="188" t="n">
         <x:f>'Project_CF'!L24</x:f>
@@ -8051,7 +8031,7 @@
       </x:c>
       <x:c r="K64" s="188" t="n">
         <x:f>'Project_CF'!K24</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L64" s="188" t="n">
         <x:f>'Project_CF'!L24</x:f>
@@ -8349,7 +8329,7 @@
       </x:c>
       <x:c r="K70" s="188" t="n">
         <x:f>'Equity_CF'!K20+('Energy_Revenue'!K14*-0.09999999999999998)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>99.47363509714314</x:v>
+        <x:v>99.47363509714292</x:v>
       </x:c>
       <x:c r="L70" s="188" t="n">
         <x:f>'Equity_CF'!L20+('Energy_Revenue'!L14*-0.09999999999999998)*(1-'Dep_Tax'!L24)</x:f>
@@ -8477,7 +8457,7 @@
       </x:c>
       <x:c r="K71" s="188" t="n">
         <x:f>'Equity_CF'!K20+('Energy_Revenue'!K14*-0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>139.59992451798462</x:v>
+        <x:v>139.5999245179844</x:v>
       </x:c>
       <x:c r="L71" s="188" t="n">
         <x:f>'Equity_CF'!L20+('Energy_Revenue'!L14*-0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -8605,7 +8585,7 @@
       </x:c>
       <x:c r="K72" s="188" t="n">
         <x:f>'Equity_CF'!K20+('Energy_Revenue'!K14*0)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>179.7262139388262</x:v>
+        <x:v>179.72621393882596</x:v>
       </x:c>
       <x:c r="L72" s="188" t="n">
         <x:f>'Equity_CF'!L20+('Energy_Revenue'!L14*0)*(1-'Dep_Tax'!L24)</x:f>
@@ -8733,7 +8713,7 @@
       </x:c>
       <x:c r="K73" s="188" t="n">
         <x:f>'Equity_CF'!K20+('Energy_Revenue'!K14*0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>219.85250335966776</x:v>
+        <x:v>219.85250335966754</x:v>
       </x:c>
       <x:c r="L73" s="188" t="n">
         <x:f>'Equity_CF'!L20+('Energy_Revenue'!L14*0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -8861,7 +8841,7 @@
       </x:c>
       <x:c r="K74" s="188" t="n">
         <x:f>'Equity_CF'!K20+('Energy_Revenue'!K14*0.10000000000000009)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>259.9787927805093</x:v>
+        <x:v>259.9787927805091</x:v>
       </x:c>
       <x:c r="L74" s="188" t="n">
         <x:f>'Equity_CF'!L20+('Energy_Revenue'!L14*0.10000000000000009)*(1-'Dep_Tax'!L24)</x:f>
@@ -8989,7 +8969,7 @@
       </x:c>
       <x:c r="K75" s="188" t="n">
         <x:f>'Equity_CF'!K20+('Energy_Revenue'!K14*-0.09999999999999998)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>99.47363509714314</x:v>
+        <x:v>99.47363509714292</x:v>
       </x:c>
       <x:c r="L75" s="188" t="n">
         <x:f>'Equity_CF'!L20+('Energy_Revenue'!L14*-0.09999999999999998)*(1-'Dep_Tax'!L24)</x:f>
@@ -9117,7 +9097,7 @@
       </x:c>
       <x:c r="K76" s="188" t="n">
         <x:f>'Equity_CF'!K20+('Energy_Revenue'!K14*-0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>139.59992451798462</x:v>
+        <x:v>139.5999245179844</x:v>
       </x:c>
       <x:c r="L76" s="188" t="n">
         <x:f>'Equity_CF'!L20+('Energy_Revenue'!L14*-0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -9245,7 +9225,7 @@
       </x:c>
       <x:c r="K77" s="188" t="n">
         <x:f>'Equity_CF'!K20+('Energy_Revenue'!K14*0)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>179.7262139388262</x:v>
+        <x:v>179.72621393882596</x:v>
       </x:c>
       <x:c r="L77" s="188" t="n">
         <x:f>'Equity_CF'!L20+('Energy_Revenue'!L14*0)*(1-'Dep_Tax'!L24)</x:f>
@@ -9373,7 +9353,7 @@
       </x:c>
       <x:c r="K78" s="188" t="n">
         <x:f>'Equity_CF'!K20+('Energy_Revenue'!K14*0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>219.85250335966776</x:v>
+        <x:v>219.85250335966754</x:v>
       </x:c>
       <x:c r="L78" s="188" t="n">
         <x:f>'Equity_CF'!L20+('Energy_Revenue'!L14*0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -9501,7 +9481,7 @@
       </x:c>
       <x:c r="K79" s="188" t="n">
         <x:f>'Equity_CF'!K20+('Energy_Revenue'!K14*0.10000000000000009)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>259.9787927805093</x:v>
+        <x:v>259.9787927805091</x:v>
       </x:c>
       <x:c r="L79" s="188" t="n">
         <x:f>'Equity_CF'!L20+('Energy_Revenue'!L14*0.10000000000000009)*(1-'Dep_Tax'!L24)</x:f>
@@ -9629,7 +9609,7 @@
       </x:c>
       <x:c r="K80" s="188" t="n">
         <x:f>'Equity_CF'!K20-(('CAPEX'!K15-'CAPEX'!K17-'Debt'!K12)*-0.09999999999999998)</x:f>
-        <x:v>179.7262139388262</x:v>
+        <x:v>179.72621393882596</x:v>
       </x:c>
       <x:c r="L80" s="188" t="n">
         <x:f>'Equity_CF'!L20-(('CAPEX'!L15-'CAPEX'!L17-'Debt'!L12)*-0.09999999999999998)</x:f>
@@ -9757,7 +9737,7 @@
       </x:c>
       <x:c r="K81" s="189" t="n">
         <x:f>'Equity_CF'!K20-(('CAPEX'!K15-'CAPEX'!K17-'Debt'!K12)*-0.050000000000000044)</x:f>
-        <x:v>179.7262139388262</x:v>
+        <x:v>179.72621393882596</x:v>
       </x:c>
       <x:c r="L81" s="189" t="n">
         <x:f>'Equity_CF'!L20-(('CAPEX'!L15-'CAPEX'!L17-'Debt'!L12)*-0.050000000000000044)</x:f>
@@ -9885,7 +9865,7 @@
       </x:c>
       <x:c r="K82" s="189" t="n">
         <x:f>'Equity_CF'!K20-(('CAPEX'!K15-'CAPEX'!K17-'Debt'!K12)*0)</x:f>
-        <x:v>179.7262139388262</x:v>
+        <x:v>179.72621393882596</x:v>
       </x:c>
       <x:c r="L82" s="189" t="n">
         <x:f>'Equity_CF'!L20-(('CAPEX'!L15-'CAPEX'!L17-'Debt'!L12)*0)</x:f>
@@ -10013,7 +9993,7 @@
       </x:c>
       <x:c r="K83" s="189" t="n">
         <x:f>'Equity_CF'!K20-(('CAPEX'!K15-'CAPEX'!K17-'Debt'!K12)*0.050000000000000044)</x:f>
-        <x:v>179.7262139388262</x:v>
+        <x:v>179.72621393882596</x:v>
       </x:c>
       <x:c r="L83" s="189" t="n">
         <x:f>'Equity_CF'!L20-(('CAPEX'!L15-'CAPEX'!L17-'Debt'!L12)*0.050000000000000044)</x:f>
@@ -10141,7 +10121,7 @@
       </x:c>
       <x:c r="K84" s="189" t="n">
         <x:f>'Equity_CF'!K20-(('CAPEX'!K15-'CAPEX'!K17-'Debt'!K12)*0.10000000000000009)</x:f>
-        <x:v>179.7262139388262</x:v>
+        <x:v>179.72621393882596</x:v>
       </x:c>
       <x:c r="L84" s="189" t="n">
         <x:f>'Equity_CF'!L20-(('CAPEX'!L15-'CAPEX'!L17-'Debt'!L12)*0.10000000000000009)</x:f>
@@ -10269,7 +10249,7 @@
       </x:c>
       <x:c r="K85" s="189" t="n">
         <x:f>'Equity_CF'!K20-('Energy_Revenue'!K19*-0.09999999999999998)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>192.38555638662666</x:v>
+        <x:v>192.38555638662643</x:v>
       </x:c>
       <x:c r="L85" s="189" t="n">
         <x:f>'Equity_CF'!L20-('Energy_Revenue'!L19*-0.09999999999999998)*(1-'Dep_Tax'!L24)</x:f>
@@ -10397,7 +10377,7 @@
       </x:c>
       <x:c r="K86" s="189" t="n">
         <x:f>'Equity_CF'!K20-('Energy_Revenue'!K19*-0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>186.0558851627264</x:v>
+        <x:v>186.0558851627262</x:v>
       </x:c>
       <x:c r="L86" s="189" t="n">
         <x:f>'Equity_CF'!L20-('Energy_Revenue'!L19*-0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -10445,7 +10425,7 @@
       </x:c>
       <x:c r="W86" s="189" t="n">
         <x:f>'Equity_CF'!W20-('Energy_Revenue'!W19*-0.050000000000000044)*(1-'Dep_Tax'!W24)</x:f>
-        <x:v>574.6907892195969</x:v>
+        <x:v>574.690789219597</x:v>
       </x:c>
       <x:c r="X86" s="189" t="n">
         <x:f>'Equity_CF'!X20-('Energy_Revenue'!X19*-0.050000000000000044)*(1-'Dep_Tax'!X24)</x:f>
@@ -10525,7 +10505,7 @@
       </x:c>
       <x:c r="K87" s="189" t="n">
         <x:f>'Equity_CF'!K20-('Energy_Revenue'!K19*0)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>179.7262139388262</x:v>
+        <x:v>179.72621393882596</x:v>
       </x:c>
       <x:c r="L87" s="189" t="n">
         <x:f>'Equity_CF'!L20-('Energy_Revenue'!L19*0)*(1-'Dep_Tax'!L24)</x:f>
@@ -10653,7 +10633,7 @@
       </x:c>
       <x:c r="K88" s="189" t="n">
         <x:f>'Equity_CF'!K20-('Energy_Revenue'!K19*0.050000000000000044)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>173.39654271492597</x:v>
+        <x:v>173.39654271492572</x:v>
       </x:c>
       <x:c r="L88" s="189" t="n">
         <x:f>'Equity_CF'!L20-('Energy_Revenue'!L19*0.050000000000000044)*(1-'Dep_Tax'!L24)</x:f>
@@ -10701,7 +10681,7 @@
       </x:c>
       <x:c r="W88" s="189" t="n">
         <x:f>'Equity_CF'!W20-('Energy_Revenue'!W19*0.050000000000000044)*(1-'Dep_Tax'!W24)</x:f>
-        <x:v>559.4914668488472</x:v>
+        <x:v>559.491466848847</x:v>
       </x:c>
       <x:c r="X88" s="189" t="n">
         <x:f>'Equity_CF'!X20-('Energy_Revenue'!X19*0.050000000000000044)*(1-'Dep_Tax'!X24)</x:f>
@@ -10773,7 +10753,7 @@
       </x:c>
       <x:c r="I89" s="189" t="n">
         <x:f>'Equity_CF'!I20-('Energy_Revenue'!I19*0.10000000000000009)*(1-'Dep_Tax'!I24)</x:f>
-        <x:v>116.43530918532053</x:v>
+        <x:v>116.43530918532052</x:v>
       </x:c>
       <x:c r="J89" s="189" t="n">
         <x:f>'Equity_CF'!J20-('Energy_Revenue'!J19*0.10000000000000009)*(1-'Dep_Tax'!J24)</x:f>
@@ -10781,7 +10761,7 @@
       </x:c>
       <x:c r="K89" s="189" t="n">
         <x:f>'Equity_CF'!K20-('Energy_Revenue'!K19*0.10000000000000009)*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>167.06687149102572</x:v>
+        <x:v>167.0668714910255</x:v>
       </x:c>
       <x:c r="L89" s="189" t="n">
         <x:f>'Equity_CF'!L20-('Energy_Revenue'!L19*0.10000000000000009)*(1-'Dep_Tax'!L24)</x:f>
@@ -10793,7 +10773,7 @@
       </x:c>
       <x:c r="N89" s="189" t="n">
         <x:f>'Equity_CF'!N20-('Energy_Revenue'!N19*0.10000000000000009)*(1-'Dep_Tax'!N24)</x:f>
-        <x:v>242.11634933105023</x:v>
+        <x:v>242.1163493310502</x:v>
       </x:c>
       <x:c r="O89" s="189" t="n">
         <x:f>'Equity_CF'!O20-('Energy_Revenue'!O19*0.10000000000000009)*(1-'Dep_Tax'!O24)</x:f>
@@ -10909,7 +10889,7 @@
       </x:c>
       <x:c r="K90" s="189" t="n">
         <x:f>'Equity_CF'!K20-'Debt'!K16*-0.09999999999999998*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>198.27971393882618</x:v>
+        <x:v>198.27971393882595</x:v>
       </x:c>
       <x:c r="L90" s="189" t="n">
         <x:f>'Equity_CF'!L20-'Debt'!L16*-0.09999999999999998*(1-'Dep_Tax'!L24)</x:f>
@@ -11037,7 +11017,7 @@
       </x:c>
       <x:c r="K91" s="189" t="n">
         <x:f>'Equity_CF'!K20-'Debt'!K16*-0.050000000000000044*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>189.0029639388262</x:v>
+        <x:v>189.00296393882599</x:v>
       </x:c>
       <x:c r="L91" s="189" t="n">
         <x:f>'Equity_CF'!L20-'Debt'!L16*-0.050000000000000044*(1-'Dep_Tax'!L24)</x:f>
@@ -11165,7 +11145,7 @@
       </x:c>
       <x:c r="K92" s="189" t="n">
         <x:f>'Equity_CF'!K20-'Debt'!K16*0*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>179.7262139388262</x:v>
+        <x:v>179.72621393882596</x:v>
       </x:c>
       <x:c r="L92" s="189" t="n">
         <x:f>'Equity_CF'!L20-'Debt'!L16*0*(1-'Dep_Tax'!L24)</x:f>
@@ -11293,7 +11273,7 @@
       </x:c>
       <x:c r="K93" s="189" t="n">
         <x:f>'Equity_CF'!K20-'Debt'!K16*0.050000000000000044*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>170.44946393882617</x:v>
+        <x:v>170.44946393882594</x:v>
       </x:c>
       <x:c r="L93" s="189" t="n">
         <x:f>'Equity_CF'!L20-'Debt'!L16*0.050000000000000044*(1-'Dep_Tax'!L24)</x:f>
@@ -11421,7 +11401,7 @@
       </x:c>
       <x:c r="K94" s="189" t="n">
         <x:f>'Equity_CF'!K20-'Debt'!K16*0.10000000000000009*(1-'Dep_Tax'!K24)</x:f>
-        <x:v>161.17271393882618</x:v>
+        <x:v>161.17271393882595</x:v>
       </x:c>
       <x:c r="L94" s="189" t="n">
         <x:f>'Equity_CF'!L20-'Debt'!L16*0.10000000000000009*(1-'Dep_Tax'!L24)</x:f>
@@ -11739,7 +11719,7 @@
       </x:c>
       <x:c r="B12" s="198" t="n">
         <x:f>'Equity_CF'!C27</x:f>
-        <x:v>0.09099776668955893</x:v>
+        <x:v>0.09099776668955771</x:v>
       </x:c>
       <x:c r="C12" s="1" t="str">
         <x:v>%</x:v>
@@ -11788,7 +11768,7 @@
       </x:c>
       <x:c r="H13" s="199" t="n">
         <x:f>'Debt'!C33</x:f>
-        <x:v>1.2366039111450327</x:v>
+        <x:v>1.2366039111450324</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -18201,123 +18181,123 @@
         <x:v>Chi phí O&amp;M</x:v>
       </x:c>
       <x:c r="C19" s="153" t="n">
-        <x:f>IF(C$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(C$8-1),0)</x:f>
+        <x:f>IF(C$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(C$8-1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D19" s="153" t="n">
-        <x:f>IF(D$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(D$8-1),0)</x:f>
+        <x:f>IF(D$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(D$8-1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="153" t="n">
-        <x:f>IF(E$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(E$8-1),0)</x:f>
-        <x:v>111.6</x:v>
+        <x:f>IF(E$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(E$8-1),0)</x:f>
+        <x:v>111.60000000000001</x:v>
       </x:c>
       <x:c r="F19" s="153" t="n">
-        <x:f>IF(F$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(F$8-1),0)</x:f>
-        <x:v>114.948</x:v>
+        <x:f>IF(F$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(F$8-1),0)</x:f>
+        <x:v>114.94800000000001</x:v>
       </x:c>
       <x:c r="G19" s="153" t="n">
-        <x:f>IF(G$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(G$8-1),0)</x:f>
-        <x:v>118.39643999999998</x:v>
+        <x:f>IF(G$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(G$8-1),0)</x:f>
+        <x:v>118.39644</x:v>
       </x:c>
       <x:c r="H19" s="153" t="n">
-        <x:f>IF(H$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(H$8-1),0)</x:f>
-        <x:v>121.9483332</x:v>
+        <x:f>IF(H$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(H$8-1),0)</x:f>
+        <x:v>121.94833320000001</x:v>
       </x:c>
       <x:c r="I19" s="153" t="n">
-        <x:f>IF(I$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(I$8-1),0)</x:f>
-        <x:v>125.60678319600001</x:v>
+        <x:f>IF(I$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(I$8-1),0)</x:f>
+        <x:v>125.60678319600002</x:v>
       </x:c>
       <x:c r="J19" s="153" t="n">
-        <x:f>IF(J$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(J$8-1),0)</x:f>
-        <x:v>129.37498669188</x:v>
+        <x:f>IF(J$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(J$8-1),0)</x:f>
+        <x:v>129.37498669188003</x:v>
       </x:c>
       <x:c r="K19" s="153" t="n">
-        <x:f>IF(K$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(K$8-1),0)</x:f>
-        <x:v>133.2562362926364</x:v>
+        <x:f>IF(K$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(K$8-1),0)</x:f>
+        <x:v>133.25623629263643</x:v>
       </x:c>
       <x:c r="L19" s="153" t="n">
-        <x:f>IF(L$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(L$8-1),0)</x:f>
+        <x:f>IF(L$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(L$8-1),0)</x:f>
         <x:v>137.25392338141552</x:v>
       </x:c>
       <x:c r="M19" s="153" t="n">
-        <x:f>IF(M$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(M$8-1),0)</x:f>
+        <x:f>IF(M$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(M$8-1),0)</x:f>
         <x:v>141.371541082858</x:v>
       </x:c>
       <x:c r="N19" s="153" t="n">
-        <x:f>IF(N$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(N$8-1),0)</x:f>
-        <x:v>145.61268731534372</x:v>
+        <x:f>IF(N$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(N$8-1),0)</x:f>
+        <x:v>145.61268731534375</x:v>
       </x:c>
       <x:c r="O19" s="153" t="n">
-        <x:f>IF(O$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(O$8-1),0)</x:f>
-        <x:v>149.98106793480403</x:v>
+        <x:f>IF(O$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(O$8-1),0)</x:f>
+        <x:v>149.98106793480406</x:v>
       </x:c>
       <x:c r="P19" s="153" t="n">
-        <x:f>IF(P$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(P$8-1),0)</x:f>
-        <x:v>154.48049997284815</x:v>
+        <x:f>IF(P$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(P$8-1),0)</x:f>
+        <x:v>154.48049997284818</x:v>
       </x:c>
       <x:c r="Q19" s="153" t="n">
-        <x:f>IF(Q$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(Q$8-1),0)</x:f>
-        <x:v>159.1149149720336</x:v>
+        <x:f>IF(Q$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(Q$8-1),0)</x:f>
+        <x:v>159.11491497203363</x:v>
       </x:c>
       <x:c r="R19" s="153" t="n">
-        <x:f>IF(R$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(R$8-1),0)</x:f>
-        <x:v>163.8883624211946</x:v>
+        <x:f>IF(R$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(R$8-1),0)</x:f>
+        <x:v>163.88836242119464</x:v>
       </x:c>
       <x:c r="S19" s="153" t="n">
-        <x:f>IF(S$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(S$8-1),0)</x:f>
-        <x:v>168.80501329383048</x:v>
+        <x:f>IF(S$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(S$8-1),0)</x:f>
+        <x:v>168.8050132938305</x:v>
       </x:c>
       <x:c r="T19" s="153" t="n">
-        <x:f>IF(T$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(T$8-1),0)</x:f>
-        <x:v>173.86916369264537</x:v>
+        <x:f>IF(T$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(T$8-1),0)</x:f>
+        <x:v>173.8691636926454</x:v>
       </x:c>
       <x:c r="U19" s="153" t="n">
-        <x:f>IF(U$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(U$8-1),0)</x:f>
-        <x:v>179.08523860342476</x:v>
+        <x:f>IF(U$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(U$8-1),0)</x:f>
+        <x:v>179.08523860342478</x:v>
       </x:c>
       <x:c r="V19" s="153" t="n">
-        <x:f>IF(V$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(V$8-1),0)</x:f>
-        <x:v>184.45779576152748</x:v>
+        <x:f>IF(V$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(V$8-1),0)</x:f>
+        <x:v>184.4577957615275</x:v>
       </x:c>
       <x:c r="W19" s="153" t="n">
-        <x:f>IF(W$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(W$8-1),0)</x:f>
-        <x:v>189.99152963437334</x:v>
+        <x:f>IF(W$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(W$8-1),0)</x:f>
+        <x:v>189.99152963437336</x:v>
       </x:c>
       <x:c r="X19" s="153" t="n">
-        <x:f>IF(X$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(X$8-1),0)</x:f>
-        <x:v>195.69127552340453</x:v>
+        <x:f>IF(X$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(X$8-1),0)</x:f>
+        <x:v>195.69127552340456</x:v>
       </x:c>
       <x:c r="Y19" s="153" t="n">
-        <x:f>IF(Y$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(Y$8-1),0)</x:f>
+        <x:f>IF(Y$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(Y$8-1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z19" s="153" t="n">
-        <x:f>IF(Z$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(Z$8-1),0)</x:f>
+        <x:f>IF(Z$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(Z$8-1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AA19" s="153" t="n">
-        <x:f>IF(AA$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(AA$8-1),0)</x:f>
+        <x:f>IF(AA$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(AA$8-1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB19" s="153" t="n">
-        <x:f>IF(AB$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(AB$8-1),0)</x:f>
+        <x:f>IF(AB$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(AB$8-1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AC19" s="153" t="n">
-        <x:f>IF(AC$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(AC$8-1),0)</x:f>
+        <x:f>IF(AC$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(AC$8-1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD19" s="153" t="n">
-        <x:f>IF(AD$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(AD$8-1),0)</x:f>
+        <x:f>IF(AD$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(AD$8-1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AE19" s="153" t="n">
-        <x:f>IF(AE$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(AE$8-1),0)</x:f>
+        <x:f>IF(AE$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(AE$8-1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AF19" s="153" t="n">
-        <x:f>IF(AF$8&gt;0,'Input'!$D$50*(1+'Input'!$D$51)^(AF$8-1),0)</x:f>
+        <x:f>IF(AF$8&gt;0,'Input'!$D$21*'Input'!$D$50*(1+'Input'!$D$51)^(AF$8-1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -18362,7 +18342,7 @@
       </x:c>
       <x:c r="K20" s="150" t="n">
         <x:f>K16-K19</x:f>
-        <x:v>711.5077515145538</x:v>
+        <x:v>711.5077515145537</x:v>
       </x:c>
       <x:c r="L20" s="150" t="n">
         <x:f>L16-L19</x:f>
@@ -18490,7 +18470,7 @@
       </x:c>
       <x:c r="K21" s="163" t="n">
         <x:f>IF(K16=0,0,K20/K16)</x:f>
-        <x:v>0.8422562535619701</x:v>
+        <x:v>0.84225625356197</x:v>
       </x:c>
       <x:c r="L21" s="163" t="n">
         <x:f>IF(L16=0,0,L20/L16)</x:f>
@@ -22533,7 +22513,7 @@
       </x:c>
       <x:c r="K22" s="153" t="n">
         <x:f>'Project_CF'!K18</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L22" s="153" t="n">
         <x:f>'Project_CF'!L18</x:f>
@@ -22661,7 +22641,7 @@
       </x:c>
       <x:c r="K23" s="168" t="n">
         <x:f>IF(K17=0,0,K22/K17)</x:f>
-        <x:v>1.32634641693323</x:v>
+        <x:v>1.3263464169332297</x:v>
       </x:c>
       <x:c r="L23" s="168" t="n">
         <x:f>IF(L17=0,0,L22/L17)</x:f>
@@ -22787,7 +22767,7 @@
       </x:c>
       <x:c r="K24" s="170" t="n">
         <x:f>IF(K17&gt;0,K23,"")</x:f>
-        <x:v>1.32634641693323</x:v>
+        <x:v>1.3263464169332297</x:v>
       </x:c>
       <x:c r="L24" s="170" t="n">
         <x:f>IF(L17&gt;0,L23,"")</x:f>
@@ -22899,7 +22879,7 @@
       </x:c>
       <x:c r="K25" s="153" t="n">
         <x:f>IF(AND(K13&gt;=1,K13&lt;='Input'!$D$58),K22/(1+'Input'!$D$57)^K13,0)</x:f>
-        <x:v>354.4697246916065</x:v>
+        <x:v>354.46972469160636</x:v>
       </x:c>
       <x:c r="L25" s="153" t="n">
         <x:f>IF(AND(L13&gt;=1,L13&lt;='Input'!$D$58),L22/(1+'Input'!$D$57)^L13,0)</x:f>
@@ -23270,7 +23250,7 @@
       </x:c>
       <x:c r="C33" s="222" t="n">
         <x:f>IF('Input'!$D$63=0,0,SUM(C25:AF25)/'Input'!$D$63)</x:f>
-        <x:v>1.2366039111450327</x:v>
+        <x:v>1.2366039111450324</x:v>
       </x:c>
       <x:c r="D33" s="209"/>
       <x:c r="E33" s="209"/>
@@ -25953,7 +25933,7 @@
       </x:c>
       <x:c r="K15" s="153" t="n">
         <x:f>'Energy_Revenue'!K20</x:f>
-        <x:v>711.5077515145538</x:v>
+        <x:v>711.5077515145537</x:v>
       </x:c>
       <x:c r="L15" s="153" t="n">
         <x:f>'Energy_Revenue'!L20</x:f>
@@ -26081,7 +26061,7 @@
       </x:c>
       <x:c r="K16" s="150" t="n">
         <x:f>K15-K12</x:f>
-        <x:v>414.9307515145538</x:v>
+        <x:v>414.93075151455366</x:v>
       </x:c>
       <x:c r="L16" s="150" t="n">
         <x:f>L15-L12</x:f>
@@ -26337,7 +26317,7 @@
       </x:c>
       <x:c r="K18" s="153" t="n">
         <x:f>K16-K17</x:f>
-        <x:v>219.63075151455376</x:v>
+        <x:v>219.63075151455365</x:v>
       </x:c>
       <x:c r="L18" s="153" t="n">
         <x:f>L16-L17</x:f>
@@ -26977,7 +26957,7 @@
       </x:c>
       <x:c r="K23" s="153" t="n">
         <x:f>MAX(0,K18-K21)</x:f>
-        <x:v>219.63075151455376</x:v>
+        <x:v>219.63075151455365</x:v>
       </x:c>
       <x:c r="L23" s="153" t="n">
         <x:f>MAX(0,L18-L21)</x:f>
@@ -27233,7 +27213,7 @@
       </x:c>
       <x:c r="K25" s="150" t="n">
         <x:f>K23*K24</x:f>
-        <x:v>10.981537575727689</x:v>
+        <x:v>10.981537575727684</x:v>
       </x:c>
       <x:c r="L25" s="150" t="n">
         <x:f>L23*L24</x:f>
@@ -27361,7 +27341,7 @@
       </x:c>
       <x:c r="K26" s="150" t="n">
         <x:f>K18-K25</x:f>
-        <x:v>208.64921393882608</x:v>
+        <x:v>208.64921393882597</x:v>
       </x:c>
       <x:c r="L26" s="150" t="n">
         <x:f>L18-L25</x:f>
@@ -30106,31 +30086,31 @@
       </x:c>
       <x:c r="E12" s="153" t="n">
         <x:f>'Energy_Revenue'!E19</x:f>
-        <x:v>111.6</x:v>
+        <x:v>111.60000000000001</x:v>
       </x:c>
       <x:c r="F12" s="153" t="n">
         <x:f>'Energy_Revenue'!F19</x:f>
-        <x:v>114.948</x:v>
+        <x:v>114.94800000000001</x:v>
       </x:c>
       <x:c r="G12" s="153" t="n">
         <x:f>'Energy_Revenue'!G19</x:f>
-        <x:v>118.39643999999998</x:v>
+        <x:v>118.39644</x:v>
       </x:c>
       <x:c r="H12" s="153" t="n">
         <x:f>'Energy_Revenue'!H19</x:f>
-        <x:v>121.9483332</x:v>
+        <x:v>121.94833320000001</x:v>
       </x:c>
       <x:c r="I12" s="153" t="n">
         <x:f>'Energy_Revenue'!I19</x:f>
-        <x:v>125.60678319600001</x:v>
+        <x:v>125.60678319600002</x:v>
       </x:c>
       <x:c r="J12" s="153" t="n">
         <x:f>'Energy_Revenue'!J19</x:f>
-        <x:v>129.37498669188</x:v>
+        <x:v>129.37498669188003</x:v>
       </x:c>
       <x:c r="K12" s="153" t="n">
         <x:f>'Energy_Revenue'!K19</x:f>
-        <x:v>133.2562362926364</x:v>
+        <x:v>133.25623629263643</x:v>
       </x:c>
       <x:c r="L12" s="153" t="n">
         <x:f>'Energy_Revenue'!L19</x:f>
@@ -30142,47 +30122,47 @@
       </x:c>
       <x:c r="N12" s="153" t="n">
         <x:f>'Energy_Revenue'!N19</x:f>
-        <x:v>145.61268731534372</x:v>
+        <x:v>145.61268731534375</x:v>
       </x:c>
       <x:c r="O12" s="153" t="n">
         <x:f>'Energy_Revenue'!O19</x:f>
-        <x:v>149.98106793480403</x:v>
+        <x:v>149.98106793480406</x:v>
       </x:c>
       <x:c r="P12" s="153" t="n">
         <x:f>'Energy_Revenue'!P19</x:f>
-        <x:v>154.48049997284815</x:v>
+        <x:v>154.48049997284818</x:v>
       </x:c>
       <x:c r="Q12" s="153" t="n">
         <x:f>'Energy_Revenue'!Q19</x:f>
-        <x:v>159.1149149720336</x:v>
+        <x:v>159.11491497203363</x:v>
       </x:c>
       <x:c r="R12" s="153" t="n">
         <x:f>'Energy_Revenue'!R19</x:f>
-        <x:v>163.8883624211946</x:v>
+        <x:v>163.88836242119464</x:v>
       </x:c>
       <x:c r="S12" s="153" t="n">
         <x:f>'Energy_Revenue'!S19</x:f>
-        <x:v>168.80501329383048</x:v>
+        <x:v>168.8050132938305</x:v>
       </x:c>
       <x:c r="T12" s="153" t="n">
         <x:f>'Energy_Revenue'!T19</x:f>
-        <x:v>173.86916369264537</x:v>
+        <x:v>173.8691636926454</x:v>
       </x:c>
       <x:c r="U12" s="153" t="n">
         <x:f>'Energy_Revenue'!U19</x:f>
-        <x:v>179.08523860342476</x:v>
+        <x:v>179.08523860342478</x:v>
       </x:c>
       <x:c r="V12" s="153" t="n">
         <x:f>'Energy_Revenue'!V19</x:f>
-        <x:v>184.45779576152748</x:v>
+        <x:v>184.4577957615275</x:v>
       </x:c>
       <x:c r="W12" s="153" t="n">
         <x:f>'Energy_Revenue'!W19</x:f>
-        <x:v>189.99152963437334</x:v>
+        <x:v>189.99152963437336</x:v>
       </x:c>
       <x:c r="X12" s="153" t="n">
         <x:f>'Energy_Revenue'!X19</x:f>
-        <x:v>195.69127552340453</x:v>
+        <x:v>195.69127552340456</x:v>
       </x:c>
       <x:c r="Y12" s="153" t="n">
         <x:f>'Energy_Revenue'!Y19</x:f>
@@ -30258,7 +30238,7 @@
       </x:c>
       <x:c r="K13" s="150" t="n">
         <x:f>K11-K12</x:f>
-        <x:v>711.5077515145538</x:v>
+        <x:v>711.5077515145537</x:v>
       </x:c>
       <x:c r="L13" s="150" t="n">
         <x:f>L11-L12</x:f>
@@ -30514,7 +30494,7 @@
       </x:c>
       <x:c r="K15" s="150" t="n">
         <x:f>K13-K14</x:f>
-        <x:v>414.9307515145538</x:v>
+        <x:v>414.93075151455366</x:v>
       </x:c>
       <x:c r="L15" s="150" t="n">
         <x:f>L13-L14</x:f>
@@ -30770,7 +30750,7 @@
       </x:c>
       <x:c r="K17" s="150" t="n">
         <x:f>K15-K16</x:f>
-        <x:v>219.63075151455376</x:v>
+        <x:v>219.63075151455365</x:v>
       </x:c>
       <x:c r="L17" s="150" t="n">
         <x:f>L15-L16</x:f>
@@ -31026,7 +31006,7 @@
       </x:c>
       <x:c r="K19" s="153" t="n">
         <x:f>'Dep_Tax'!K23</x:f>
-        <x:v>219.63075151455376</x:v>
+        <x:v>219.63075151455365</x:v>
       </x:c>
       <x:c r="L19" s="153" t="n">
         <x:f>'Dep_Tax'!L23</x:f>
@@ -31154,7 +31134,7 @@
       </x:c>
       <x:c r="K20" s="153" t="n">
         <x:f>'Dep_Tax'!K25</x:f>
-        <x:v>10.981537575727689</x:v>
+        <x:v>10.981537575727684</x:v>
       </x:c>
       <x:c r="L20" s="153" t="n">
         <x:f>'Dep_Tax'!L25</x:f>
@@ -31282,7 +31262,7 @@
       </x:c>
       <x:c r="K21" s="150" t="n">
         <x:f>K17-K20</x:f>
-        <x:v>208.64921393882608</x:v>
+        <x:v>208.64921393882597</x:v>
       </x:c>
       <x:c r="L21" s="150" t="n">
         <x:f>L17-L20</x:f>
@@ -34352,31 +34332,31 @@
       </x:c>
       <x:c r="E13" s="153" t="n">
         <x:f>'Energy_Revenue'!E19</x:f>
-        <x:v>111.6</x:v>
+        <x:v>111.60000000000001</x:v>
       </x:c>
       <x:c r="F13" s="153" t="n">
         <x:f>'Energy_Revenue'!F19</x:f>
-        <x:v>114.948</x:v>
+        <x:v>114.94800000000001</x:v>
       </x:c>
       <x:c r="G13" s="153" t="n">
         <x:f>'Energy_Revenue'!G19</x:f>
-        <x:v>118.39643999999998</x:v>
+        <x:v>118.39644</x:v>
       </x:c>
       <x:c r="H13" s="153" t="n">
         <x:f>'Energy_Revenue'!H19</x:f>
-        <x:v>121.9483332</x:v>
+        <x:v>121.94833320000001</x:v>
       </x:c>
       <x:c r="I13" s="153" t="n">
         <x:f>'Energy_Revenue'!I19</x:f>
-        <x:v>125.60678319600001</x:v>
+        <x:v>125.60678319600002</x:v>
       </x:c>
       <x:c r="J13" s="153" t="n">
         <x:f>'Energy_Revenue'!J19</x:f>
-        <x:v>129.37498669188</x:v>
+        <x:v>129.37498669188003</x:v>
       </x:c>
       <x:c r="K13" s="153" t="n">
         <x:f>'Energy_Revenue'!K19</x:f>
-        <x:v>133.2562362926364</x:v>
+        <x:v>133.25623629263643</x:v>
       </x:c>
       <x:c r="L13" s="153" t="n">
         <x:f>'Energy_Revenue'!L19</x:f>
@@ -34388,47 +34368,47 @@
       </x:c>
       <x:c r="N13" s="153" t="n">
         <x:f>'Energy_Revenue'!N19</x:f>
-        <x:v>145.61268731534372</x:v>
+        <x:v>145.61268731534375</x:v>
       </x:c>
       <x:c r="O13" s="153" t="n">
         <x:f>'Energy_Revenue'!O19</x:f>
-        <x:v>149.98106793480403</x:v>
+        <x:v>149.98106793480406</x:v>
       </x:c>
       <x:c r="P13" s="153" t="n">
         <x:f>'Energy_Revenue'!P19</x:f>
-        <x:v>154.48049997284815</x:v>
+        <x:v>154.48049997284818</x:v>
       </x:c>
       <x:c r="Q13" s="153" t="n">
         <x:f>'Energy_Revenue'!Q19</x:f>
-        <x:v>159.1149149720336</x:v>
+        <x:v>159.11491497203363</x:v>
       </x:c>
       <x:c r="R13" s="153" t="n">
         <x:f>'Energy_Revenue'!R19</x:f>
-        <x:v>163.8883624211946</x:v>
+        <x:v>163.88836242119464</x:v>
       </x:c>
       <x:c r="S13" s="153" t="n">
         <x:f>'Energy_Revenue'!S19</x:f>
-        <x:v>168.80501329383048</x:v>
+        <x:v>168.8050132938305</x:v>
       </x:c>
       <x:c r="T13" s="153" t="n">
         <x:f>'Energy_Revenue'!T19</x:f>
-        <x:v>173.86916369264537</x:v>
+        <x:v>173.8691636926454</x:v>
       </x:c>
       <x:c r="U13" s="153" t="n">
         <x:f>'Energy_Revenue'!U19</x:f>
-        <x:v>179.08523860342476</x:v>
+        <x:v>179.08523860342478</x:v>
       </x:c>
       <x:c r="V13" s="153" t="n">
         <x:f>'Energy_Revenue'!V19</x:f>
-        <x:v>184.45779576152748</x:v>
+        <x:v>184.4577957615275</x:v>
       </x:c>
       <x:c r="W13" s="153" t="n">
         <x:f>'Energy_Revenue'!W19</x:f>
-        <x:v>189.99152963437334</x:v>
+        <x:v>189.99152963437336</x:v>
       </x:c>
       <x:c r="X13" s="153" t="n">
         <x:f>'Energy_Revenue'!X19</x:f>
-        <x:v>195.69127552340453</x:v>
+        <x:v>195.69127552340456</x:v>
       </x:c>
       <x:c r="Y13" s="153" t="n">
         <x:f>'Energy_Revenue'!Y19</x:f>
@@ -34504,7 +34484,7 @@
       </x:c>
       <x:c r="K14" s="150" t="n">
         <x:f>K12-K13</x:f>
-        <x:v>711.5077515145538</x:v>
+        <x:v>711.5077515145537</x:v>
       </x:c>
       <x:c r="L14" s="150" t="n">
         <x:f>L12-L13</x:f>
@@ -34760,7 +34740,7 @@
       </x:c>
       <x:c r="K16" s="153" t="n">
         <x:f>K14-K15</x:f>
-        <x:v>414.9307515145538</x:v>
+        <x:v>414.93075151455366</x:v>
       </x:c>
       <x:c r="L16" s="153" t="n">
         <x:f>L14-L15</x:f>
@@ -34888,7 +34868,7 @@
       </x:c>
       <x:c r="K17" s="153" t="n">
         <x:f>MAX(0,K16)*'Dep_Tax'!K24</x:f>
-        <x:v>20.74653757572769</x:v>
+        <x:v>20.746537575727686</x:v>
       </x:c>
       <x:c r="L17" s="153" t="n">
         <x:f>MAX(0,L16)*'Dep_Tax'!L24</x:f>
@@ -35016,7 +34996,7 @@
       </x:c>
       <x:c r="K18" s="150" t="n">
         <x:f>K14-K17</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L18" s="150" t="n">
         <x:f>L14-L17</x:f>
@@ -35598,7 +35578,7 @@
       </x:c>
       <x:c r="K24" s="150" t="n">
         <x:f>K18-K21+K22+K23</x:f>
-        <x:v>690.7612139388261</x:v>
+        <x:v>690.761213938826</x:v>
       </x:c>
       <x:c r="L24" s="150" t="n">
         <x:f>L18-L21+L22+L23</x:f>
@@ -35854,7 +35834,7 @@
       </x:c>
       <x:c r="K26" s="150" t="n">
         <x:f>K24*K25</x:f>
-        <x:v>322.24520426509673</x:v>
+        <x:v>322.2452042650967</x:v>
       </x:c>
       <x:c r="L26" s="150" t="n">
         <x:f>L24*L25</x:f>
@@ -35982,15 +35962,15 @@
       </x:c>
       <x:c r="K27" s="150" t="n">
         <x:f>J27+K24</x:f>
-        <x:v>-549.182949731472</x:v>
+        <x:v>-549.1829497314721</x:v>
       </x:c>
       <x:c r="L27" s="150" t="n">
         <x:f>K27+L24</x:f>
-        <x:v>136.17540989617999</x:v>
+        <x:v>136.17540989617987</x:v>
       </x:c>
       <x:c r="M27" s="150" t="n">
         <x:f>L27+M24</x:f>
-        <x:v>816.0201912337816</x:v>
+        <x:v>816.0201912337815</x:v>
       </x:c>
       <x:c r="N27" s="150" t="n">
         <x:f>M27+N24</x:f>
@@ -36205,15 +36185,15 @@
       </x:c>
       <x:c r="E29" s="153" t="n">
         <x:f>(E21-E22+E13-E23)*E25</x:f>
-        <x:v>-184.46280991735537</x:v>
+        <x:v>-184.46280991735534</x:v>
       </x:c>
       <x:c r="F29" s="153" t="n">
         <x:f>(F21-F22+F13-F23)*F25</x:f>
-        <x:v>86.36213373403453</x:v>
+        <x:v>86.36213373403454</x:v>
       </x:c>
       <x:c r="G29" s="153" t="n">
         <x:f>(G21-G22+G13-G23)*G25</x:f>
-        <x:v>80.86636158732324</x:v>
+        <x:v>80.86636158732325</x:v>
       </x:c>
       <x:c r="H29" s="153" t="n">
         <x:f>(H21-H22+H13-H23)*H25</x:f>
@@ -36225,11 +36205,11 @@
       </x:c>
       <x:c r="J29" s="153" t="n">
         <x:f>(J21-J22+J13-J23)*J25</x:f>
-        <x:v>66.38982471692783</x:v>
+        <x:v>66.38982471692785</x:v>
       </x:c>
       <x:c r="K29" s="153" t="n">
         <x:f>(K21-K22+K13-K23)*K25</x:f>
-        <x:v>62.165017689486966</x:v>
+        <x:v>62.16501768948698</x:v>
       </x:c>
       <x:c r="L29" s="153" t="n">
         <x:f>(L21-L22+L13-L23)*L25</x:f>
@@ -36241,47 +36221,47 @@
       </x:c>
       <x:c r="N29" s="153" t="n">
         <x:f>(N21-N22+N13-N23)*N25</x:f>
-        <x:v>51.03635859111947</x:v>
+        <x:v>51.03635859111949</x:v>
       </x:c>
       <x:c r="O29" s="153" t="n">
         <x:f>(O21-O22+O13-O23)*O25</x:f>
-        <x:v>47.78859031713914</x:v>
+        <x:v>47.788590317139146</x:v>
       </x:c>
       <x:c r="P29" s="153" t="n">
         <x:f>(P21-P22+P13-P23)*P25</x:f>
-        <x:v>44.747498206048455</x:v>
+        <x:v>44.74749820604847</x:v>
       </x:c>
       <x:c r="Q29" s="153" t="n">
         <x:f>(Q21-Q22+Q13-Q23)*Q25</x:f>
-        <x:v>41.899930138390836</x:v>
+        <x:v>41.89993013839084</x:v>
       </x:c>
       <x:c r="R29" s="153" t="n">
         <x:f>(R21-R22+R13-R23)*R25</x:f>
-        <x:v>39.233570947765955</x:v>
+        <x:v>39.23357094776596</x:v>
       </x:c>
       <x:c r="S29" s="153" t="n">
         <x:f>(S21-S22+S13-S23)*S25</x:f>
-        <x:v>36.73688916018086</x:v>
+        <x:v>36.736889160180866</x:v>
       </x:c>
       <x:c r="T29" s="153" t="n">
         <x:f>(T21-T22+T13-T23)*T25</x:f>
-        <x:v>34.39908712271479</x:v>
+        <x:v>34.399087122714796</x:v>
       </x:c>
       <x:c r="U29" s="153" t="n">
         <x:f>(U21-U22+U13-U23)*U25</x:f>
-        <x:v>32.21005430581476</x:v>
+        <x:v>32.210054305814765</x:v>
       </x:c>
       <x:c r="V29" s="153" t="n">
         <x:f>(V21-V22+V13-V23)*V25</x:f>
-        <x:v>30.16032357726291</x:v>
+        <x:v>30.160323577262915</x:v>
       </x:c>
       <x:c r="W29" s="153" t="n">
         <x:f>(W21-W22+W13-W23)*W25</x:f>
-        <x:v>28.241030258709813</x:v>
+        <x:v>28.24103025870982</x:v>
       </x:c>
       <x:c r="X29" s="153" t="n">
         <x:f>(X21-X22+X13-X23)*X25</x:f>
-        <x:v>26.443873787701005</x:v>
+        <x:v>26.44387378770101</x:v>
       </x:c>
       <x:c r="Y29" s="153" t="n">
         <x:f>(Y21-Y22+Y13-Y23)*Y25</x:f>
@@ -38998,7 +38978,7 @@
       </x:c>
       <x:c r="K11" s="153" t="n">
         <x:f>'Energy_Revenue'!K20</x:f>
-        <x:v>711.5077515145538</x:v>
+        <x:v>711.5077515145537</x:v>
       </x:c>
       <x:c r="L11" s="153" t="n">
         <x:f>'Energy_Revenue'!L20</x:f>
@@ -39894,7 +39874,7 @@
       </x:c>
       <x:c r="K18" s="153" t="n">
         <x:f>'Dep_Tax'!K25</x:f>
-        <x:v>10.981537575727689</x:v>
+        <x:v>10.981537575727684</x:v>
       </x:c>
       <x:c r="L18" s="153" t="n">
         <x:f>'Dep_Tax'!L25</x:f>
@@ -40150,7 +40130,7 @@
       </x:c>
       <x:c r="K20" s="150" t="n">
         <x:f>K11-K12+K13+K14-K15-K16-K17-K18+K19</x:f>
-        <x:v>179.7262139388262</x:v>
+        <x:v>179.72621393882596</x:v>
       </x:c>
       <x:c r="L20" s="150" t="n">
         <x:f>L11-L12+L13+L14-L15-L16-L17-L18+L19</x:f>
@@ -40406,7 +40386,7 @@
       </x:c>
       <x:c r="K22" s="150" t="n">
         <x:f>K20*K21</x:f>
-        <x:v>72.58840343812379</x:v>
+        <x:v>72.5884034381237</x:v>
       </x:c>
       <x:c r="L22" s="150" t="n">
         <x:f>L20*L21</x:f>
@@ -40534,39 +40514,39 @@
       </x:c>
       <x:c r="K23" s="150" t="n">
         <x:f>J23+K20</x:f>
-        <x:v>-1328.7554497314732</x:v>
+        <x:v>-1328.7554497314734</x:v>
       </x:c>
       <x:c r="L23" s="150" t="n">
         <x:f>K23+L20</x:f>
-        <x:v>-1123.509590103821</x:v>
+        <x:v>-1123.5095901038212</x:v>
       </x:c>
       <x:c r="M23" s="150" t="n">
         <x:f>L23+M20</x:f>
-        <x:v>-892.8548087662194</x:v>
+        <x:v>-892.8548087662197</x:v>
       </x:c>
       <x:c r="N23" s="150" t="n">
         <x:f>M23+N20</x:f>
-        <x:v>-636.9052541402116</x:v>
+        <x:v>-636.9052541402118</x:v>
       </x:c>
       <x:c r="O23" s="150" t="n">
         <x:f>N23+O20</x:f>
-        <x:v>-355.77860161784236</x:v>
+        <x:v>-355.7786016178426</x:v>
       </x:c>
       <x:c r="P23" s="150" t="n">
         <x:f>O23+P20</x:f>
-        <x:v>-49.59615916573591</x:v>
+        <x:v>-49.59615916573614</x:v>
       </x:c>
       <x:c r="Q23" s="150" t="n">
         <x:f>P23+Q20</x:f>
-        <x:v>607.0170239022917</x:v>
+        <x:v>607.0170239022915</x:v>
       </x:c>
       <x:c r="R23" s="150" t="n">
         <x:f>Q23+R20</x:f>
-        <x:v>1238.8824122055207</x:v>
+        <x:v>1238.8824122055205</x:v>
       </x:c>
       <x:c r="S23" s="150" t="n">
         <x:f>R23+S20</x:f>
-        <x:v>1864.8234002944127</x:v>
+        <x:v>1864.8234002944125</x:v>
       </x:c>
       <x:c r="T23" s="150" t="n">
         <x:f>S23+T20</x:f>
@@ -40814,7 +40794,7 @@
       </x:c>
       <x:c r="C27" s="223" t="n">
         <x:f>IF(COUNTIF(C20:AF20,"&lt;0")*COUNTIF(C20:AF20,"&gt;0")=0,0,IRR(C20:AF20))</x:f>
-        <x:v>0.09099776668955893</x:v>
+        <x:v>0.09099776668955771</x:v>
       </x:c>
       <x:c r="D27" s="209"/>
       <x:c r="E27" s="209"/>

</xml_diff>

<commit_message>
Hiển thị O&M năm đầu theo tỷ lệ CAPEX
</commit_message>
<xml_diff>
--- a/PTKTTC_Ver1.xlsx
+++ b/PTKTTC_Ver1.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" r:id="Rc310633ffde44cec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R061370693bf6492e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX" sheetId="3" r:id="Reb06c5ec79324dd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy_Revenue" sheetId="4" r:id="R0cc2f33818df45df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" r:id="Rea1521bda04f41ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dep_Tax" sheetId="6" r:id="R76dfcb523ed9434e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income_Statement" sheetId="7" r:id="Rda7ac03acc1d4187"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_CF" sheetId="8" r:id="R9abbdf0a67804dec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity_CF" sheetId="9" r:id="R1e06b0648fc44981"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="10" r:id="R22615fcf2ae643c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" r:id="R1364ba9c146b4cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R2e339bf3be6444c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX" sheetId="3" r:id="R8121608d71d641e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy_Revenue" sheetId="4" r:id="R49a17dd412834e2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" r:id="R4225193d746c436c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dep_Tax" sheetId="6" r:id="R8be0283316b54ef9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income_Statement" sheetId="7" r:id="R08c8dca8eca34ac6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_CF" sheetId="8" r:id="R91af78cc0e8c4fe7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity_CF" sheetId="9" r:id="Ree3f3110fdc34bb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="10" r:id="R9c52ff7a5cbe403a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -340,7 +340,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="225">
+  <x:cellXfs count="226">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -912,6 +912,9 @@
     <x:xf numFmtId="201" fontId="21" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="206" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1707,14 +1710,14 @@
       <x:c r="G19" s="112"/>
       <x:c r="H19" s="103"/>
       <x:c r="I19" s="85" t="str">
-        <x:v>Chi phí O&amp;M năm đầu</x:v>
-      </x:c>
-      <x:c r="J19" s="93" t="n">
-        <x:f>IF(OR(D21="",D50=""),"",D21*D50)</x:f>
-        <x:v>111.60000000000001</x:v>
+        <x:v>Tỷ lệ O&amp;M năm đầu</x:v>
+      </x:c>
+      <x:c r="J19" s="225" t="n">
+        <x:f>'Input'!$D$50</x:f>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="K19" s="85" t="str">
-        <x:v>Tỷ VND</x:v>
+        <x:v>% CAPEX/năm</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="22" hidden="0" customHeight="1">
@@ -2469,10 +2472,10 @@
         <x:v>OPE-01</x:v>
       </x:c>
       <x:c r="B50" s="47" t="str">
-        <x:v>Tỷ lệ chi phí O&amp;M năm đầu trên CAPEX</x:v>
+        <x:v>Tỷ lệ O&amp;M năm đầu trên CAPEX</x:v>
       </x:c>
       <x:c r="C50" s="109" t="str">
-        <x:v>O&amp;M / CAPEX</x:v>
+        <x:v>O&amp;M rate Y1</x:v>
       </x:c>
       <x:c r="D50" s="78" t="n">
         <x:v>0.02</x:v>
@@ -3318,7 +3321,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7940091c99940a9"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb5b49259a96436c"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Bổ sung danh mục từ viết tắt song ngữ
</commit_message>
<xml_diff>
--- a/PTKTTC_Ver1.xlsx
+++ b/PTKTTC_Ver1.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" r:id="Ra507fbc988174fa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R66431c235f9f4596"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX" sheetId="3" r:id="R74e448285e444d63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy_Revenue" sheetId="4" r:id="R98989db918524973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" r:id="R107842c29c7247fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dep_Tax" sheetId="6" r:id="R22f0a93e25604e45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income_Statement" sheetId="7" r:id="R91e18e0931154cfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_CF" sheetId="8" r:id="Rfd4eb3643c424cef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity_CF" sheetId="9" r:id="R61ac6b2a98614c4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="10" r:id="Rfd760c7533584d44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Abbreviations" sheetId="11" r:id="Rf6a10f758d27497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" r:id="R91744dfc01c04149"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R0a1b3b2efaca48b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX" sheetId="3" r:id="R56f31c6acd2c43b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy_Revenue" sheetId="4" r:id="R3ce6434f4ca041b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" r:id="R8f683f6169d04077"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dep_Tax" sheetId="6" r:id="R7eda5ff112e74ae1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income_Statement" sheetId="7" r:id="R1142550595cb4c77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_CF" sheetId="8" r:id="R02028e0e70b14c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity_CF" sheetId="9" r:id="R79aeab4d2281492e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="10" r:id="Rceb7184cad9e440f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -104,7 +105,7 @@
     <x:numFmt numFmtId="214" formatCode="0.00%;[Red](0.00%);-"/>
     <x:numFmt numFmtId="215" formatCode="0.0000x"/>
   </x:numFmts>
-  <x:fonts count="26">
+  <x:fonts count="30">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -252,8 +253,31 @@
       <x:color rgb="FF0000FF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -330,8 +354,23 @@
         <x:fgColor rgb="FFFFF2E8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="10">
+  <x:borders count="12">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -408,11 +447,39 @@
         <x:color rgb="FFD9B3AE"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="281">
+  <x:cellXfs count="301">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1116,6 +1183,48 @@
     <x:xf numFmtId="210" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -3664,7 +3773,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e885c07f680458c"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re52c99a2a78440f0"/>
 </x:worksheet>
 </file>
 
@@ -11843,6 +11952,656 @@
     <x:mergeCell ref="A14:G14"/>
     <x:mergeCell ref="A23:G25"/>
     <x:mergeCell ref="A28:AF28"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="7" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="40" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="284" t="str">
+        <x:v>DANH MỤC TỪ VIẾT TẮT / LIST OF ABBREVIATIONS</x:v>
+      </x:c>
+      <x:c r="B1" s="284"/>
+      <x:c r="C1" s="284"/>
+      <x:c r="D1" s="284"/>
+      <x:c r="E1" s="284"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="288" t="str">
+        <x:v>Mô hình phân tích kinh tế – tài chính dự án năng lượng tái tạo</x:v>
+      </x:c>
+      <x:c r="B2" s="288"/>
+      <x:c r="C2" s="288"/>
+      <x:c r="D2" s="288"/>
+      <x:c r="E2" s="288"/>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="294" t="str">
+        <x:v>STT</x:v>
+      </x:c>
+      <x:c r="B4" s="294" t="str">
+        <x:v>Từ viết tắt</x:v>
+      </x:c>
+      <x:c r="C4" s="294" t="str">
+        <x:v>Tên đầy đủ tiếng Anh</x:v>
+      </x:c>
+      <x:c r="D4" s="294" t="str">
+        <x:v>Tên tiếng Việt</x:v>
+      </x:c>
+      <x:c r="E4" s="294" t="str">
+        <x:v>Giải thích / Cách sử dụng trong mô hình</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="299" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="300" t="str">
+        <x:v>AEP</x:v>
+      </x:c>
+      <x:c r="C5" s="298" t="str">
+        <x:v>Annual Energy Production</x:v>
+      </x:c>
+      <x:c r="D5" s="298" t="str">
+        <x:v>Sản lượng điện năng hằng năm</x:v>
+      </x:c>
+      <x:c r="E5" s="298" t="str">
+        <x:v>Sản lượng điện dự kiến phát trong một năm.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="299" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="300" t="str">
+        <x:v>CAPEX</x:v>
+      </x:c>
+      <x:c r="C6" s="298" t="str">
+        <x:v>Capital Expenditure</x:v>
+      </x:c>
+      <x:c r="D6" s="298" t="str">
+        <x:v>Chi phí đầu tư / Tổng mức đầu tư</x:v>
+      </x:c>
+      <x:c r="E6" s="298" t="str">
+        <x:v>Chi phí hình thành tài sản của dự án, gồm nhà máy điện và đấu nối.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="299" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="300" t="str">
+        <x:v>CF</x:v>
+      </x:c>
+      <x:c r="C7" s="298" t="str">
+        <x:v>Capacity Factor</x:v>
+      </x:c>
+      <x:c r="D7" s="298" t="str">
+        <x:v>Hệ số công suất</x:v>
+      </x:c>
+      <x:c r="E7" s="298" t="str">
+        <x:v>Tỷ lệ giữa sản lượng thực tế và sản lượng lý thuyết ở công suất định mức.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="299" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="300" t="str">
+        <x:v>CFADS</x:v>
+      </x:c>
+      <x:c r="C8" s="298" t="str">
+        <x:v>Cash Flow Available for Debt Service</x:v>
+      </x:c>
+      <x:c r="D8" s="298" t="str">
+        <x:v>Dòng tiền sẵn có để trả nợ</x:v>
+      </x:c>
+      <x:c r="E8" s="298" t="str">
+        <x:v>Dòng tiền dùng để thanh toán gốc và lãi vay.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="299" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="300" t="str">
+        <x:v>COD</x:v>
+      </x:c>
+      <x:c r="C9" s="298" t="str">
+        <x:v>Commercial Operation Date</x:v>
+      </x:c>
+      <x:c r="D9" s="298" t="str">
+        <x:v>Ngày vận hành thương mại</x:v>
+      </x:c>
+      <x:c r="E9" s="298" t="str">
+        <x:v>Thời điểm dự án bắt đầu vận hành và ghi nhận doanh thu.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="299" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B10" s="300" t="str">
+        <x:v>CIT</x:v>
+      </x:c>
+      <x:c r="C10" s="298" t="str">
+        <x:v>Corporate Income Tax</x:v>
+      </x:c>
+      <x:c r="D10" s="298" t="str">
+        <x:v>Thuế thu nhập doanh nghiệp (TNDN)</x:v>
+      </x:c>
+      <x:c r="E10" s="298" t="str">
+        <x:v>Thuế tính trên thu nhập chịu thuế của doanh nghiệp dự án.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="299" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B11" s="300" t="str">
+        <x:v>DCF</x:v>
+      </x:c>
+      <x:c r="C11" s="298" t="str">
+        <x:v>Discounted Cash Flow</x:v>
+      </x:c>
+      <x:c r="D11" s="298" t="str">
+        <x:v>Dòng tiền chiết khấu</x:v>
+      </x:c>
+      <x:c r="E11" s="298" t="str">
+        <x:v>Phương pháp quy đổi dòng tiền tương lai về giá trị hiện tại.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="299" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B12" s="300" t="str">
+        <x:v>Dep.</x:v>
+      </x:c>
+      <x:c r="C12" s="298" t="str">
+        <x:v>Depreciation</x:v>
+      </x:c>
+      <x:c r="D12" s="298" t="str">
+        <x:v>Khấu hao</x:v>
+      </x:c>
+      <x:c r="E12" s="298" t="str">
+        <x:v>Phân bổ nguyên giá tài sản cố định vào chi phí qua thời gian.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="299" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B13" s="300" t="str">
+        <x:v>DSCR</x:v>
+      </x:c>
+      <x:c r="C13" s="298" t="str">
+        <x:v>Debt Service Coverage Ratio</x:v>
+      </x:c>
+      <x:c r="D13" s="298" t="str">
+        <x:v>Hệ số khả năng trả nợ</x:v>
+      </x:c>
+      <x:c r="E13" s="298" t="str">
+        <x:v>CFADS chia cho tổng gốc và lãi phải trả trong kỳ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="299" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B14" s="300" t="str">
+        <x:v>EBIT</x:v>
+      </x:c>
+      <x:c r="C14" s="298" t="str">
+        <x:v>Earnings Before Interest and Taxes</x:v>
+      </x:c>
+      <x:c r="D14" s="298" t="str">
+        <x:v>Lợi nhuận trước lãi vay và thuế</x:v>
+      </x:c>
+      <x:c r="E14" s="298" t="str">
+        <x:v>Doanh thu trừ chi phí hoạt động và khấu hao.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="299" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B15" s="300" t="str">
+        <x:v>EBITDA</x:v>
+      </x:c>
+      <x:c r="C15" s="298" t="str">
+        <x:v>Earnings Before Interest, Taxes, Depreciation and Amortization</x:v>
+      </x:c>
+      <x:c r="D15" s="298" t="str">
+        <x:v>Lợi nhuận trước lãi vay, thuế và khấu hao</x:v>
+      </x:c>
+      <x:c r="E15" s="298" t="str">
+        <x:v>Chỉ tiêu phản ánh hiệu quả hoạt động trước chi phí tài trợ và khấu hao.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="299" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B16" s="300" t="str">
+        <x:v>EIRR</x:v>
+      </x:c>
+      <x:c r="C16" s="298" t="str">
+        <x:v>Economic Internal Rate of Return</x:v>
+      </x:c>
+      <x:c r="D16" s="298" t="str">
+        <x:v>Tỷ suất hoàn vốn nội bộ kinh tế</x:v>
+      </x:c>
+      <x:c r="E16" s="298" t="str">
+        <x:v>IRR theo góc nhìn kinh tế – xã hội, nếu có phân tích kinh tế.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="299" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B17" s="300" t="str">
+        <x:v>ENPV</x:v>
+      </x:c>
+      <x:c r="C17" s="298" t="str">
+        <x:v>Economic Net Present Value</x:v>
+      </x:c>
+      <x:c r="D17" s="298" t="str">
+        <x:v>Giá trị hiện tại thuần kinh tế</x:v>
+      </x:c>
+      <x:c r="E17" s="298" t="str">
+        <x:v>NPV theo góc nhìn kinh tế – xã hội, nếu có phân tích kinh tế.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
+      <x:c r="A18" s="299" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B18" s="300" t="str">
+        <x:v>Equity CF</x:v>
+      </x:c>
+      <x:c r="C18" s="298" t="str">
+        <x:v>Equity Cash Flow</x:v>
+      </x:c>
+      <x:c r="D18" s="298" t="str">
+        <x:v>Dòng tiền vốn chủ sở hữu</x:v>
+      </x:c>
+      <x:c r="E18" s="298" t="str">
+        <x:v>Dòng tiền còn lại cho chủ đầu tư sau tài trợ, trả nợ và thuế.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
+      <x:c r="A19" s="299" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B19" s="300" t="str">
+        <x:v>Equity IRR</x:v>
+      </x:c>
+      <x:c r="C19" s="298" t="str">
+        <x:v>Equity Internal Rate of Return</x:v>
+      </x:c>
+      <x:c r="D19" s="298" t="str">
+        <x:v>Tỷ suất hoàn vốn nội bộ vốn chủ sở hữu</x:v>
+      </x:c>
+      <x:c r="E19" s="298" t="str">
+        <x:v>Mức sinh lời nội bộ của phần vốn chủ sở hữu.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="34" customHeight="1">
+      <x:c r="A20" s="299" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B20" s="300" t="str">
+        <x:v>Equity NPV</x:v>
+      </x:c>
+      <x:c r="C20" s="298" t="str">
+        <x:v>Equity Net Present Value</x:v>
+      </x:c>
+      <x:c r="D20" s="298" t="str">
+        <x:v>Giá trị hiện tại thuần vốn chủ sở hữu</x:v>
+      </x:c>
+      <x:c r="E20" s="298" t="str">
+        <x:v>Giá trị hiện tại của dòng tiền vốn chủ sau khi trừ vốn góp ban đầu.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="299" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B21" s="300" t="str">
+        <x:v>FLH</x:v>
+      </x:c>
+      <x:c r="C21" s="298" t="str">
+        <x:v>Full Load Hours</x:v>
+      </x:c>
+      <x:c r="D21" s="298" t="str">
+        <x:v>Số giờ vận hành quy đổi toàn tải</x:v>
+      </x:c>
+      <x:c r="E21" s="298" t="str">
+        <x:v>AEP chia cho công suất lắp đặt; FLH = CF × 8.760 giờ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="34" customHeight="1">
+      <x:c r="A22" s="299" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B22" s="300" t="str">
+        <x:v>IDC</x:v>
+      </x:c>
+      <x:c r="C22" s="298" t="str">
+        <x:v>Interest During Construction</x:v>
+      </x:c>
+      <x:c r="D22" s="298" t="str">
+        <x:v>Lãi vay trong thời gian xây dựng</x:v>
+      </x:c>
+      <x:c r="E22" s="298" t="str">
+        <x:v>Lãi vay phát sinh trước COD, thường được vốn hóa vào tổng đầu tư.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="34" customHeight="1">
+      <x:c r="A23" s="299" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B23" s="300" t="str">
+        <x:v>IRR</x:v>
+      </x:c>
+      <x:c r="C23" s="298" t="str">
+        <x:v>Internal Rate of Return</x:v>
+      </x:c>
+      <x:c r="D23" s="298" t="str">
+        <x:v>Tỷ suất hoàn vốn nội bộ</x:v>
+      </x:c>
+      <x:c r="E23" s="298" t="str">
+        <x:v>Tỷ lệ chiết khấu làm NPV của dòng tiền bằng 0.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="299" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B24" s="300" t="str">
+        <x:v>kWh</x:v>
+      </x:c>
+      <x:c r="C24" s="298" t="str">
+        <x:v>Kilowatt-hour</x:v>
+      </x:c>
+      <x:c r="D24" s="298" t="str">
+        <x:v>Kilôwatt giờ</x:v>
+      </x:c>
+      <x:c r="E24" s="298" t="str">
+        <x:v>Đơn vị điện năng.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="34" customHeight="1">
+      <x:c r="A25" s="299" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B25" s="300" t="str">
+        <x:v>LCOE</x:v>
+      </x:c>
+      <x:c r="C25" s="298" t="str">
+        <x:v>Levelized Cost of Energy</x:v>
+      </x:c>
+      <x:c r="D25" s="298" t="str">
+        <x:v>Chi phí điện quy dẫn</x:v>
+      </x:c>
+      <x:c r="E25" s="298" t="str">
+        <x:v>Chi phí bình quân chiết khấu để sản xuất một đơn vị điện năng.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="34" customHeight="1">
+      <x:c r="A26" s="299" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B26" s="300" t="str">
+        <x:v>LLCR</x:v>
+      </x:c>
+      <x:c r="C26" s="298" t="str">
+        <x:v>Loan Life Coverage Ratio</x:v>
+      </x:c>
+      <x:c r="D26" s="298" t="str">
+        <x:v>Hệ số bảo đảm trả nợ trong thời hạn vay</x:v>
+      </x:c>
+      <x:c r="E26" s="298" t="str">
+        <x:v>Giá trị hiện tại của CFADS trong thời hạn vay chia cho dư nợ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" s="299" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B27" s="300" t="str">
+        <x:v>MW</x:v>
+      </x:c>
+      <x:c r="C27" s="298" t="str">
+        <x:v>Megawatt</x:v>
+      </x:c>
+      <x:c r="D27" s="298" t="str">
+        <x:v>Megawatt</x:v>
+      </x:c>
+      <x:c r="E27" s="298" t="str">
+        <x:v>Đơn vị công suất, bằng 1.000 kW.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="34" customHeight="1">
+      <x:c r="A28" s="299" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B28" s="300" t="str">
+        <x:v>MWh</x:v>
+      </x:c>
+      <x:c r="C28" s="298" t="str">
+        <x:v>Megawatt-hour</x:v>
+      </x:c>
+      <x:c r="D28" s="298" t="str">
+        <x:v>Megawatt giờ</x:v>
+      </x:c>
+      <x:c r="E28" s="298" t="str">
+        <x:v>Đơn vị điện năng, bằng 1.000 kWh.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
+      <x:c r="A29" s="299" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B29" s="300" t="str">
+        <x:v>NPV</x:v>
+      </x:c>
+      <x:c r="C29" s="298" t="str">
+        <x:v>Net Present Value</x:v>
+      </x:c>
+      <x:c r="D29" s="298" t="str">
+        <x:v>Giá trị hiện tại thuần</x:v>
+      </x:c>
+      <x:c r="E29" s="298" t="str">
+        <x:v>Tổng giá trị hiện tại của dòng tiền vào trừ dòng tiền ra.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="34" customHeight="1">
+      <x:c r="A30" s="299" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B30" s="300" t="str">
+        <x:v>O&amp;M</x:v>
+      </x:c>
+      <x:c r="C30" s="298" t="str">
+        <x:v>Operation and Maintenance</x:v>
+      </x:c>
+      <x:c r="D30" s="298" t="str">
+        <x:v>Vận hành và bảo dưỡng</x:v>
+      </x:c>
+      <x:c r="E30" s="298" t="str">
+        <x:v>Chi phí vận hành, bảo dưỡng hằng năm; mô hình nhập theo % CAPEX/năm.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
+      <x:c r="A31" s="299" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B31" s="300" t="str">
+        <x:v>P50</x:v>
+      </x:c>
+      <x:c r="C31" s="298" t="str">
+        <x:v>50% Probability of Exceedance</x:v>
+      </x:c>
+      <x:c r="D31" s="298" t="str">
+        <x:v>Mức sản lượng có xác suất vượt 50%</x:v>
+      </x:c>
+      <x:c r="E31" s="298" t="str">
+        <x:v>Kịch bản sản lượng cơ sở/trung vị.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="34" customHeight="1">
+      <x:c r="A32" s="299" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B32" s="300" t="str">
+        <x:v>P75</x:v>
+      </x:c>
+      <x:c r="C32" s="298" t="str">
+        <x:v>75% Probability of Exceedance</x:v>
+      </x:c>
+      <x:c r="D32" s="298" t="str">
+        <x:v>Mức sản lượng có xác suất vượt 75%</x:v>
+      </x:c>
+      <x:c r="E32" s="298" t="str">
+        <x:v>Kịch bản sản lượng thận trọng hơn P50.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="34" customHeight="1">
+      <x:c r="A33" s="299" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B33" s="300" t="str">
+        <x:v>P90</x:v>
+      </x:c>
+      <x:c r="C33" s="298" t="str">
+        <x:v>90% Probability of Exceedance</x:v>
+      </x:c>
+      <x:c r="D33" s="298" t="str">
+        <x:v>Mức sản lượng có xác suất vượt 90%</x:v>
+      </x:c>
+      <x:c r="E33" s="298" t="str">
+        <x:v>Kịch bản bảo thủ thường dùng để kiểm tra khả năng trả nợ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="34" customHeight="1">
+      <x:c r="A34" s="299" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B34" s="300" t="str">
+        <x:v>PPA</x:v>
+      </x:c>
+      <x:c r="C34" s="298" t="str">
+        <x:v>Power Purchase Agreement</x:v>
+      </x:c>
+      <x:c r="D34" s="298" t="str">
+        <x:v>Hợp đồng mua bán điện</x:v>
+      </x:c>
+      <x:c r="E34" s="298" t="str">
+        <x:v>Quy định giá điện, sản lượng và các điều kiện thương mại.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="34" customHeight="1">
+      <x:c r="A35" s="299" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B35" s="300" t="str">
+        <x:v>Project CF</x:v>
+      </x:c>
+      <x:c r="C35" s="298" t="str">
+        <x:v>Project Cash Flow</x:v>
+      </x:c>
+      <x:c r="D35" s="298" t="str">
+        <x:v>Dòng tiền toàn dự án</x:v>
+      </x:c>
+      <x:c r="E35" s="298" t="str">
+        <x:v>Dòng tiền trước tài trợ, không phụ thuộc cơ cấu vay và vốn chủ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="34" customHeight="1">
+      <x:c r="A36" s="299" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B36" s="300" t="str">
+        <x:v>Project IRR</x:v>
+      </x:c>
+      <x:c r="C36" s="298" t="str">
+        <x:v>Project Internal Rate of Return</x:v>
+      </x:c>
+      <x:c r="D36" s="298" t="str">
+        <x:v>Tỷ suất hoàn vốn nội bộ dự án</x:v>
+      </x:c>
+      <x:c r="E36" s="298" t="str">
+        <x:v>IRR của dòng tiền toàn dự án trước tài trợ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="34" customHeight="1">
+      <x:c r="A37" s="299" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B37" s="300" t="str">
+        <x:v>Project NPV</x:v>
+      </x:c>
+      <x:c r="C37" s="298" t="str">
+        <x:v>Project Net Present Value</x:v>
+      </x:c>
+      <x:c r="D37" s="298" t="str">
+        <x:v>Giá trị hiện tại thuần dự án</x:v>
+      </x:c>
+      <x:c r="E37" s="298" t="str">
+        <x:v>NPV của dòng tiền toàn dự án tại tỷ lệ chiết khấu dự án.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="34" customHeight="1">
+      <x:c r="A38" s="299" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B38" s="300" t="str">
+        <x:v>VAT</x:v>
+      </x:c>
+      <x:c r="C38" s="298" t="str">
+        <x:v>Value Added Tax</x:v>
+      </x:c>
+      <x:c r="D38" s="298" t="str">
+        <x:v>Thuế giá trị gia tăng (GTGT)</x:v>
+      </x:c>
+      <x:c r="E38" s="298" t="str">
+        <x:v>Thuế gián thu áp dụng cho hàng hóa và dịch vụ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="34" customHeight="1">
+      <x:c r="A39" s="299" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B39" s="300" t="str">
+        <x:v>WACC</x:v>
+      </x:c>
+      <x:c r="C39" s="298" t="str">
+        <x:v>Weighted Average Cost of Capital</x:v>
+      </x:c>
+      <x:c r="D39" s="298" t="str">
+        <x:v>Chi phí sử dụng vốn bình quân gia quyền</x:v>
+      </x:c>
+      <x:c r="E39" s="298" t="str">
+        <x:v>Tỷ lệ chiết khấu phản ánh chi phí bình quân của vốn vay và vốn chủ.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>